<commit_message>
Fix Shop Tracker participation data — re-pull CETD with grid clear
Found stale-data bug in batch CETD pull: grid wasn't clearing between
shop queries, so each shop was reading the previous shop's employees.
Result: Nathan showed up on January shops he never worked.

Fixed __pullOne to call grid.getStore().removeAll() before each query
and re-pulled all 22 shops cleanly.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1101,7 +1101,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G14" s="29" t="n"/>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H14" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C14:G14,"Y"),"")</f>
         <v/>
@@ -1136,11 +1140,7 @@
         </is>
       </c>
       <c r="F15" s="29" t="n"/>
-      <c r="G15" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G15" s="29" t="n"/>
       <c r="H15" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C15:G15,"Y"),"")</f>
         <v/>
@@ -1167,11 +1167,7 @@
       <c r="D16" s="29" t="n"/>
       <c r="E16" s="29" t="n"/>
       <c r="F16" s="29" t="n"/>
-      <c r="G16" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G16" s="29" t="n"/>
       <c r="H16" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C16:G16,"Y"),"")</f>
         <v/>
@@ -1198,11 +1194,7 @@
       <c r="D17" s="29" t="n"/>
       <c r="E17" s="29" t="n"/>
       <c r="F17" s="29" t="n"/>
-      <c r="G17" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G17" s="29" t="n"/>
       <c r="H17" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C17:G17,"Y"),"")</f>
         <v/>
@@ -1522,11 +1514,7 @@
       <c r="D29" s="18" t="n"/>
       <c r="E29" s="18" t="n"/>
       <c r="F29" s="18" t="n"/>
-      <c r="G29" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G29" s="18" t="n"/>
       <c r="H29" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C29:G29,"Y"),"")</f>
         <v/>
@@ -2282,7 +2270,11 @@
           <t>Vicki L.</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n"/>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2326,7 +2318,11 @@
           <t>Kasey W.</t>
         </is>
       </c>
-      <c r="C16" s="29" t="n"/>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D16" s="29" t="n"/>
       <c r="E16" s="29" t="n"/>
       <c r="F16" s="28" t="inlineStr">
@@ -2362,7 +2358,11 @@
           <t>Nathan R.</t>
         </is>
       </c>
-      <c r="C17" s="29" t="n"/>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D17" s="29" t="n"/>
       <c r="E17" s="29" t="n"/>
       <c r="F17" s="29" t="n"/>
@@ -2684,7 +2684,11 @@
           <t>Jeremiah</t>
         </is>
       </c>
-      <c r="C29" s="18" t="n"/>
+      <c r="C29" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D29" s="18" t="n"/>
       <c r="E29" s="28" t="inlineStr">
         <is>
@@ -2900,11 +2904,7 @@
           <t>Mike</t>
         </is>
       </c>
-      <c r="C35" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C35" s="18" t="n"/>
       <c r="D35" s="18" t="n"/>
       <c r="E35" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Tighten shop participation rules — peak rush window + 30 min minimum
Bobby caught Vicki marked Y on Apr 23 dinner shop when she was a day
worker who clocked out at 15:07. Old filter counted any overlap with
the broad meal period (15:00-21:59); new filter requires 30+ min
overlap with the peak shop window (Lunch 11:30-1:30, Dinner 5:00-7:30,
Late Dinner 8:00-10:00).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1134,11 +1134,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E15" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E15" s="29" t="n"/>
       <c r="F15" s="29" t="n"/>
       <c r="G15" s="29" t="n"/>
       <c r="H15" s="17">
@@ -1254,17 +1250,9 @@
           <t>Ash</t>
         </is>
       </c>
-      <c r="C21" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C21" s="18" t="n"/>
       <c r="D21" s="18" t="n"/>
-      <c r="E21" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E21" s="18" t="n"/>
       <c r="F21" s="18" t="n"/>
       <c r="G21" s="18" t="n"/>
       <c r="H21" s="17">
@@ -1420,11 +1408,7 @@
         </is>
       </c>
       <c r="E26" s="35" t="n"/>
-      <c r="F26" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F26" s="35" t="n"/>
       <c r="G26" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1618,26 +1602,14 @@
           <t>Lidy</t>
         </is>
       </c>
-      <c r="C33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C33" s="18" t="n"/>
       <c r="D33" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
       <c r="G33" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2243,11 +2215,7 @@
         </is>
       </c>
       <c r="G14" s="29" t="n"/>
-      <c r="H14" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="H14" s="29" t="n"/>
       <c r="I14" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C14:H14,"Y"),"")</f>
         <v/>
@@ -2275,21 +2243,13 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D15" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D15" s="29" t="n"/>
       <c r="E15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F15" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F15" s="29" t="n"/>
       <c r="G15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2577,21 +2537,13 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D26" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D26" s="35" t="n"/>
       <c r="E26" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F26" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F26" s="35" t="n"/>
       <c r="G26" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2651,11 +2603,7 @@
       <c r="C28" s="35" t="n"/>
       <c r="D28" s="35" t="n"/>
       <c r="E28" s="35" t="n"/>
-      <c r="F28" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F28" s="35" t="n"/>
       <c r="G28" s="35" t="n"/>
       <c r="H28" s="28" t="inlineStr">
         <is>
@@ -2690,11 +2638,7 @@
         </is>
       </c>
       <c r="D29" s="18" t="n"/>
-      <c r="E29" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E29" s="18" t="n"/>
       <c r="F29" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2731,17 +2675,9 @@
       <c r="C30" s="35" t="n"/>
       <c r="D30" s="35" t="n"/>
       <c r="E30" s="35" t="n"/>
-      <c r="F30" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F30" s="35" t="n"/>
       <c r="G30" s="35" t="n"/>
-      <c r="H30" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="H30" s="35" t="n"/>
       <c r="I30" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C30:H30,"Y"),"")</f>
         <v/>
@@ -2825,11 +2761,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D33" s="18" t="n"/>
       <c r="E33" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2841,11 +2773,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="H33" s="18" t="n"/>
       <c r="I33" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C33:H33,"Y"),"")</f>
         <v/>
@@ -3446,11 +3374,7 @@
           <t>Vicki L.</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C15" s="29" t="n"/>
       <c r="D15" s="29" t="n"/>
       <c r="E15" s="28" t="inlineStr">
         <is>
@@ -3944,11 +3868,7 @@
           <t>Lidy</t>
         </is>
       </c>
-      <c r="C33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C33" s="18" t="n"/>
       <c r="D33" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4576,11 +4496,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G15" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G15" s="29" t="n"/>
       <c r="H15" s="29" t="n"/>
       <c r="I15" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C15:H15,"Y"),"")</f>
@@ -4644,11 +4560,7 @@
           <t>Nathan R.</t>
         </is>
       </c>
-      <c r="C17" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C17" s="29" t="n"/>
       <c r="D17" s="29" t="n"/>
       <c r="E17" s="28" t="inlineStr">
         <is>
@@ -4656,11 +4568,7 @@
         </is>
       </c>
       <c r="F17" s="29" t="n"/>
-      <c r="G17" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G17" s="29" t="n"/>
       <c r="H17" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5106,31 +5014,19 @@
           <t>Lidy</t>
         </is>
       </c>
-      <c r="C33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C33" s="18" t="n"/>
       <c r="D33" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E33" s="18" t="n"/>
       <c r="F33" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G33" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G33" s="18" t="n"/>
       <c r="H33" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5228,11 +5124,7 @@
         </is>
       </c>
       <c r="D36" s="35" t="n"/>
-      <c r="E36" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E36" s="35" t="n"/>
       <c r="F36" s="28" t="inlineStr">
         <is>
           <t>Y</t>

</xml_diff>

<commit_message>
Apply final shop window rules per Bobby
Lunch shop window:        11:00 AM - 1:30 PM
Dinner shop window:        4:00 PM - 7:00 PM
Late Dinner shop window:   7:00 PM - 10:00 PM
Minimum overlap:           30 minutes

Employees only count if their actual clock-in/clock-out had at
least 30 minutes inside the exact shop window. Day workers who
finished at/around 4 PM are now correctly excluded from dinner
shops.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1252,7 +1252,11 @@
       </c>
       <c r="C21" s="18" t="n"/>
       <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
+      <c r="E21" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F21" s="18" t="n"/>
       <c r="G21" s="18" t="n"/>
       <c r="H21" s="17">
@@ -2215,7 +2219,11 @@
         </is>
       </c>
       <c r="G14" s="29" t="n"/>
-      <c r="H14" s="29" t="n"/>
+      <c r="H14" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I14" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C14:H14,"Y"),"")</f>
         <v/>
@@ -2603,7 +2611,11 @@
       <c r="C28" s="35" t="n"/>
       <c r="D28" s="35" t="n"/>
       <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G28" s="35" t="n"/>
       <c r="H28" s="28" t="inlineStr">
         <is>
@@ -4560,7 +4572,11 @@
           <t>Nathan R.</t>
         </is>
       </c>
-      <c r="C17" s="29" t="n"/>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D17" s="29" t="n"/>
       <c r="E17" s="28" t="inlineStr">
         <is>
@@ -4568,7 +4584,11 @@
         </is>
       </c>
       <c r="F17" s="29" t="n"/>
-      <c r="G17" s="29" t="n"/>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H17" s="28" t="inlineStr">
         <is>
           <t>Y</t>

</xml_diff>

<commit_message>
Expand lunch shop window to 11am-4pm
Lunch shops can occur 11-1:30pm (lunch rush) or 1:30-4pm (day shift).
Both fall under the "Lunch" Marketforce label, so the window is the
full day-shift block.

Final shop windows:
  Lunch:        11:00 AM - 4:00 PM
  Dinner:        4:00 PM - 7:00 PM
  Late Dinner:   7:00 PM - 10:00 PM
  Min overlap:   30 minutes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -364,13 +364,13 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1090,7 +1090,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D14" s="29" t="n"/>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E14" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1110,11 +1114,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C14:G14,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="29">
         <f>COUNTIF(C14:G14,"Y")</f>
         <v/>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C14:G14="Y"))*50</f>
         <v/>
       </c>
@@ -1128,24 +1132,24 @@
           <t>Vicki L.</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n"/>
+      <c r="C15" s="31" t="n"/>
       <c r="D15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E15" s="29" t="n"/>
-      <c r="F15" s="29" t="n"/>
-      <c r="G15" s="29" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="31" t="n"/>
       <c r="H15" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C15:G15,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I15" s="30">
+      <c r="I15" s="29">
         <f>COUNTIF(C15:G15,"Y")</f>
         <v/>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C15:G15="Y"))*50</f>
         <v/>
       </c>
@@ -1159,20 +1163,20 @@
           <t>Kasey W.</t>
         </is>
       </c>
-      <c r="C16" s="29" t="n"/>
-      <c r="D16" s="29" t="n"/>
-      <c r="E16" s="29" t="n"/>
-      <c r="F16" s="29" t="n"/>
-      <c r="G16" s="29" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
       <c r="H16" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C16:G16,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="29">
         <f>COUNTIF(C16:G16,"Y")</f>
         <v/>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C16:G16="Y"))*50</f>
         <v/>
       </c>
@@ -1186,20 +1190,20 @@
           <t>Nathan R.</t>
         </is>
       </c>
-      <c r="C17" s="29" t="n"/>
-      <c r="D17" s="29" t="n"/>
-      <c r="E17" s="29" t="n"/>
-      <c r="F17" s="29" t="n"/>
-      <c r="G17" s="29" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="31" t="n"/>
       <c r="H17" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C17:G17,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I17" s="30">
+      <c r="I17" s="29">
         <f>COUNTIF(C17:G17,"Y")</f>
         <v/>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C17:G17="Y"))*50</f>
         <v/>
       </c>
@@ -1232,11 +1236,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C20:G20,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I20" s="30">
+      <c r="I20" s="29">
         <f>COUNTIF(C20:G20,"Y")</f>
         <v/>
       </c>
-      <c r="J20" s="31">
+      <c r="J20" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C20:G20="Y"))*50</f>
         <v/>
       </c>
@@ -1263,11 +1267,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C21:G21,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="29">
         <f>COUNTIF(C21:G21,"Y")</f>
         <v/>
       </c>
-      <c r="J21" s="31">
+      <c r="J21" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C21:G21="Y"))*50</f>
         <v/>
       </c>
@@ -1298,11 +1302,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C22:G22,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="29">
         <f>COUNTIF(C22:G22,"Y")</f>
         <v/>
       </c>
-      <c r="J22" s="31">
+      <c r="J22" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C22:G22="Y"))*50</f>
         <v/>
       </c>
@@ -1329,11 +1333,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C23:G23,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I23" s="30">
+      <c r="I23" s="29">
         <f>COUNTIF(C23:G23,"Y")</f>
         <v/>
       </c>
-      <c r="J23" s="31">
+      <c r="J23" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C23:G23="Y"))*50</f>
         <v/>
       </c>
@@ -1356,11 +1360,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C24:G24,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I24" s="30">
+      <c r="I24" s="29">
         <f>COUNTIF(C24:G24,"Y")</f>
         <v/>
       </c>
-      <c r="J24" s="31">
+      <c r="J24" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C24:G24="Y"))*50</f>
         <v/>
       </c>
@@ -1383,11 +1387,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C25:G25,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="29">
         <f>COUNTIF(C25:G25,"Y")</f>
         <v/>
       </c>
-      <c r="J25" s="31">
+      <c r="J25" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C25:G25="Y"))*50</f>
         <v/>
       </c>
@@ -1422,11 +1426,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C26:G26,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I26" s="30">
+      <c r="I26" s="29">
         <f>COUNTIF(C26:G26,"Y")</f>
         <v/>
       </c>
-      <c r="J26" s="31">
+      <c r="J26" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C26:G26="Y"))*50</f>
         <v/>
       </c>
@@ -1449,11 +1453,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C27:G27,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I27" s="30">
+      <c r="I27" s="29">
         <f>COUNTIF(C27:G27,"Y")</f>
         <v/>
       </c>
-      <c r="J27" s="31">
+      <c r="J27" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C27:G27="Y"))*50</f>
         <v/>
       </c>
@@ -1476,11 +1480,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C28:G28,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I28" s="30">
+      <c r="I28" s="29">
         <f>COUNTIF(C28:G28,"Y")</f>
         <v/>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C28:G28="Y"))*50</f>
         <v/>
       </c>
@@ -1499,19 +1503,27 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D29" s="18" t="n"/>
+      <c r="D29" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E29" s="18" t="n"/>
       <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
+      <c r="G29" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H29" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C29:G29,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I29" s="30">
+      <c r="I29" s="29">
         <f>COUNTIF(C29:G29,"Y")</f>
         <v/>
       </c>
-      <c r="J29" s="31">
+      <c r="J29" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C29:G29="Y"))*50</f>
         <v/>
       </c>
@@ -1534,11 +1546,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C30:G30,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I30" s="30">
+      <c r="I30" s="29">
         <f>COUNTIF(C30:G30,"Y")</f>
         <v/>
       </c>
-      <c r="J30" s="31">
+      <c r="J30" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C30:G30="Y"))*50</f>
         <v/>
       </c>
@@ -1561,11 +1573,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C31:G31,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I31" s="30">
+      <c r="I31" s="29">
         <f>COUNTIF(C31:G31,"Y")</f>
         <v/>
       </c>
-      <c r="J31" s="31">
+      <c r="J31" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C31:G31="Y"))*50</f>
         <v/>
       </c>
@@ -1588,11 +1600,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C32:G32,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I32" s="30">
+      <c r="I32" s="29">
         <f>COUNTIF(C32:G32,"Y")</f>
         <v/>
       </c>
-      <c r="J32" s="31">
+      <c r="J32" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C32:G32="Y"))*50</f>
         <v/>
       </c>
@@ -1623,11 +1635,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C33:G33,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I33" s="30">
+      <c r="I33" s="29">
         <f>COUNTIF(C33:G33,"Y")</f>
         <v/>
       </c>
-      <c r="J33" s="31">
+      <c r="J33" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C33:G33="Y"))*50</f>
         <v/>
       </c>
@@ -1646,7 +1658,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D34" s="35" t="n"/>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E34" s="35" t="n"/>
       <c r="F34" s="28" t="inlineStr">
         <is>
@@ -1658,11 +1674,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C34:G34,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I34" s="30">
+      <c r="I34" s="29">
         <f>COUNTIF(C34:G34,"Y")</f>
         <v/>
       </c>
-      <c r="J34" s="31">
+      <c r="J34" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C34:G34="Y"))*50</f>
         <v/>
       </c>
@@ -1688,16 +1704,20 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G35" s="18" t="n"/>
+      <c r="G35" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H35" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C35:G35,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I35" s="30">
+      <c r="I35" s="29">
         <f>COUNTIF(C35:G35,"Y")</f>
         <v/>
       </c>
-      <c r="J35" s="31">
+      <c r="J35" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C35:G35="Y"))*50</f>
         <v/>
       </c>
@@ -1720,11 +1740,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C36:G36,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I36" s="30">
+      <c r="I36" s="29">
         <f>COUNTIF(C36:G36,"Y")</f>
         <v/>
       </c>
-      <c r="J36" s="31">
+      <c r="J36" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C36:G36="Y"))*50</f>
         <v/>
       </c>
@@ -1759,11 +1779,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C37:G37,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I37" s="30">
+      <c r="I37" s="29">
         <f>COUNTIF(C37:G37,"Y")</f>
         <v/>
       </c>
-      <c r="J37" s="31">
+      <c r="J37" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C37:G37="Y"))*50</f>
         <v/>
       </c>
@@ -1786,11 +1806,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C38:G38,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I38" s="30">
+      <c r="I38" s="29">
         <f>COUNTIF(C38:G38,"Y")</f>
         <v/>
       </c>
-      <c r="J38" s="31">
+      <c r="J38" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C38:G38="Y"))*50</f>
         <v/>
       </c>
@@ -2206,19 +2226,23 @@
           <t>Madison C.</t>
         </is>
       </c>
-      <c r="C14" s="29" t="n"/>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D14" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E14" s="29" t="n"/>
+      <c r="E14" s="31" t="n"/>
       <c r="F14" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G14" s="29" t="n"/>
+      <c r="G14" s="31" t="n"/>
       <c r="H14" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2228,11 +2252,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C14:H14,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="29">
         <f>COUNTIF(C14:H14,"Y")</f>
         <v/>
       </c>
-      <c r="K14" s="31">
+      <c r="K14" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C14:H14="Y"))*50</f>
         <v/>
       </c>
@@ -2251,28 +2275,28 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D15" s="29" t="n"/>
+      <c r="D15" s="31" t="n"/>
       <c r="E15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F15" s="29" t="n"/>
+      <c r="F15" s="31" t="n"/>
       <c r="G15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H15" s="29" t="n"/>
+      <c r="H15" s="31" t="n"/>
       <c r="I15" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C15:H15,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="29">
         <f>COUNTIF(C15:H15,"Y")</f>
         <v/>
       </c>
-      <c r="K15" s="31">
+      <c r="K15" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C15:H15="Y"))*50</f>
         <v/>
       </c>
@@ -2291,14 +2315,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D16" s="29" t="n"/>
-      <c r="E16" s="29" t="n"/>
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="31" t="n"/>
       <c r="F16" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G16" s="29" t="n"/>
+      <c r="G16" s="31" t="n"/>
       <c r="H16" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2308,11 +2332,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C16:H16,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="29">
         <f>COUNTIF(C16:H16,"Y")</f>
         <v/>
       </c>
-      <c r="K16" s="31">
+      <c r="K16" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C16:H16="Y"))*50</f>
         <v/>
       </c>
@@ -2331,20 +2355,20 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D17" s="29" t="n"/>
-      <c r="E17" s="29" t="n"/>
-      <c r="F17" s="29" t="n"/>
-      <c r="G17" s="29" t="n"/>
-      <c r="H17" s="29" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="n"/>
       <c r="I17" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C17:H17,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J17" s="30">
+      <c r="J17" s="29">
         <f>COUNTIF(C17:H17,"Y")</f>
         <v/>
       </c>
-      <c r="K17" s="31">
+      <c r="K17" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C17:H17="Y"))*50</f>
         <v/>
       </c>
@@ -2378,11 +2402,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C20:H20,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J20" s="30">
+      <c r="J20" s="29">
         <f>COUNTIF(C20:H20,"Y")</f>
         <v/>
       </c>
-      <c r="K20" s="31">
+      <c r="K20" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C20:H20="Y"))*50</f>
         <v/>
       </c>
@@ -2406,11 +2430,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C21:H21,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J21" s="30">
+      <c r="J21" s="29">
         <f>COUNTIF(C21:H21,"Y")</f>
         <v/>
       </c>
-      <c r="K21" s="31">
+      <c r="K21" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C21:H21="Y"))*50</f>
         <v/>
       </c>
@@ -2438,11 +2462,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C22:H22,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J22" s="30">
+      <c r="J22" s="29">
         <f>COUNTIF(C22:H22,"Y")</f>
         <v/>
       </c>
-      <c r="K22" s="31">
+      <c r="K22" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C22:H22="Y"))*50</f>
         <v/>
       </c>
@@ -2466,11 +2490,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C23:H23,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J23" s="30">
+      <c r="J23" s="29">
         <f>COUNTIF(C23:H23,"Y")</f>
         <v/>
       </c>
-      <c r="K23" s="31">
+      <c r="K23" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C23:H23="Y"))*50</f>
         <v/>
       </c>
@@ -2494,11 +2518,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C24:H24,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J24" s="30">
+      <c r="J24" s="29">
         <f>COUNTIF(C24:H24,"Y")</f>
         <v/>
       </c>
-      <c r="K24" s="31">
+      <c r="K24" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C24:H24="Y"))*50</f>
         <v/>
       </c>
@@ -2522,11 +2546,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C25:H25,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J25" s="30">
+      <c r="J25" s="29">
         <f>COUNTIF(C25:H25,"Y")</f>
         <v/>
       </c>
-      <c r="K25" s="31">
+      <c r="K25" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C25:H25="Y"))*50</f>
         <v/>
       </c>
@@ -2562,11 +2586,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C26:H26,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J26" s="30">
+      <c r="J26" s="29">
         <f>COUNTIF(C26:H26,"Y")</f>
         <v/>
       </c>
-      <c r="K26" s="31">
+      <c r="K26" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C26:H26="Y"))*50</f>
         <v/>
       </c>
@@ -2590,11 +2614,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C27:H27,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J27" s="30">
+      <c r="J27" s="29">
         <f>COUNTIF(C27:H27,"Y")</f>
         <v/>
       </c>
-      <c r="K27" s="31">
+      <c r="K27" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C27:H27="Y"))*50</f>
         <v/>
       </c>
@@ -2626,11 +2650,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C28:H28,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J28" s="30">
+      <c r="J28" s="29">
         <f>COUNTIF(C28:H28,"Y")</f>
         <v/>
       </c>
-      <c r="K28" s="31">
+      <c r="K28" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C28:H28="Y"))*50</f>
         <v/>
       </c>
@@ -2656,7 +2680,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G29" s="18" t="n"/>
+      <c r="G29" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H29" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2666,11 +2694,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C29:H29,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J29" s="30">
+      <c r="J29" s="29">
         <f>COUNTIF(C29:H29,"Y")</f>
         <v/>
       </c>
-      <c r="K29" s="31">
+      <c r="K29" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C29:H29="Y"))*50</f>
         <v/>
       </c>
@@ -2694,11 +2722,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C30:H30,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J30" s="30">
+      <c r="J30" s="29">
         <f>COUNTIF(C30:H30,"Y")</f>
         <v/>
       </c>
-      <c r="K30" s="31">
+      <c r="K30" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C30:H30="Y"))*50</f>
         <v/>
       </c>
@@ -2722,11 +2750,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C31:H31,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J31" s="30">
+      <c r="J31" s="29">
         <f>COUNTIF(C31:H31,"Y")</f>
         <v/>
       </c>
-      <c r="K31" s="31">
+      <c r="K31" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C31:H31="Y"))*50</f>
         <v/>
       </c>
@@ -2750,11 +2778,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C32:H32,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J32" s="30">
+      <c r="J32" s="29">
         <f>COUNTIF(C32:H32,"Y")</f>
         <v/>
       </c>
-      <c r="K32" s="31">
+      <c r="K32" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C32:H32="Y"))*50</f>
         <v/>
       </c>
@@ -2790,11 +2818,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C33:H33,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J33" s="30">
+      <c r="J33" s="29">
         <f>COUNTIF(C33:H33,"Y")</f>
         <v/>
       </c>
-      <c r="K33" s="31">
+      <c r="K33" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C33:H33="Y"))*50</f>
         <v/>
       </c>
@@ -2808,29 +2836,41 @@
           <t>Maylin</t>
         </is>
       </c>
-      <c r="C34" s="35" t="n"/>
+      <c r="C34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D34" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E34" s="35" t="n"/>
+      <c r="E34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F34" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G34" s="35" t="n"/>
+      <c r="G34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H34" s="35" t="n"/>
       <c r="I34" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C34:H34,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J34" s="30">
+      <c r="J34" s="29">
         <f>COUNTIF(C34:H34,"Y")</f>
         <v/>
       </c>
-      <c r="K34" s="31">
+      <c r="K34" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C34:H34="Y"))*50</f>
         <v/>
       </c>
@@ -2866,11 +2906,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C35:H35,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J35" s="30">
+      <c r="J35" s="29">
         <f>COUNTIF(C35:H35,"Y")</f>
         <v/>
       </c>
-      <c r="K35" s="31">
+      <c r="K35" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C35:H35="Y"))*50</f>
         <v/>
       </c>
@@ -2884,7 +2924,11 @@
           <t>Richard</t>
         </is>
       </c>
-      <c r="C36" s="35" t="n"/>
+      <c r="C36" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D36" s="35" t="n"/>
       <c r="E36" s="35" t="n"/>
       <c r="F36" s="35" t="n"/>
@@ -2894,11 +2938,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C36:H36,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J36" s="30">
+      <c r="J36" s="29">
         <f>COUNTIF(C36:H36,"Y")</f>
         <v/>
       </c>
-      <c r="K36" s="31">
+      <c r="K36" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C36:H36="Y"))*50</f>
         <v/>
       </c>
@@ -2930,11 +2974,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C37:H37,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J37" s="30">
+      <c r="J37" s="29">
         <f>COUNTIF(C37:H37,"Y")</f>
         <v/>
       </c>
-      <c r="K37" s="31">
+      <c r="K37" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C37:H37="Y"))*50</f>
         <v/>
       </c>
@@ -2958,11 +3002,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C38:H38,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J38" s="30">
+      <c r="J38" s="29">
         <f>COUNTIF(C38:H38,"Y")</f>
         <v/>
       </c>
-      <c r="K38" s="31">
+      <c r="K38" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C38:H38="Y"))*50</f>
         <v/>
       </c>
@@ -3356,23 +3400,31 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D14" s="29" t="n"/>
-      <c r="E14" s="29" t="n"/>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="n"/>
       <c r="F14" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G14" s="29" t="n"/>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H14" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C14:G14,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="29">
         <f>COUNTIF(C14:G14,"Y")</f>
         <v/>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C14:G14="Y"))*50</f>
         <v/>
       </c>
@@ -3386,14 +3438,14 @@
           <t>Vicki L.</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n"/>
-      <c r="D15" s="29" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
       <c r="E15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F15" s="29" t="n"/>
+      <c r="F15" s="31" t="n"/>
       <c r="G15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3403,11 +3455,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C15:G15,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I15" s="30">
+      <c r="I15" s="29">
         <f>COUNTIF(C15:G15,"Y")</f>
         <v/>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C15:G15="Y"))*50</f>
         <v/>
       </c>
@@ -3426,19 +3478,23 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D16" s="29" t="n"/>
-      <c r="E16" s="29" t="n"/>
-      <c r="F16" s="29" t="n"/>
-      <c r="G16" s="29" t="n"/>
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
       <c r="H16" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C16:G16,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="29">
         <f>COUNTIF(C16:G16,"Y")</f>
         <v/>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C16:G16="Y"))*50</f>
         <v/>
       </c>
@@ -3452,10 +3508,10 @@
           <t>Nathan R.</t>
         </is>
       </c>
-      <c r="C17" s="29" t="n"/>
-      <c r="D17" s="29" t="n"/>
-      <c r="E17" s="29" t="n"/>
-      <c r="F17" s="29" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
       <c r="G17" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3465,11 +3521,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C17:G17,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I17" s="30">
+      <c r="I17" s="29">
         <f>COUNTIF(C17:G17,"Y")</f>
         <v/>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C17:G17="Y"))*50</f>
         <v/>
       </c>
@@ -3502,11 +3558,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C20:G20,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I20" s="30">
+      <c r="I20" s="29">
         <f>COUNTIF(C20:G20,"Y")</f>
         <v/>
       </c>
-      <c r="J20" s="31">
+      <c r="J20" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C20:G20="Y"))*50</f>
         <v/>
       </c>
@@ -3529,11 +3585,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C21:G21,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="29">
         <f>COUNTIF(C21:G21,"Y")</f>
         <v/>
       </c>
-      <c r="J21" s="31">
+      <c r="J21" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C21:G21="Y"))*50</f>
         <v/>
       </c>
@@ -3564,11 +3620,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C22:G22,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="29">
         <f>COUNTIF(C22:G22,"Y")</f>
         <v/>
       </c>
-      <c r="J22" s="31">
+      <c r="J22" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C22:G22="Y"))*50</f>
         <v/>
       </c>
@@ -3595,11 +3651,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C23:G23,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I23" s="30">
+      <c r="I23" s="29">
         <f>COUNTIF(C23:G23,"Y")</f>
         <v/>
       </c>
-      <c r="J23" s="31">
+      <c r="J23" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C23:G23="Y"))*50</f>
         <v/>
       </c>
@@ -3622,11 +3678,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C24:G24,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I24" s="30">
+      <c r="I24" s="29">
         <f>COUNTIF(C24:G24,"Y")</f>
         <v/>
       </c>
-      <c r="J24" s="31">
+      <c r="J24" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C24:G24="Y"))*50</f>
         <v/>
       </c>
@@ -3649,11 +3705,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C25:G25,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="29">
         <f>COUNTIF(C25:G25,"Y")</f>
         <v/>
       </c>
-      <c r="J25" s="31">
+      <c r="J25" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C25:G25="Y"))*50</f>
         <v/>
       </c>
@@ -3692,11 +3748,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C26:G26,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I26" s="30">
+      <c r="I26" s="29">
         <f>COUNTIF(C26:G26,"Y")</f>
         <v/>
       </c>
-      <c r="J26" s="31">
+      <c r="J26" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C26:G26="Y"))*50</f>
         <v/>
       </c>
@@ -3719,11 +3775,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C27:G27,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I27" s="30">
+      <c r="I27" s="29">
         <f>COUNTIF(C27:G27,"Y")</f>
         <v/>
       </c>
-      <c r="J27" s="31">
+      <c r="J27" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C27:G27="Y"))*50</f>
         <v/>
       </c>
@@ -3754,11 +3810,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C28:G28,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I28" s="30">
+      <c r="I28" s="29">
         <f>COUNTIF(C28:G28,"Y")</f>
         <v/>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C28:G28="Y"))*50</f>
         <v/>
       </c>
@@ -3774,18 +3830,22 @@
       </c>
       <c r="C29" s="18" t="n"/>
       <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
+      <c r="E29" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F29" s="18" t="n"/>
       <c r="G29" s="18" t="n"/>
       <c r="H29" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C29:G29,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I29" s="30">
+      <c r="I29" s="29">
         <f>COUNTIF(C29:G29,"Y")</f>
         <v/>
       </c>
-      <c r="J29" s="31">
+      <c r="J29" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C29:G29="Y"))*50</f>
         <v/>
       </c>
@@ -3808,11 +3868,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C30:G30,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I30" s="30">
+      <c r="I30" s="29">
         <f>COUNTIF(C30:G30,"Y")</f>
         <v/>
       </c>
-      <c r="J30" s="31">
+      <c r="J30" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C30:G30="Y"))*50</f>
         <v/>
       </c>
@@ -3835,11 +3895,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C31:G31,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I31" s="30">
+      <c r="I31" s="29">
         <f>COUNTIF(C31:G31,"Y")</f>
         <v/>
       </c>
-      <c r="J31" s="31">
+      <c r="J31" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C31:G31="Y"))*50</f>
         <v/>
       </c>
@@ -3862,11 +3922,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C32:G32,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I32" s="30">
+      <c r="I32" s="29">
         <f>COUNTIF(C32:G32,"Y")</f>
         <v/>
       </c>
-      <c r="J32" s="31">
+      <c r="J32" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C32:G32="Y"))*50</f>
         <v/>
       </c>
@@ -3897,11 +3957,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C33:G33,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I33" s="30">
+      <c r="I33" s="29">
         <f>COUNTIF(C33:G33,"Y")</f>
         <v/>
       </c>
-      <c r="J33" s="31">
+      <c r="J33" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C33:G33="Y"))*50</f>
         <v/>
       </c>
@@ -3920,23 +3980,35 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D34" s="35" t="n"/>
-      <c r="E34" s="35" t="n"/>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F34" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G34" s="35" t="n"/>
+      <c r="G34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H34" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C34:G34,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I34" s="30">
+      <c r="I34" s="29">
         <f>COUNTIF(C34:G34,"Y")</f>
         <v/>
       </c>
-      <c r="J34" s="31">
+      <c r="J34" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C34:G34="Y"))*50</f>
         <v/>
       </c>
@@ -3959,11 +4031,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C35:G35,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I35" s="30">
+      <c r="I35" s="29">
         <f>COUNTIF(C35:G35,"Y")</f>
         <v/>
       </c>
-      <c r="J35" s="31">
+      <c r="J35" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C35:G35="Y"))*50</f>
         <v/>
       </c>
@@ -3986,11 +4058,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C36:G36,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I36" s="30">
+      <c r="I36" s="29">
         <f>COUNTIF(C36:G36,"Y")</f>
         <v/>
       </c>
-      <c r="J36" s="31">
+      <c r="J36" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C36:G36="Y"))*50</f>
         <v/>
       </c>
@@ -4017,11 +4089,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C37:G37,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I37" s="30">
+      <c r="I37" s="29">
         <f>COUNTIF(C37:G37,"Y")</f>
         <v/>
       </c>
-      <c r="J37" s="31">
+      <c r="J37" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C37:G37="Y"))*50</f>
         <v/>
       </c>
@@ -4044,11 +4116,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$G$7,C38:G38,"Y"),"")</f>
         <v/>
       </c>
-      <c r="I38" s="30">
+      <c r="I38" s="29">
         <f>COUNTIF(C38:G38,"Y")</f>
         <v/>
       </c>
-      <c r="J38" s="31">
+      <c r="J38" s="30">
         <f>SUMPRODUCT((C$7:$G$7=1)*(C38:G38="Y"))*50</f>
         <v/>
       </c>
@@ -4469,20 +4541,24 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D14" s="29" t="n"/>
-      <c r="E14" s="29" t="n"/>
-      <c r="F14" s="29" t="n"/>
-      <c r="G14" s="29" t="n"/>
-      <c r="H14" s="29" t="n"/>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
       <c r="I14" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C14:H14,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="29">
         <f>COUNTIF(C14:H14,"Y")</f>
         <v/>
       </c>
-      <c r="K14" s="31">
+      <c r="K14" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C14:H14="Y"))*50</f>
         <v/>
       </c>
@@ -4496,29 +4572,29 @@
           <t>Vicki L.</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n"/>
+      <c r="C15" s="31" t="n"/>
       <c r="D15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E15" s="29" t="n"/>
+      <c r="E15" s="31" t="n"/>
       <c r="F15" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G15" s="29" t="n"/>
-      <c r="H15" s="29" t="n"/>
+      <c r="G15" s="31" t="n"/>
+      <c r="H15" s="31" t="n"/>
       <c r="I15" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C15:H15,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="29">
         <f>COUNTIF(C15:H15,"Y")</f>
         <v/>
       </c>
-      <c r="K15" s="31">
+      <c r="K15" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C15:H15="Y"))*50</f>
         <v/>
       </c>
@@ -4542,23 +4618,27 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E16" s="29" t="n"/>
-      <c r="F16" s="29" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G16" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H16" s="29" t="n"/>
+      <c r="H16" s="31" t="n"/>
       <c r="I16" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C16:H16,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="29">
         <f>COUNTIF(C16:H16,"Y")</f>
         <v/>
       </c>
-      <c r="K16" s="31">
+      <c r="K16" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C16:H16="Y"))*50</f>
         <v/>
       </c>
@@ -4577,13 +4657,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D17" s="29" t="n"/>
+      <c r="D17" s="31" t="n"/>
       <c r="E17" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F17" s="29" t="n"/>
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G17" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4598,11 +4682,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C17:H17,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J17" s="30">
+      <c r="J17" s="29">
         <f>COUNTIF(C17:H17,"Y")</f>
         <v/>
       </c>
-      <c r="K17" s="31">
+      <c r="K17" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C17:H17="Y"))*50</f>
         <v/>
       </c>
@@ -4636,11 +4720,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C20:H20,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J20" s="30">
+      <c r="J20" s="29">
         <f>COUNTIF(C20:H20,"Y")</f>
         <v/>
       </c>
-      <c r="K20" s="31">
+      <c r="K20" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C20:H20="Y"))*50</f>
         <v/>
       </c>
@@ -4664,11 +4748,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C21:H21,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J21" s="30">
+      <c r="J21" s="29">
         <f>COUNTIF(C21:H21,"Y")</f>
         <v/>
       </c>
-      <c r="K21" s="31">
+      <c r="K21" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C21:H21="Y"))*50</f>
         <v/>
       </c>
@@ -4700,11 +4784,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C22:H22,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J22" s="30">
+      <c r="J22" s="29">
         <f>COUNTIF(C22:H22,"Y")</f>
         <v/>
       </c>
-      <c r="K22" s="31">
+      <c r="K22" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C22:H22="Y"))*50</f>
         <v/>
       </c>
@@ -4732,11 +4816,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C23:H23,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J23" s="30">
+      <c r="J23" s="29">
         <f>COUNTIF(C23:H23,"Y")</f>
         <v/>
       </c>
-      <c r="K23" s="31">
+      <c r="K23" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C23:H23="Y"))*50</f>
         <v/>
       </c>
@@ -4764,11 +4848,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C24:H24,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J24" s="30">
+      <c r="J24" s="29">
         <f>COUNTIF(C24:H24,"Y")</f>
         <v/>
       </c>
-      <c r="K24" s="31">
+      <c r="K24" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C24:H24="Y"))*50</f>
         <v/>
       </c>
@@ -4792,11 +4876,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C25:H25,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J25" s="30">
+      <c r="J25" s="29">
         <f>COUNTIF(C25:H25,"Y")</f>
         <v/>
       </c>
-      <c r="K25" s="31">
+      <c r="K25" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C25:H25="Y"))*50</f>
         <v/>
       </c>
@@ -4832,11 +4916,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C26:H26,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J26" s="30">
+      <c r="J26" s="29">
         <f>COUNTIF(C26:H26,"Y")</f>
         <v/>
       </c>
-      <c r="K26" s="31">
+      <c r="K26" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C26:H26="Y"))*50</f>
         <v/>
       </c>
@@ -4860,11 +4944,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C27:H27,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J27" s="30">
+      <c r="J27" s="29">
         <f>COUNTIF(C27:H27,"Y")</f>
         <v/>
       </c>
-      <c r="K27" s="31">
+      <c r="K27" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C27:H27="Y"))*50</f>
         <v/>
       </c>
@@ -4892,11 +4976,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C28:H28,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J28" s="30">
+      <c r="J28" s="29">
         <f>COUNTIF(C28:H28,"Y")</f>
         <v/>
       </c>
-      <c r="K28" s="31">
+      <c r="K28" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C28:H28="Y"))*50</f>
         <v/>
       </c>
@@ -4925,18 +5009,22 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F29" s="18" t="n"/>
+      <c r="F29" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G29" s="18" t="n"/>
       <c r="H29" s="18" t="n"/>
       <c r="I29" s="17">
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C29:H29,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J29" s="30">
+      <c r="J29" s="29">
         <f>COUNTIF(C29:H29,"Y")</f>
         <v/>
       </c>
-      <c r="K29" s="31">
+      <c r="K29" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C29:H29="Y"))*50</f>
         <v/>
       </c>
@@ -4960,11 +5048,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C30:H30,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J30" s="30">
+      <c r="J30" s="29">
         <f>COUNTIF(C30:H30,"Y")</f>
         <v/>
       </c>
-      <c r="K30" s="31">
+      <c r="K30" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C30:H30="Y"))*50</f>
         <v/>
       </c>
@@ -4988,11 +5076,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C31:H31,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J31" s="30">
+      <c r="J31" s="29">
         <f>COUNTIF(C31:H31,"Y")</f>
         <v/>
       </c>
-      <c r="K31" s="31">
+      <c r="K31" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C31:H31="Y"))*50</f>
         <v/>
       </c>
@@ -5016,11 +5104,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C32:H32,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J32" s="30">
+      <c r="J32" s="29">
         <f>COUNTIF(C32:H32,"Y")</f>
         <v/>
       </c>
-      <c r="K32" s="31">
+      <c r="K32" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C32:H32="Y"))*50</f>
         <v/>
       </c>
@@ -5056,11 +5144,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C33:H33,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J33" s="30">
+      <c r="J33" s="29">
         <f>COUNTIF(C33:H33,"Y")</f>
         <v/>
       </c>
-      <c r="K33" s="31">
+      <c r="K33" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C33:H33="Y"))*50</f>
         <v/>
       </c>
@@ -5079,9 +5167,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D34" s="35" t="n"/>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E34" s="35" t="n"/>
-      <c r="F34" s="35" t="n"/>
+      <c r="F34" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G34" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5092,11 +5188,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C34:H34,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J34" s="30">
+      <c r="J34" s="29">
         <f>COUNTIF(C34:H34,"Y")</f>
         <v/>
       </c>
-      <c r="K34" s="31">
+      <c r="K34" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C34:H34="Y"))*50</f>
         <v/>
       </c>
@@ -5120,11 +5216,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C35:H35,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J35" s="30">
+      <c r="J35" s="29">
         <f>COUNTIF(C35:H35,"Y")</f>
         <v/>
       </c>
-      <c r="K35" s="31">
+      <c r="K35" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C35:H35="Y"))*50</f>
         <v/>
       </c>
@@ -5143,7 +5239,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D36" s="35" t="n"/>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E36" s="35" t="n"/>
       <c r="F36" s="28" t="inlineStr">
         <is>
@@ -5160,11 +5260,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C36:H36,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J36" s="30">
+      <c r="J36" s="29">
         <f>COUNTIF(C36:H36,"Y")</f>
         <v/>
       </c>
-      <c r="K36" s="31">
+      <c r="K36" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C36:H36="Y"))*50</f>
         <v/>
       </c>
@@ -5192,11 +5292,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C37:H37,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J37" s="30">
+      <c r="J37" s="29">
         <f>COUNTIF(C37:H37,"Y")</f>
         <v/>
       </c>
-      <c r="K37" s="31">
+      <c r="K37" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C37:H37="Y"))*50</f>
         <v/>
       </c>
@@ -5220,11 +5320,11 @@
         <f>IFERROR(AVERAGEIFS($C$7:$H$7,C38:H38,"Y"),"")</f>
         <v/>
       </c>
-      <c r="J38" s="30">
+      <c r="J38" s="29">
         <f>COUNTIF(C38:H38,"Y")</f>
         <v/>
       </c>
-      <c r="K38" s="31">
+      <c r="K38" s="30">
         <f>SUMPRODUCT((C$7:$H$7=1)*(C38:H38="Y"))*50</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
April shop tracker — locked in with exact visit-time windows
Bobby provided the exact visit-time bucket from Marketforce for each
April shop. Applied 30-min minimum overlap rule against the actual
shop window (not the broad meal-period label).

April visit windows:
  4/2  Dinner   → 7-10 PM
  4/9  Lunch    → 11-1:30 PM
  4/11 Dinner   → 7:30-10 PM
  4/17 Lunch    → 11-1:30 PM
  4/23 Dinner   → 4-7 PM
  4/25 Lunch    → 1:30-4 PM

Jan-Mar still use approximate meal-period windows pending visit times.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -4541,11 +4541,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D14" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D14" s="31" t="n"/>
       <c r="E14" s="31" t="n"/>
       <c r="F14" s="31" t="n"/>
       <c r="G14" s="31" t="n"/>
@@ -4608,22 +4604,14 @@
           <t>Kasey W.</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C16" s="31" t="n"/>
       <c r="D16" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="E16" s="31" t="n"/>
-      <c r="F16" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F16" s="31" t="n"/>
       <c r="G16" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4652,22 +4640,14 @@
           <t>Nathan R.</t>
         </is>
       </c>
-      <c r="C17" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C17" s="31" t="n"/>
       <c r="D17" s="31" t="n"/>
       <c r="E17" s="28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F17" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F17" s="31" t="n"/>
       <c r="G17" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4894,11 +4874,7 @@
           <t>Francisco</t>
         </is>
       </c>
-      <c r="C26" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C26" s="35" t="n"/>
       <c r="D26" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5009,11 +4985,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F29" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="18" t="n"/>
       <c r="H29" s="18" t="n"/>
       <c r="I29" s="17">
@@ -5167,17 +5139,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D34" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D34" s="35" t="n"/>
       <c r="E34" s="35" t="n"/>
-      <c r="F34" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F34" s="35" t="n"/>
       <c r="G34" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5239,12 +5203,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D36" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E36" s="35" t="n"/>
+      <c r="D36" s="35" t="n"/>
+      <c r="E36" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F36" s="28" t="inlineStr">
         <is>
           <t>Y</t>

</xml_diff>

<commit_message>
Refresh shop tracker with full 22-shop participation
Pipeline now end-to-end working in CI: visit-time → CETD → tracker.
Local rebuild ensures the XLSX in repo reflects current data even if
CI's openpyxl produced bytewise-identical output.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -2270,11 +2270,7 @@
           <t>Vicki L.</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C15" s="31" t="n"/>
       <c r="D15" s="31" t="n"/>
       <c r="E15" s="28" t="inlineStr">
         <is>
@@ -2310,11 +2306,7 @@
           <t>Kasey W.</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C16" s="31" t="n"/>
       <c r="D16" s="31" t="n"/>
       <c r="E16" s="31" t="n"/>
       <c r="F16" s="28" t="inlineStr">
@@ -2350,11 +2342,7 @@
           <t>Nathan R.</t>
         </is>
       </c>
-      <c r="C17" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C17" s="31" t="n"/>
       <c r="D17" s="31" t="n"/>
       <c r="E17" s="31" t="n"/>
       <c r="F17" s="31" t="n"/>
@@ -2836,11 +2824,7 @@
           <t>Maylin</t>
         </is>
       </c>
-      <c r="C34" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C34" s="35" t="n"/>
       <c r="D34" s="28" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2884,7 +2868,11 @@
           <t>Mike</t>
         </is>
       </c>
-      <c r="C35" s="18" t="n"/>
+      <c r="C35" s="28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D35" s="18" t="n"/>
       <c r="E35" s="28" t="inlineStr">
         <is>
@@ -2924,11 +2912,7 @@
           <t>Richard</t>
         </is>
       </c>
-      <c r="C36" s="28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="C36" s="35" t="n"/>
       <c r="D36" s="35" t="n"/>
       <c r="E36" s="35" t="n"/>
       <c r="F36" s="35" t="n"/>

</xml_diff>

<commit_message>
Daily dashboard refresh — 2026-05-14 (business date 05-13)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -7438,7 +7438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7452,9 +7452,10 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -7467,7 +7468,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Five Guys Store 2065 · Louisville, KY · 9 shops · Source: Marketforce + CrunchTime</t>
+          <t>Five Guys Store 2065 · Louisville, KY · 10 shops · Source: Marketforce + CrunchTime</t>
         </is>
       </c>
     </row>
@@ -7524,17 +7525,22 @@
           <t>#9</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>AVG</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>BONUS</t>
         </is>
@@ -7592,9 +7598,14 @@
           <t>05/01</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>05/11</t>
+        </is>
+      </c>
       <c r="M5" s="7" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr"/>
+      <c r="O5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="7" t="inlineStr"/>
@@ -7648,9 +7659,14 @@
           <t>L</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr"/>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="M6" s="7" t="inlineStr"/>
       <c r="N6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="12" t="inlineStr"/>
@@ -7686,12 +7702,15 @@
       <c r="K7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="18">
-        <f>IFERROR(AVERAGE(C7:K7),"")</f>
-        <v/>
-      </c>
-      <c r="M7" s="12" t="inlineStr"/>
+      <c r="L7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="18">
+        <f>IFERROR(AVERAGE(C7:L7),"")</f>
+        <v/>
+      </c>
       <c r="N7" s="12" t="inlineStr"/>
+      <c r="O7" s="12" t="inlineStr"/>
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="19" t="inlineStr"/>
@@ -7709,12 +7728,13 @@
       <c r="I8" s="19" t="inlineStr"/>
       <c r="J8" s="19" t="inlineStr"/>
       <c r="K8" s="19" t="inlineStr"/>
-      <c r="L8" s="21">
-        <f>IFERROR(AVERAGE(C8:K8),"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="19" t="inlineStr"/>
+      <c r="L8" s="19" t="inlineStr"/>
+      <c r="M8" s="21">
+        <f>IFERROR(AVERAGE(C8:L8),"")</f>
+        <v/>
+      </c>
       <c r="N8" s="19" t="inlineStr"/>
+      <c r="O8" s="19" t="inlineStr"/>
     </row>
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="19" t="inlineStr"/>
@@ -7732,12 +7752,13 @@
       <c r="I9" s="19" t="inlineStr"/>
       <c r="J9" s="19" t="inlineStr"/>
       <c r="K9" s="19" t="inlineStr"/>
-      <c r="L9" s="21">
-        <f>IFERROR(AVERAGE(C9:K9),"")</f>
-        <v/>
-      </c>
-      <c r="M9" s="19" t="inlineStr"/>
+      <c r="L9" s="19" t="inlineStr"/>
+      <c r="M9" s="21">
+        <f>IFERROR(AVERAGE(C9:L9),"")</f>
+        <v/>
+      </c>
       <c r="N9" s="19" t="inlineStr"/>
+      <c r="O9" s="19" t="inlineStr"/>
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="19" t="inlineStr"/>
@@ -7755,12 +7776,13 @@
       <c r="I10" s="19" t="inlineStr"/>
       <c r="J10" s="19" t="inlineStr"/>
       <c r="K10" s="19" t="inlineStr"/>
-      <c r="L10" s="21">
-        <f>IFERROR(AVERAGE(C10:K10),"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="19" t="inlineStr"/>
+      <c r="L10" s="19" t="inlineStr"/>
+      <c r="M10" s="21">
+        <f>IFERROR(AVERAGE(C10:L10),"")</f>
+        <v/>
+      </c>
       <c r="N10" s="19" t="inlineStr"/>
+      <c r="O10" s="19" t="inlineStr"/>
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="19" t="inlineStr"/>
@@ -7778,12 +7800,13 @@
       <c r="I11" s="19" t="inlineStr"/>
       <c r="J11" s="19" t="inlineStr"/>
       <c r="K11" s="19" t="inlineStr"/>
-      <c r="L11" s="21">
-        <f>IFERROR(AVERAGE(C11:K11),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="19" t="inlineStr"/>
+      <c r="L11" s="19" t="inlineStr"/>
+      <c r="M11" s="21">
+        <f>IFERROR(AVERAGE(C11:L11),"")</f>
+        <v/>
+      </c>
       <c r="N11" s="19" t="inlineStr"/>
+      <c r="O11" s="19" t="inlineStr"/>
     </row>
     <row r="12" ht="6" customHeight="1">
       <c r="A12" s="22" t="n"/>
@@ -7841,16 +7864,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L14" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C14:K14,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="28">
-        <f>COUNTIF(C14:K14,"Y")</f>
-        <v/>
-      </c>
-      <c r="N14" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C14:K14="Y"))*50</f>
+      <c r="L14" s="27" t="n"/>
+      <c r="M14" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C14:L14,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="28">
+        <f>COUNTIF(C14:L14,"Y")</f>
+        <v/>
+      </c>
+      <c r="O14" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C14:L14="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -7876,16 +7900,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L15" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C15:K15,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M15" s="28">
-        <f>COUNTIF(C15:K15,"Y")</f>
-        <v/>
-      </c>
-      <c r="N15" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C15:K15="Y"))*50</f>
+      <c r="L15" s="27" t="n"/>
+      <c r="M15" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C15:L15,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="28">
+        <f>COUNTIF(C15:L15,"Y")</f>
+        <v/>
+      </c>
+      <c r="O15" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C15:L15="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -7907,16 +7932,17 @@
       <c r="I16" s="27" t="n"/>
       <c r="J16" s="27" t="n"/>
       <c r="K16" s="27" t="n"/>
-      <c r="L16" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C16:K16,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M16" s="28">
-        <f>COUNTIF(C16:K16,"Y")</f>
-        <v/>
-      </c>
-      <c r="N16" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C16:K16="Y"))*50</f>
+      <c r="L16" s="27" t="n"/>
+      <c r="M16" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C16:L16,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="28">
+        <f>COUNTIF(C16:L16,"Y")</f>
+        <v/>
+      </c>
+      <c r="O16" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C16:L16="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -7938,16 +7964,17 @@
       <c r="I17" s="27" t="n"/>
       <c r="J17" s="27" t="n"/>
       <c r="K17" s="27" t="n"/>
-      <c r="L17" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C17:K17,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M17" s="28">
-        <f>COUNTIF(C17:K17,"Y")</f>
-        <v/>
-      </c>
-      <c r="N17" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C17:K17="Y"))*50</f>
+      <c r="L17" s="27" t="n"/>
+      <c r="M17" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C17:L17,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="28">
+        <f>COUNTIF(C17:L17,"Y")</f>
+        <v/>
+      </c>
+      <c r="O17" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C17:L17="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -7979,16 +8006,17 @@
       <c r="I20" s="33" t="n"/>
       <c r="J20" s="33" t="n"/>
       <c r="K20" s="33" t="n"/>
-      <c r="L20" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C20:K20,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="28">
-        <f>COUNTIF(C20:K20,"Y")</f>
-        <v/>
-      </c>
-      <c r="N20" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C20:K20="Y"))*50</f>
+      <c r="L20" s="33" t="n"/>
+      <c r="M20" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C20:L20,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="28">
+        <f>COUNTIF(C20:L20,"Y")</f>
+        <v/>
+      </c>
+      <c r="O20" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C20:L20="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8010,16 +8038,17 @@
       <c r="I21" s="19" t="n"/>
       <c r="J21" s="19" t="n"/>
       <c r="K21" s="19" t="n"/>
-      <c r="L21" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C21:K21,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M21" s="28">
-        <f>COUNTIF(C21:K21,"Y")</f>
-        <v/>
-      </c>
-      <c r="N21" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C21:K21="Y"))*50</f>
+      <c r="L21" s="19" t="n"/>
+      <c r="M21" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C21:L21,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N21" s="28">
+        <f>COUNTIF(C21:L21,"Y")</f>
+        <v/>
+      </c>
+      <c r="O21" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C21:L21="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8049,16 +8078,17 @@
       <c r="I22" s="33" t="n"/>
       <c r="J22" s="33" t="n"/>
       <c r="K22" s="33" t="n"/>
-      <c r="L22" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C22:K22,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M22" s="28">
-        <f>COUNTIF(C22:K22,"Y")</f>
-        <v/>
-      </c>
-      <c r="N22" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C22:K22="Y"))*50</f>
+      <c r="L22" s="33" t="n"/>
+      <c r="M22" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C22:L22,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N22" s="28">
+        <f>COUNTIF(C22:L22,"Y")</f>
+        <v/>
+      </c>
+      <c r="O22" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C22:L22="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8080,16 +8110,17 @@
       <c r="I23" s="19" t="n"/>
       <c r="J23" s="19" t="n"/>
       <c r="K23" s="19" t="n"/>
-      <c r="L23" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C23:K23,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M23" s="28">
-        <f>COUNTIF(C23:K23,"Y")</f>
-        <v/>
-      </c>
-      <c r="N23" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C23:K23="Y"))*50</f>
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C23:L23,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="28">
+        <f>COUNTIF(C23:L23,"Y")</f>
+        <v/>
+      </c>
+      <c r="O23" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C23:L23="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8111,16 +8142,17 @@
       <c r="I24" s="33" t="n"/>
       <c r="J24" s="33" t="n"/>
       <c r="K24" s="33" t="n"/>
-      <c r="L24" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C24:K24,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M24" s="28">
-        <f>COUNTIF(C24:K24,"Y")</f>
-        <v/>
-      </c>
-      <c r="N24" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C24:K24="Y"))*50</f>
+      <c r="L24" s="33" t="n"/>
+      <c r="M24" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C24:L24,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="28">
+        <f>COUNTIF(C24:L24,"Y")</f>
+        <v/>
+      </c>
+      <c r="O24" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C24:L24="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8142,16 +8174,17 @@
       <c r="I25" s="19" t="n"/>
       <c r="J25" s="19" t="n"/>
       <c r="K25" s="19" t="n"/>
-      <c r="L25" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C25:K25,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M25" s="28">
-        <f>COUNTIF(C25:K25,"Y")</f>
-        <v/>
-      </c>
-      <c r="N25" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C25:K25="Y"))*50</f>
+      <c r="L25" s="19" t="n"/>
+      <c r="M25" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C25:L25,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="28">
+        <f>COUNTIF(C25:L25,"Y")</f>
+        <v/>
+      </c>
+      <c r="O25" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C25:L25="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8181,16 +8214,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L26" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C26:K26,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M26" s="28">
-        <f>COUNTIF(C26:K26,"Y")</f>
-        <v/>
-      </c>
-      <c r="N26" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C26:K26="Y"))*50</f>
+      <c r="L26" s="33" t="n"/>
+      <c r="M26" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C26:L26,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="28">
+        <f>COUNTIF(C26:L26,"Y")</f>
+        <v/>
+      </c>
+      <c r="O26" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C26:L26="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8212,16 +8246,17 @@
       <c r="I27" s="19" t="n"/>
       <c r="J27" s="19" t="n"/>
       <c r="K27" s="19" t="n"/>
-      <c r="L27" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C27:K27,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="28">
-        <f>COUNTIF(C27:K27,"Y")</f>
-        <v/>
-      </c>
-      <c r="N27" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C27:K27="Y"))*50</f>
+      <c r="L27" s="19" t="n"/>
+      <c r="M27" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C27:L27,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="28">
+        <f>COUNTIF(C27:L27,"Y")</f>
+        <v/>
+      </c>
+      <c r="O27" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C27:L27="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8243,16 +8278,17 @@
       <c r="I28" s="33" t="n"/>
       <c r="J28" s="33" t="n"/>
       <c r="K28" s="33" t="n"/>
-      <c r="L28" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C28:K28,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="28">
-        <f>COUNTIF(C28:K28,"Y")</f>
-        <v/>
-      </c>
-      <c r="N28" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C28:K28="Y"))*50</f>
+      <c r="L28" s="33" t="n"/>
+      <c r="M28" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C28:L28,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="28">
+        <f>COUNTIF(C28:L28,"Y")</f>
+        <v/>
+      </c>
+      <c r="O28" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C28:L28="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8302,16 +8338,17 @@
         </is>
       </c>
       <c r="K29" s="19" t="n"/>
-      <c r="L29" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C29:K29,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="28">
-        <f>COUNTIF(C29:K29,"Y")</f>
-        <v/>
-      </c>
-      <c r="N29" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C29:K29="Y"))*50</f>
+      <c r="L29" s="19" t="n"/>
+      <c r="M29" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C29:L29,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N29" s="28">
+        <f>COUNTIF(C29:L29,"Y")</f>
+        <v/>
+      </c>
+      <c r="O29" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C29:L29="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8333,16 +8370,17 @@
       <c r="I30" s="33" t="n"/>
       <c r="J30" s="33" t="n"/>
       <c r="K30" s="33" t="n"/>
-      <c r="L30" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C30:K30,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="28">
-        <f>COUNTIF(C30:K30,"Y")</f>
-        <v/>
-      </c>
-      <c r="N30" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C30:K30="Y"))*50</f>
+      <c r="L30" s="33" t="n"/>
+      <c r="M30" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C30:L30,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N30" s="28">
+        <f>COUNTIF(C30:L30,"Y")</f>
+        <v/>
+      </c>
+      <c r="O30" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C30:L30="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8364,16 +8402,17 @@
       <c r="I31" s="19" t="n"/>
       <c r="J31" s="19" t="n"/>
       <c r="K31" s="19" t="n"/>
-      <c r="L31" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C31:K31,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M31" s="28">
-        <f>COUNTIF(C31:K31,"Y")</f>
-        <v/>
-      </c>
-      <c r="N31" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C31:K31="Y"))*50</f>
+      <c r="L31" s="19" t="n"/>
+      <c r="M31" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C31:L31,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N31" s="28">
+        <f>COUNTIF(C31:L31,"Y")</f>
+        <v/>
+      </c>
+      <c r="O31" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C31:L31="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8395,16 +8434,17 @@
       <c r="I32" s="33" t="n"/>
       <c r="J32" s="33" t="n"/>
       <c r="K32" s="33" t="n"/>
-      <c r="L32" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C32:K32,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="28">
-        <f>COUNTIF(C32:K32,"Y")</f>
-        <v/>
-      </c>
-      <c r="N32" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C32:K32="Y"))*50</f>
+      <c r="L32" s="33" t="n"/>
+      <c r="M32" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C32:L32,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N32" s="28">
+        <f>COUNTIF(C32:L32,"Y")</f>
+        <v/>
+      </c>
+      <c r="O32" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C32:L32="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8438,16 +8478,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L33" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C33:K33,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="28">
-        <f>COUNTIF(C33:K33,"Y")</f>
-        <v/>
-      </c>
-      <c r="N33" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C33:K33="Y"))*50</f>
+      <c r="L33" s="19" t="n"/>
+      <c r="M33" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C33:L33,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N33" s="28">
+        <f>COUNTIF(C33:L33,"Y")</f>
+        <v/>
+      </c>
+      <c r="O33" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C33:L33="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8473,16 +8514,17 @@
       <c r="I34" s="33" t="n"/>
       <c r="J34" s="33" t="n"/>
       <c r="K34" s="33" t="n"/>
-      <c r="L34" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C34:K34,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M34" s="28">
-        <f>COUNTIF(C34:K34,"Y")</f>
-        <v/>
-      </c>
-      <c r="N34" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C34:K34="Y"))*50</f>
+      <c r="L34" s="33" t="n"/>
+      <c r="M34" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C34:L34,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="28">
+        <f>COUNTIF(C34:L34,"Y")</f>
+        <v/>
+      </c>
+      <c r="O34" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C34:L34="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8504,16 +8546,17 @@
       <c r="I35" s="19" t="n"/>
       <c r="J35" s="19" t="n"/>
       <c r="K35" s="19" t="n"/>
-      <c r="L35" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C35:K35,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M35" s="28">
-        <f>COUNTIF(C35:K35,"Y")</f>
-        <v/>
-      </c>
-      <c r="N35" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C35:K35="Y"))*50</f>
+      <c r="L35" s="19" t="n"/>
+      <c r="M35" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C35:L35,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N35" s="28">
+        <f>COUNTIF(C35:L35,"Y")</f>
+        <v/>
+      </c>
+      <c r="O35" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C35:L35="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8535,16 +8578,17 @@
       <c r="I36" s="33" t="n"/>
       <c r="J36" s="33" t="n"/>
       <c r="K36" s="33" t="n"/>
-      <c r="L36" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C36:K36,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M36" s="28">
-        <f>COUNTIF(C36:K36,"Y")</f>
-        <v/>
-      </c>
-      <c r="N36" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C36:K36="Y"))*50</f>
+      <c r="L36" s="33" t="n"/>
+      <c r="M36" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C36:L36,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N36" s="28">
+        <f>COUNTIF(C36:L36,"Y")</f>
+        <v/>
+      </c>
+      <c r="O36" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C36:L36="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8578,16 +8622,17 @@
       </c>
       <c r="J37" s="19" t="n"/>
       <c r="K37" s="19" t="n"/>
-      <c r="L37" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C37:K37,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M37" s="28">
-        <f>COUNTIF(C37:K37,"Y")</f>
-        <v/>
-      </c>
-      <c r="N37" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C37:K37="Y"))*50</f>
+      <c r="L37" s="19" t="n"/>
+      <c r="M37" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C37:L37,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N37" s="28">
+        <f>COUNTIF(C37:L37,"Y")</f>
+        <v/>
+      </c>
+      <c r="O37" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C37:L37="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8609,16 +8654,17 @@
       <c r="I38" s="33" t="n"/>
       <c r="J38" s="33" t="n"/>
       <c r="K38" s="33" t="n"/>
-      <c r="L38" s="18">
-        <f>IFERROR(AVERAGEIFS($C$7:$K$7,C38:K38,"Y"),"")</f>
-        <v/>
-      </c>
-      <c r="M38" s="28">
-        <f>COUNTIF(C38:K38,"Y")</f>
-        <v/>
-      </c>
-      <c r="N38" s="29">
-        <f>SUMPRODUCT((C$7:$K$7=1)*(C38:K38="Y"))*50</f>
+      <c r="L38" s="33" t="n"/>
+      <c r="M38" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$L$7,C38:L38,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="N38" s="28">
+        <f>COUNTIF(C38:L38,"Y")</f>
+        <v/>
+      </c>
+      <c r="O38" s="29">
+        <f>SUMPRODUCT((C$7:$L$7=1)*(C38:L38="Y"))*50</f>
         <v/>
       </c>
     </row>
@@ -8665,13 +8711,17 @@
         <f>COUNTIF(K14:K38,"Y")</f>
         <v/>
       </c>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="6">
-        <f>SUM(M14:M38)</f>
-        <v/>
-      </c>
-      <c r="N39" s="37">
+      <c r="L39" s="6">
+        <f>COUNTIF(L14:L38,"Y")</f>
+        <v/>
+      </c>
+      <c r="M39" s="3" t="inlineStr"/>
+      <c r="N39" s="6">
         <f>SUM(N14:N38)</f>
+        <v/>
+      </c>
+      <c r="O39" s="37">
+        <f>SUM(O14:O38)</f>
         <v/>
       </c>
     </row>
@@ -8684,13 +8734,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A40:N40"/>
-    <mergeCell ref="A18:N18"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A19:N19"/>
-    <mergeCell ref="A13:N13"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A12:O12"/>
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A13:O13"/>
+    <mergeCell ref="A19:O19"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A40:O40"/>
+    <mergeCell ref="A18:O18"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
shops: fill participation + payout draft for job 20770900 (May 11 Dinner 100%)
Manually ran pipeline to unblock 100% shop payout for job 20770900.
Participation pulled from CrunchTime CETD: Bri, Dakayla, Francisco,
Madison, Maylin. Payout draft written to data/drafts/. Emailed.json
updated. Shop tracker Excel rebuilt. Dashboard wired.
Fixed Windows cp1252 encoding crash in scrape_shop_participation.py.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -7864,7 +7864,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L14" s="27" t="n"/>
+      <c r="L14" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M14" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$L$7,C14:L14,"Y"),"")</f>
         <v/>
@@ -8110,7 +8114,11 @@
       <c r="I23" s="19" t="n"/>
       <c r="J23" s="19" t="n"/>
       <c r="K23" s="19" t="n"/>
-      <c r="L23" s="19" t="n"/>
+      <c r="L23" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M23" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$L$7,C23:L23,"Y"),"")</f>
         <v/>
@@ -8142,7 +8150,11 @@
       <c r="I24" s="33" t="n"/>
       <c r="J24" s="33" t="n"/>
       <c r="K24" s="33" t="n"/>
-      <c r="L24" s="33" t="n"/>
+      <c r="L24" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M24" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$L$7,C24:L24,"Y"),"")</f>
         <v/>
@@ -8214,7 +8226,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="L26" s="33" t="n"/>
+      <c r="L26" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M26" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$L$7,C26:L26,"Y"),"")</f>
         <v/>
@@ -8514,7 +8530,11 @@
       <c r="I34" s="33" t="n"/>
       <c r="J34" s="33" t="n"/>
       <c r="K34" s="33" t="n"/>
-      <c r="L34" s="33" t="n"/>
+      <c r="L34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M34" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$L$7,C34:L34,"Y"),"")</f>
         <v/>

</xml_diff>

<commit_message>
daily: 2026-05-27 scrape — sales $3,558, labor 24.8%, compliance 57%
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Daily brief 2026-06-11 — team notes + dashboard wire + shop refresh (6/04 Lunch 100%)
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
shop tracker: add June; latest shop 2026-06-04 100% Lunch
MONTHS dict + build loop extended to include month 6 (June).
Shop_Tracker_2065_2026.xlsx regenerated — June tab now present
with job 20808696 (2026-06-04, Lunch, 100%, on-shift: Robert
Cline, DaKayla Dorsey, Lidy Henry, Nathan Roberts, Kasey Wilson,
Jada Cox).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9050,4 +9051,1394 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="1" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SECRET SHOPPER SCORES — JUNE 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Five Guys Store 2065 · Louisville, KY · 11 shops · Source: Marketforce + CrunchTime</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="4" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>SHOP →</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>#7</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>#8</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>#11</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>BONUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="7" t="inlineStr"/>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>06/02</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>06/06</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>06/11</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>06/14</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>06/19</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>06/20</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>06/21</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>06/26</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>06/28</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>06/02</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>06/04</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr"/>
+      <c r="O5" s="7" t="inlineStr"/>
+      <c r="P5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="7" t="inlineStr"/>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Meal</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr"/>
+      <c r="P6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="12" t="inlineStr"/>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Total Score</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="17" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="18">
+        <f>IFERROR(AVERAGE(C7:M7),"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="12" t="inlineStr"/>
+      <c r="P7" s="12" t="inlineStr"/>
+    </row>
+    <row r="8" ht="13" customHeight="1">
+      <c r="A8" s="19" t="inlineStr"/>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr"/>
+      <c r="D8" s="19" t="inlineStr"/>
+      <c r="E8" s="19" t="inlineStr"/>
+      <c r="F8" s="19" t="inlineStr"/>
+      <c r="G8" s="19" t="inlineStr"/>
+      <c r="H8" s="19" t="inlineStr"/>
+      <c r="I8" s="19" t="inlineStr"/>
+      <c r="J8" s="19" t="inlineStr"/>
+      <c r="K8" s="19" t="inlineStr"/>
+      <c r="L8" s="19" t="inlineStr"/>
+      <c r="M8" s="19" t="inlineStr"/>
+      <c r="N8" s="21">
+        <f>IFERROR(AVERAGE(C8:M8),"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="19" t="inlineStr"/>
+      <c r="P8" s="19" t="inlineStr"/>
+    </row>
+    <row r="9" ht="13" customHeight="1">
+      <c r="A9" s="19" t="inlineStr"/>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr"/>
+      <c r="D9" s="19" t="inlineStr"/>
+      <c r="E9" s="19" t="inlineStr"/>
+      <c r="F9" s="19" t="inlineStr"/>
+      <c r="G9" s="19" t="inlineStr"/>
+      <c r="H9" s="19" t="inlineStr"/>
+      <c r="I9" s="19" t="inlineStr"/>
+      <c r="J9" s="19" t="inlineStr"/>
+      <c r="K9" s="19" t="inlineStr"/>
+      <c r="L9" s="19" t="inlineStr"/>
+      <c r="M9" s="19" t="inlineStr"/>
+      <c r="N9" s="21">
+        <f>IFERROR(AVERAGE(C9:M9),"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="19" t="inlineStr"/>
+      <c r="P9" s="19" t="inlineStr"/>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="19" t="inlineStr"/>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Cleanliness</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr"/>
+      <c r="D10" s="19" t="inlineStr"/>
+      <c r="E10" s="19" t="inlineStr"/>
+      <c r="F10" s="19" t="inlineStr"/>
+      <c r="G10" s="19" t="inlineStr"/>
+      <c r="H10" s="19" t="inlineStr"/>
+      <c r="I10" s="19" t="inlineStr"/>
+      <c r="J10" s="19" t="inlineStr"/>
+      <c r="K10" s="19" t="inlineStr"/>
+      <c r="L10" s="19" t="inlineStr"/>
+      <c r="M10" s="19" t="inlineStr"/>
+      <c r="N10" s="21">
+        <f>IFERROR(AVERAGE(C10:M10),"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="19" t="inlineStr"/>
+      <c r="P10" s="19" t="inlineStr"/>
+    </row>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="19" t="inlineStr"/>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Customer Sat</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr"/>
+      <c r="D11" s="19" t="inlineStr"/>
+      <c r="E11" s="19" t="inlineStr"/>
+      <c r="F11" s="19" t="inlineStr"/>
+      <c r="G11" s="19" t="inlineStr"/>
+      <c r="H11" s="19" t="inlineStr"/>
+      <c r="I11" s="19" t="inlineStr"/>
+      <c r="J11" s="19" t="inlineStr"/>
+      <c r="K11" s="19" t="inlineStr"/>
+      <c r="L11" s="19" t="inlineStr"/>
+      <c r="M11" s="19" t="inlineStr"/>
+      <c r="N11" s="21">
+        <f>IFERROR(AVERAGE(C11:M11),"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="19" t="inlineStr"/>
+      <c r="P11" s="19" t="inlineStr"/>
+    </row>
+    <row r="12" ht="6" customHeight="1">
+      <c r="A12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>MANAGERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>Madison C.</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="n"/>
+      <c r="D14" s="27" t="n"/>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G14" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I14" s="27" t="n"/>
+      <c r="J14" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K14" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L14" s="27" t="n"/>
+      <c r="M14" s="27" t="n"/>
+      <c r="N14" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C14:M14,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="28">
+        <f>COUNTIF(C14:M14,"Y")</f>
+        <v/>
+      </c>
+      <c r="P14" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C14:M14="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>Vicki L.</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="n"/>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="n"/>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I15" s="27" t="n"/>
+      <c r="J15" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M15" s="27" t="n"/>
+      <c r="N15" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C15:M15,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="28">
+        <f>COUNTIF(C15:M15,"Y")</f>
+        <v/>
+      </c>
+      <c r="P15" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C15:M15="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>Kasey W.</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="27" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="27" t="n"/>
+      <c r="K16" s="27" t="n"/>
+      <c r="L16" s="27" t="n"/>
+      <c r="M16" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N16" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C16:M16,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="28">
+        <f>COUNTIF(C16:M16,"Y")</f>
+        <v/>
+      </c>
+      <c r="P16" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C16:M16="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>Nathan R.</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="n"/>
+      <c r="D17" s="27" t="n"/>
+      <c r="E17" s="27" t="n"/>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="27" t="n"/>
+      <c r="I17" s="27" t="n"/>
+      <c r="J17" s="27" t="n"/>
+      <c r="K17" s="27" t="n"/>
+      <c r="L17" s="27" t="n"/>
+      <c r="M17" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C17:M17,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="28">
+        <f>COUNTIF(C17:M17,"Y")</f>
+        <v/>
+      </c>
+      <c r="P17" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C17:M17="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="22" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>Alen</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="33" t="n"/>
+      <c r="F20" s="33" t="n"/>
+      <c r="G20" s="33" t="n"/>
+      <c r="H20" s="33" t="n"/>
+      <c r="I20" s="33" t="n"/>
+      <c r="J20" s="33" t="n"/>
+      <c r="K20" s="33" t="n"/>
+      <c r="L20" s="33" t="n"/>
+      <c r="M20" s="33" t="n"/>
+      <c r="N20" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C20:M20,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="28">
+        <f>COUNTIF(C20:M20,"Y")</f>
+        <v/>
+      </c>
+      <c r="P20" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C20:M20="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>Ash</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="n"/>
+      <c r="H21" s="19" t="n"/>
+      <c r="I21" s="19" t="n"/>
+      <c r="J21" s="19" t="n"/>
+      <c r="K21" s="19" t="n"/>
+      <c r="L21" s="19" t="n"/>
+      <c r="M21" s="19" t="n"/>
+      <c r="N21" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C21:M21,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O21" s="28">
+        <f>COUNTIF(C21:M21,"Y")</f>
+        <v/>
+      </c>
+      <c r="P21" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C21:M21="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>Autumn</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="33" t="n"/>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F22" s="33" t="n"/>
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="33" t="n"/>
+      <c r="I22" s="33" t="n"/>
+      <c r="J22" s="33" t="n"/>
+      <c r="K22" s="33" t="n"/>
+      <c r="L22" s="33" t="n"/>
+      <c r="M22" s="33" t="n"/>
+      <c r="N22" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C22:M22,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="28">
+        <f>COUNTIF(C22:M22,"Y")</f>
+        <v/>
+      </c>
+      <c r="P22" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C22:M22="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="35" t="inlineStr">
+        <is>
+          <t>Bri</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="n"/>
+      <c r="H23" s="19" t="n"/>
+      <c r="I23" s="19" t="n"/>
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="19" t="n"/>
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="19" t="n"/>
+      <c r="N23" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C23:M23,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="28">
+        <f>COUNTIF(C23:M23,"Y")</f>
+        <v/>
+      </c>
+      <c r="P23" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C23:M23="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>Dakayla</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="33" t="n"/>
+      <c r="E24" s="33" t="n"/>
+      <c r="F24" s="33" t="n"/>
+      <c r="G24" s="33" t="n"/>
+      <c r="H24" s="33" t="n"/>
+      <c r="I24" s="33" t="n"/>
+      <c r="J24" s="33" t="n"/>
+      <c r="K24" s="33" t="n"/>
+      <c r="L24" s="33" t="n"/>
+      <c r="M24" s="33" t="n"/>
+      <c r="N24" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C24:M24,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="28">
+        <f>COUNTIF(C24:M24,"Y")</f>
+        <v/>
+      </c>
+      <c r="P24" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C24:M24="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="35" t="inlineStr">
+        <is>
+          <t>Divan</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="n"/>
+      <c r="H25" s="19" t="n"/>
+      <c r="I25" s="19" t="n"/>
+      <c r="J25" s="19" t="n"/>
+      <c r="K25" s="19" t="n"/>
+      <c r="L25" s="19" t="n"/>
+      <c r="M25" s="19" t="n"/>
+      <c r="N25" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C25:M25,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="28">
+        <f>COUNTIF(C25:M25,"Y")</f>
+        <v/>
+      </c>
+      <c r="P25" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C25:M25="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="33" t="n"/>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F26" s="33" t="n"/>
+      <c r="G26" s="33" t="n"/>
+      <c r="H26" s="33" t="n"/>
+      <c r="I26" s="33" t="n"/>
+      <c r="J26" s="33" t="n"/>
+      <c r="K26" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L26" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M26" s="33" t="n"/>
+      <c r="N26" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C26:M26,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="28">
+        <f>COUNTIF(C26:M26,"Y")</f>
+        <v/>
+      </c>
+      <c r="P26" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C26:M26="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="35" t="inlineStr">
+        <is>
+          <t>Grace</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="n"/>
+      <c r="H27" s="19" t="n"/>
+      <c r="I27" s="19" t="n"/>
+      <c r="J27" s="19" t="n"/>
+      <c r="K27" s="19" t="n"/>
+      <c r="L27" s="19" t="n"/>
+      <c r="M27" s="19" t="n"/>
+      <c r="N27" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C27:M27,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="28">
+        <f>COUNTIF(C27:M27,"Y")</f>
+        <v/>
+      </c>
+      <c r="P27" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C27:M27="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="31" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>Jada</t>
+        </is>
+      </c>
+      <c r="C28" s="33" t="n"/>
+      <c r="D28" s="33" t="n"/>
+      <c r="E28" s="33" t="n"/>
+      <c r="F28" s="33" t="n"/>
+      <c r="G28" s="33" t="n"/>
+      <c r="H28" s="33" t="n"/>
+      <c r="I28" s="33" t="n"/>
+      <c r="J28" s="33" t="n"/>
+      <c r="K28" s="33" t="n"/>
+      <c r="L28" s="33" t="n"/>
+      <c r="M28" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N28" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C28:M28,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O28" s="28">
+        <f>COUNTIF(C28:M28,"Y")</f>
+        <v/>
+      </c>
+      <c r="P28" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C28:M28="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>Jeremiah</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="n"/>
+      <c r="H29" s="19" t="n"/>
+      <c r="I29" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J29" s="19" t="n"/>
+      <c r="K29" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L29" s="19" t="n"/>
+      <c r="M29" s="19" t="n"/>
+      <c r="N29" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C29:M29,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O29" s="28">
+        <f>COUNTIF(C29:M29,"Y")</f>
+        <v/>
+      </c>
+      <c r="P29" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C29:M29="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="31" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="32" t="inlineStr">
+        <is>
+          <t>Kable</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="n"/>
+      <c r="D30" s="33" t="n"/>
+      <c r="E30" s="33" t="n"/>
+      <c r="F30" s="33" t="n"/>
+      <c r="G30" s="33" t="n"/>
+      <c r="H30" s="33" t="n"/>
+      <c r="I30" s="33" t="n"/>
+      <c r="J30" s="33" t="n"/>
+      <c r="K30" s="33" t="n"/>
+      <c r="L30" s="33" t="n"/>
+      <c r="M30" s="33" t="n"/>
+      <c r="N30" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C30:M30,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O30" s="28">
+        <f>COUNTIF(C30:M30,"Y")</f>
+        <v/>
+      </c>
+      <c r="P30" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C30:M30="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="17" customHeight="1">
+      <c r="A31" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>Kayla</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="n"/>
+      <c r="H31" s="19" t="n"/>
+      <c r="I31" s="19" t="n"/>
+      <c r="J31" s="19" t="n"/>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="19" t="n"/>
+      <c r="M31" s="19" t="n"/>
+      <c r="N31" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C31:M31,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O31" s="28">
+        <f>COUNTIF(C31:M31,"Y")</f>
+        <v/>
+      </c>
+      <c r="P31" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C31:M31="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="17" customHeight="1">
+      <c r="A32" s="31" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>Kenzie</t>
+        </is>
+      </c>
+      <c r="C32" s="33" t="n"/>
+      <c r="D32" s="33" t="n"/>
+      <c r="E32" s="33" t="n"/>
+      <c r="F32" s="33" t="n"/>
+      <c r="G32" s="33" t="n"/>
+      <c r="H32" s="33" t="n"/>
+      <c r="I32" s="33" t="n"/>
+      <c r="J32" s="33" t="n"/>
+      <c r="K32" s="33" t="n"/>
+      <c r="L32" s="33" t="n"/>
+      <c r="M32" s="33" t="n"/>
+      <c r="N32" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C32:M32,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O32" s="28">
+        <f>COUNTIF(C32:M32,"Y")</f>
+        <v/>
+      </c>
+      <c r="P32" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C32:M32="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="17" customHeight="1">
+      <c r="A33" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="35" t="inlineStr">
+        <is>
+          <t>Lidy</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G33" s="19" t="n"/>
+      <c r="H33" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="n"/>
+      <c r="J33" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K33" s="19" t="n"/>
+      <c r="L33" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M33" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N33" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C33:M33,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O33" s="28">
+        <f>COUNTIF(C33:M33,"Y")</f>
+        <v/>
+      </c>
+      <c r="P33" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C33:M33="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="17" customHeight="1">
+      <c r="A34" s="31" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>Maylin</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E34" s="33" t="n"/>
+      <c r="F34" s="33" t="n"/>
+      <c r="G34" s="33" t="n"/>
+      <c r="H34" s="33" t="n"/>
+      <c r="I34" s="33" t="n"/>
+      <c r="J34" s="33" t="n"/>
+      <c r="K34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L34" s="33" t="n"/>
+      <c r="M34" s="33" t="n"/>
+      <c r="N34" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C34:M34,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O34" s="28">
+        <f>COUNTIF(C34:M34,"Y")</f>
+        <v/>
+      </c>
+      <c r="P34" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C34:M34="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="34" t="n">
+        <v>16</v>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="19" t="n"/>
+      <c r="H35" s="19" t="n"/>
+      <c r="I35" s="19" t="n"/>
+      <c r="J35" s="19" t="n"/>
+      <c r="K35" s="19" t="n"/>
+      <c r="L35" s="19" t="n"/>
+      <c r="M35" s="19" t="n"/>
+      <c r="N35" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C35:M35,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O35" s="28">
+        <f>COUNTIF(C35:M35,"Y")</f>
+        <v/>
+      </c>
+      <c r="P35" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C35:M35="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="31" t="n">
+        <v>17</v>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C36" s="33" t="n"/>
+      <c r="D36" s="33" t="n"/>
+      <c r="E36" s="33" t="n"/>
+      <c r="F36" s="33" t="n"/>
+      <c r="G36" s="33" t="n"/>
+      <c r="H36" s="33" t="n"/>
+      <c r="I36" s="33" t="n"/>
+      <c r="J36" s="33" t="n"/>
+      <c r="K36" s="33" t="n"/>
+      <c r="L36" s="33" t="n"/>
+      <c r="M36" s="33" t="n"/>
+      <c r="N36" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C36:M36,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O36" s="28">
+        <f>COUNTIF(C36:M36,"Y")</f>
+        <v/>
+      </c>
+      <c r="P36" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C36:M36="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="n"/>
+      <c r="E37" s="19" t="n"/>
+      <c r="F37" s="19" t="n"/>
+      <c r="G37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H37" s="19" t="n"/>
+      <c r="I37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J37" s="19" t="n"/>
+      <c r="K37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L37" s="19" t="n"/>
+      <c r="M37" s="19" t="n"/>
+      <c r="N37" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C37:M37,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O37" s="28">
+        <f>COUNTIF(C37:M37,"Y")</f>
+        <v/>
+      </c>
+      <c r="P37" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C37:M37="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="31" t="n">
+        <v>19</v>
+      </c>
+      <c r="B38" s="32" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="C38" s="33" t="n"/>
+      <c r="D38" s="33" t="n"/>
+      <c r="E38" s="33" t="n"/>
+      <c r="F38" s="33" t="n"/>
+      <c r="G38" s="33" t="n"/>
+      <c r="H38" s="33" t="n"/>
+      <c r="I38" s="33" t="n"/>
+      <c r="J38" s="33" t="n"/>
+      <c r="K38" s="33" t="n"/>
+      <c r="L38" s="33" t="n"/>
+      <c r="M38" s="33" t="n"/>
+      <c r="N38" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C38:M38,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O38" s="28">
+        <f>COUNTIF(C38:M38,"Y")</f>
+        <v/>
+      </c>
+      <c r="P38" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C38:M38="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="3" t="inlineStr"/>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>Total on shift</t>
+        </is>
+      </c>
+      <c r="C39" s="6">
+        <f>COUNTIF(C14:C38,"Y")</f>
+        <v/>
+      </c>
+      <c r="D39" s="6">
+        <f>COUNTIF(D14:D38,"Y")</f>
+        <v/>
+      </c>
+      <c r="E39" s="6">
+        <f>COUNTIF(E14:E38,"Y")</f>
+        <v/>
+      </c>
+      <c r="F39" s="6">
+        <f>COUNTIF(F14:F38,"Y")</f>
+        <v/>
+      </c>
+      <c r="G39" s="6">
+        <f>COUNTIF(G14:G38,"Y")</f>
+        <v/>
+      </c>
+      <c r="H39" s="6">
+        <f>COUNTIF(H14:H38,"Y")</f>
+        <v/>
+      </c>
+      <c r="I39" s="6">
+        <f>COUNTIF(I14:I38,"Y")</f>
+        <v/>
+      </c>
+      <c r="J39" s="6">
+        <f>COUNTIF(J14:J38,"Y")</f>
+        <v/>
+      </c>
+      <c r="K39" s="6">
+        <f>COUNTIF(K14:K38,"Y")</f>
+        <v/>
+      </c>
+      <c r="L39" s="6">
+        <f>COUNTIF(L14:L38,"Y")</f>
+        <v/>
+      </c>
+      <c r="M39" s="6">
+        <f>COUNTIF(M14:M38,"Y")</f>
+        <v/>
+      </c>
+      <c r="N39" s="3" t="inlineStr"/>
+      <c r="O39" s="6">
+        <f>SUM(O14:O38)</f>
+        <v/>
+      </c>
+      <c r="P39" s="37">
+        <f>SUM(P14:P38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="12" customHeight="1">
+      <c r="A40" s="38" t="inlineStr">
+        <is>
+          <t>Y = on shift during shop's meal window. Personal Avg = average score of shops worked. Bonus = $50 per 100% shop worked.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A13:P13"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A40:P40"/>
+    <mergeCell ref="A18:P18"/>
+    <mergeCell ref="A12:P12"/>
+    <mergeCell ref="A19:P19"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
shop tracker: correct June 4 100% shop (job 20808696) on-shift list
CT timecard verification (window 11:00a-1:30p) shows exactly 5 on shift:
Bri (Brianna Gatewood), Kaisha (Kaisha Brewer), Lidy (Lidy Henry),
Vicki (Vicki Lucey), Zack (Zack Whitten).

Removes: Bobby, DaKayla, Nathan, Kasey, Jada (not clocked in during window).
Also adds Kaisha to CREW roster in build_shop_tracker.py so her Y marks render.
Regenerated Shop_Tracker_2065_2026.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -773,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W40"/>
+  <dimension ref="A1:W41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="B30" s="32" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="C30" s="33" t="n"/>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="C32" s="33" t="n"/>
@@ -2177,71 +2177,27 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Lidy</t>
-        </is>
-      </c>
-      <c r="C33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="D33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Kenzie</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="19" t="n"/>
       <c r="H33" s="19" t="n"/>
-      <c r="I33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="I33" s="19" t="n"/>
+      <c r="J33" s="19" t="n"/>
+      <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
       <c r="M33" s="19" t="n"/>
       <c r="N33" s="19" t="n"/>
-      <c r="O33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="O33" s="19" t="n"/>
       <c r="P33" s="19" t="n"/>
-      <c r="Q33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="Q33" s="19" t="n"/>
       <c r="R33" s="19" t="n"/>
       <c r="S33" s="19" t="n"/>
-      <c r="T33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="T33" s="19" t="n"/>
       <c r="U33" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$T$7,C33:T33,"Y"),"")</f>
         <v/>
@@ -2261,25 +2217,45 @@
       </c>
       <c r="B34" s="32" t="inlineStr">
         <is>
-          <t>Maylin</t>
-        </is>
-      </c>
-      <c r="C34" s="33" t="n"/>
+          <t>Lidy</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="E34" s="33" t="n"/>
-      <c r="F34" s="33" t="n"/>
-      <c r="G34" s="33" t="n"/>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H34" s="33" t="n"/>
       <c r="I34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J34" s="33" t="n"/>
+      <c r="J34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2287,29 +2263,25 @@
       </c>
       <c r="L34" s="33" t="n"/>
       <c r="M34" s="33" t="n"/>
-      <c r="N34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O34" s="33" t="n"/>
-      <c r="P34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="N34" s="33" t="n"/>
+      <c r="O34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P34" s="33" t="n"/>
       <c r="Q34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="R34" s="33" t="n"/>
-      <c r="S34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="T34" s="33" t="n"/>
+      <c r="S34" s="33" t="n"/>
+      <c r="T34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="U34" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$T$7,C34:T34,"Y"),"")</f>
         <v/>
@@ -2329,47 +2301,55 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E35" s="19" t="n"/>
       <c r="F35" s="19" t="n"/>
       <c r="G35" s="19" t="n"/>
       <c r="H35" s="19" t="n"/>
-      <c r="I35" s="19" t="n"/>
+      <c r="I35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J35" s="19" t="n"/>
-      <c r="K35" s="19" t="n"/>
+      <c r="K35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L35" s="19" t="n"/>
-      <c r="M35" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N35" s="19" t="n"/>
-      <c r="O35" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M35" s="19" t="n"/>
+      <c r="N35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O35" s="19" t="n"/>
       <c r="P35" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="Q35" s="19" t="n"/>
+      <c r="Q35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="R35" s="19" t="n"/>
       <c r="S35" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="T35" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="T35" s="19" t="n"/>
       <c r="U35" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$T$7,C35:T35,"Y"),"")</f>
         <v/>
@@ -2389,7 +2369,7 @@
       </c>
       <c r="B36" s="32" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C36" s="33" t="n"/>
@@ -2402,14 +2382,34 @@
       <c r="J36" s="33" t="n"/>
       <c r="K36" s="33" t="n"/>
       <c r="L36" s="33" t="n"/>
-      <c r="M36" s="33" t="n"/>
+      <c r="M36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="N36" s="33" t="n"/>
-      <c r="O36" s="33" t="n"/>
-      <c r="P36" s="33" t="n"/>
+      <c r="O36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="Q36" s="33" t="n"/>
       <c r="R36" s="33" t="n"/>
-      <c r="S36" s="33" t="n"/>
-      <c r="T36" s="33" t="n"/>
+      <c r="S36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="U36" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$T$7,C36:T36,"Y"),"")</f>
         <v/>
@@ -2429,58 +2429,26 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Samuel</t>
-        </is>
-      </c>
-      <c r="C37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="n"/>
       <c r="D37" s="19" t="n"/>
       <c r="E37" s="19" t="n"/>
       <c r="F37" s="19" t="n"/>
-      <c r="G37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G37" s="19" t="n"/>
       <c r="H37" s="19" t="n"/>
       <c r="I37" s="19" t="n"/>
-      <c r="J37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J37" s="19" t="n"/>
       <c r="K37" s="19" t="n"/>
-      <c r="L37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L37" s="19" t="n"/>
       <c r="M37" s="19" t="n"/>
-      <c r="N37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="N37" s="19" t="n"/>
       <c r="O37" s="19" t="n"/>
-      <c r="P37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="P37" s="19" t="n"/>
       <c r="Q37" s="19" t="n"/>
-      <c r="R37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="S37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
       <c r="T37" s="19" t="n"/>
       <c r="U37" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$T$7,C37:T37,"Y"),"")</f>
@@ -2501,26 +2469,58 @@
       </c>
       <c r="B38" s="32" t="inlineStr">
         <is>
-          <t>Zach</t>
-        </is>
-      </c>
-      <c r="C38" s="33" t="n"/>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D38" s="33" t="n"/>
       <c r="E38" s="33" t="n"/>
       <c r="F38" s="33" t="n"/>
-      <c r="G38" s="33" t="n"/>
+      <c r="G38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H38" s="33" t="n"/>
       <c r="I38" s="33" t="n"/>
-      <c r="J38" s="33" t="n"/>
+      <c r="J38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K38" s="33" t="n"/>
-      <c r="L38" s="33" t="n"/>
+      <c r="L38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M38" s="33" t="n"/>
-      <c r="N38" s="33" t="n"/>
+      <c r="N38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="O38" s="33" t="n"/>
-      <c r="P38" s="33" t="n"/>
+      <c r="P38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="Q38" s="33" t="n"/>
-      <c r="R38" s="33" t="n"/>
-      <c r="S38" s="33" t="n"/>
+      <c r="R38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="T38" s="33" t="n"/>
       <c r="U38" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$T$7,C38:T38,"Y"),"")</f>
@@ -2535,97 +2535,137 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr"/>
-      <c r="B39" s="36" t="inlineStr">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="19" t="n"/>
+      <c r="P39" s="19" t="n"/>
+      <c r="Q39" s="19" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
+      <c r="T39" s="19" t="n"/>
+      <c r="U39" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$T$7,C39:T39,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="V39" s="28">
+        <f>COUNTIF(C39:T39,"Y")</f>
+        <v/>
+      </c>
+      <c r="W39" s="29">
+        <f>SUMPRODUCT((C$7:$T$7=1)*(C39:T39="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>Total on shift</t>
         </is>
       </c>
-      <c r="C39" s="6">
-        <f>COUNTIF(C14:C38,"Y")</f>
-        <v/>
-      </c>
-      <c r="D39" s="6">
-        <f>COUNTIF(D14:D38,"Y")</f>
-        <v/>
-      </c>
-      <c r="E39" s="6">
-        <f>COUNTIF(E14:E38,"Y")</f>
-        <v/>
-      </c>
-      <c r="F39" s="6">
-        <f>COUNTIF(F14:F38,"Y")</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>COUNTIF(G14:G38,"Y")</f>
-        <v/>
-      </c>
-      <c r="H39" s="6">
-        <f>COUNTIF(H14:H38,"Y")</f>
-        <v/>
-      </c>
-      <c r="I39" s="6">
-        <f>COUNTIF(I14:I38,"Y")</f>
-        <v/>
-      </c>
-      <c r="J39" s="6">
-        <f>COUNTIF(J14:J38,"Y")</f>
-        <v/>
-      </c>
-      <c r="K39" s="6">
-        <f>COUNTIF(K14:K38,"Y")</f>
-        <v/>
-      </c>
-      <c r="L39" s="6">
-        <f>COUNTIF(L14:L38,"Y")</f>
-        <v/>
-      </c>
-      <c r="M39" s="6">
-        <f>COUNTIF(M14:M38,"Y")</f>
-        <v/>
-      </c>
-      <c r="N39" s="6">
-        <f>COUNTIF(N14:N38,"Y")</f>
-        <v/>
-      </c>
-      <c r="O39" s="6">
-        <f>COUNTIF(O14:O38,"Y")</f>
-        <v/>
-      </c>
-      <c r="P39" s="6">
-        <f>COUNTIF(P14:P38,"Y")</f>
-        <v/>
-      </c>
-      <c r="Q39" s="6">
-        <f>COUNTIF(Q14:Q38,"Y")</f>
-        <v/>
-      </c>
-      <c r="R39" s="6">
-        <f>COUNTIF(R14:R38,"Y")</f>
-        <v/>
-      </c>
-      <c r="S39" s="6">
-        <f>COUNTIF(S14:S38,"Y")</f>
-        <v/>
-      </c>
-      <c r="T39" s="6">
-        <f>COUNTIF(T14:T38,"Y")</f>
-        <v/>
-      </c>
-      <c r="U39" s="3" t="inlineStr"/>
-      <c r="V39" s="6">
-        <f>SUM(V14:V38)</f>
-        <v/>
-      </c>
-      <c r="W39" s="37">
-        <f>SUM(W14:W38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="12" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
+      <c r="C40" s="6">
+        <f>COUNTIF(C14:C39,"Y")</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>COUNTIF(D14:D39,"Y")</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>COUNTIF(E14:E39,"Y")</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>COUNTIF(F14:F39,"Y")</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>COUNTIF(G14:G39,"Y")</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>COUNTIF(H14:H39,"Y")</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>COUNTIF(I14:I39,"Y")</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>COUNTIF(J14:J39,"Y")</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>COUNTIF(K14:K39,"Y")</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>COUNTIF(L14:L39,"Y")</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>COUNTIF(M14:M39,"Y")</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>COUNTIF(N14:N39,"Y")</f>
+        <v/>
+      </c>
+      <c r="O40" s="6">
+        <f>COUNTIF(O14:O39,"Y")</f>
+        <v/>
+      </c>
+      <c r="P40" s="6">
+        <f>COUNTIF(P14:P39,"Y")</f>
+        <v/>
+      </c>
+      <c r="Q40" s="6">
+        <f>COUNTIF(Q14:Q39,"Y")</f>
+        <v/>
+      </c>
+      <c r="R40" s="6">
+        <f>COUNTIF(R14:R39,"Y")</f>
+        <v/>
+      </c>
+      <c r="S40" s="6">
+        <f>COUNTIF(S14:S39,"Y")</f>
+        <v/>
+      </c>
+      <c r="T40" s="6">
+        <f>COUNTIF(T14:T39,"Y")</f>
+        <v/>
+      </c>
+      <c r="U40" s="3" t="inlineStr"/>
+      <c r="V40" s="6">
+        <f>SUM(V14:V39)</f>
+        <v/>
+      </c>
+      <c r="W40" s="37">
+        <f>SUM(W14:W39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>Y = on shift during shop's meal window. Personal Avg = average score of shops worked. Bonus = $50 per 100% shop worked.</t>
         </is>
@@ -2635,9 +2675,9 @@
   <mergeCells count="7">
     <mergeCell ref="A13:W13"/>
     <mergeCell ref="A1:W1"/>
-    <mergeCell ref="A40:W40"/>
     <mergeCell ref="A18:W18"/>
     <mergeCell ref="A12:W12"/>
+    <mergeCell ref="A41:W41"/>
     <mergeCell ref="A2:W2"/>
     <mergeCell ref="A19:W19"/>
   </mergeCells>
@@ -2653,7 +2693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3715,7 +3755,7 @@
       </c>
       <c r="B30" s="32" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="C30" s="33" t="n"/>
@@ -3749,7 +3789,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
@@ -3783,7 +3823,7 @@
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="C32" s="33" t="n"/>
@@ -3817,36 +3857,20 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="C33" s="19" t="n"/>
-      <c r="D33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D33" s="19" t="n"/>
       <c r="E33" s="19" t="n"/>
       <c r="F33" s="19" t="n"/>
       <c r="G33" s="19" t="n"/>
       <c r="H33" s="19" t="n"/>
-      <c r="I33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="I33" s="19" t="n"/>
       <c r="J33" s="19" t="n"/>
-      <c r="K33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
-      <c r="M33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M33" s="19" t="n"/>
       <c r="N33" s="19" t="n"/>
       <c r="O33" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$N$7,C33:N33,"Y"),"")</f>
@@ -3867,39 +3891,31 @@
       </c>
       <c r="B34" s="32" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="C34" s="33" t="n"/>
-      <c r="D34" s="33" t="n"/>
-      <c r="E34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E34" s="33" t="n"/>
+      <c r="F34" s="33" t="n"/>
       <c r="G34" s="33" t="n"/>
       <c r="H34" s="33" t="n"/>
-      <c r="I34" s="33" t="n"/>
-      <c r="J34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="I34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J34" s="33" t="n"/>
       <c r="K34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L34" s="33" t="n"/>
       <c r="M34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3925,37 +3941,45 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
       <c r="D35" s="19" t="n"/>
-      <c r="E35" s="19" t="n"/>
-      <c r="F35" s="19" t="n"/>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G35" s="19" t="n"/>
       <c r="H35" s="19" t="n"/>
-      <c r="I35" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J35" s="19" t="n"/>
+      <c r="I35" s="19" t="n"/>
+      <c r="J35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K35" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L35" s="19" t="n"/>
+      <c r="L35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M35" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N35" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="N35" s="19" t="n"/>
       <c r="O35" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$N$7,C35:N35,"Y"),"")</f>
         <v/>
@@ -3975,7 +3999,7 @@
       </c>
       <c r="B36" s="32" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C36" s="33" t="n"/>
@@ -3984,12 +4008,28 @@
       <c r="F36" s="33" t="n"/>
       <c r="G36" s="33" t="n"/>
       <c r="H36" s="33" t="n"/>
-      <c r="I36" s="33" t="n"/>
+      <c r="I36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J36" s="33" t="n"/>
-      <c r="K36" s="33" t="n"/>
+      <c r="K36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L36" s="33" t="n"/>
-      <c r="M36" s="33" t="n"/>
-      <c r="N36" s="33" t="n"/>
+      <c r="M36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N36" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="O36" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$N$7,C36:N36,"Y"),"")</f>
         <v/>
@@ -4009,39 +4049,19 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="C37" s="19" t="n"/>
       <c r="D37" s="19" t="n"/>
-      <c r="E37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E37" s="19" t="n"/>
       <c r="F37" s="19" t="n"/>
-      <c r="G37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G37" s="19" t="n"/>
+      <c r="H37" s="19" t="n"/>
       <c r="I37" s="19" t="n"/>
-      <c r="J37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J37" s="19" t="n"/>
       <c r="K37" s="19" t="n"/>
-      <c r="L37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L37" s="19" t="n"/>
       <c r="M37" s="19" t="n"/>
       <c r="N37" s="19" t="n"/>
       <c r="O37" s="18">
@@ -4063,19 +4083,39 @@
       </c>
       <c r="B38" s="32" t="inlineStr">
         <is>
-          <t>Zach</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="C38" s="33" t="n"/>
       <c r="D38" s="33" t="n"/>
-      <c r="E38" s="33" t="n"/>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F38" s="33" t="n"/>
-      <c r="G38" s="33" t="n"/>
-      <c r="H38" s="33" t="n"/>
+      <c r="G38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I38" s="33" t="n"/>
-      <c r="J38" s="33" t="n"/>
+      <c r="J38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K38" s="33" t="n"/>
-      <c r="L38" s="33" t="n"/>
+      <c r="L38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M38" s="33" t="n"/>
       <c r="N38" s="33" t="n"/>
       <c r="O38" s="18">
@@ -4091,73 +4131,107 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr"/>
-      <c r="B39" s="36" t="inlineStr">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$N$7,C39:N39,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P39" s="28">
+        <f>COUNTIF(C39:N39,"Y")</f>
+        <v/>
+      </c>
+      <c r="Q39" s="29">
+        <f>SUMPRODUCT((C$7:$N$7=1)*(C39:N39="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>Total on shift</t>
         </is>
       </c>
-      <c r="C39" s="6">
-        <f>COUNTIF(C14:C38,"Y")</f>
-        <v/>
-      </c>
-      <c r="D39" s="6">
-        <f>COUNTIF(D14:D38,"Y")</f>
-        <v/>
-      </c>
-      <c r="E39" s="6">
-        <f>COUNTIF(E14:E38,"Y")</f>
-        <v/>
-      </c>
-      <c r="F39" s="6">
-        <f>COUNTIF(F14:F38,"Y")</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>COUNTIF(G14:G38,"Y")</f>
-        <v/>
-      </c>
-      <c r="H39" s="6">
-        <f>COUNTIF(H14:H38,"Y")</f>
-        <v/>
-      </c>
-      <c r="I39" s="6">
-        <f>COUNTIF(I14:I38,"Y")</f>
-        <v/>
-      </c>
-      <c r="J39" s="6">
-        <f>COUNTIF(J14:J38,"Y")</f>
-        <v/>
-      </c>
-      <c r="K39" s="6">
-        <f>COUNTIF(K14:K38,"Y")</f>
-        <v/>
-      </c>
-      <c r="L39" s="6">
-        <f>COUNTIF(L14:L38,"Y")</f>
-        <v/>
-      </c>
-      <c r="M39" s="6">
-        <f>COUNTIF(M14:M38,"Y")</f>
-        <v/>
-      </c>
-      <c r="N39" s="6">
-        <f>COUNTIF(N14:N38,"Y")</f>
-        <v/>
-      </c>
-      <c r="O39" s="3" t="inlineStr"/>
-      <c r="P39" s="6">
-        <f>SUM(P14:P38)</f>
-        <v/>
-      </c>
-      <c r="Q39" s="37">
-        <f>SUM(Q14:Q38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="12" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
+      <c r="C40" s="6">
+        <f>COUNTIF(C14:C39,"Y")</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>COUNTIF(D14:D39,"Y")</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>COUNTIF(E14:E39,"Y")</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>COUNTIF(F14:F39,"Y")</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>COUNTIF(G14:G39,"Y")</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>COUNTIF(H14:H39,"Y")</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>COUNTIF(I14:I39,"Y")</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>COUNTIF(J14:J39,"Y")</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>COUNTIF(K14:K39,"Y")</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>COUNTIF(L14:L39,"Y")</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>COUNTIF(M14:M39,"Y")</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>COUNTIF(N14:N39,"Y")</f>
+        <v/>
+      </c>
+      <c r="O40" s="3" t="inlineStr"/>
+      <c r="P40" s="6">
+        <f>SUM(P14:P39)</f>
+        <v/>
+      </c>
+      <c r="Q40" s="37">
+        <f>SUM(Q14:Q39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>Y = on shift during shop's meal window. Personal Avg = average score of shops worked. Bonus = $50 per 100% shop worked.</t>
         </is>
@@ -4165,10 +4239,10 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A40:Q40"/>
     <mergeCell ref="A18:Q18"/>
     <mergeCell ref="A12:Q12"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A41:Q41"/>
     <mergeCell ref="A19:Q19"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A13:Q13"/>
@@ -4185,7 +4259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5349,7 +5423,7 @@
       </c>
       <c r="B30" s="32" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="C30" s="33" t="n"/>
@@ -5385,7 +5459,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
@@ -5421,7 +5495,7 @@
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="C32" s="33" t="n"/>
@@ -5457,43 +5531,23 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="C33" s="19" t="n"/>
       <c r="D33" s="19" t="n"/>
-      <c r="E33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
       <c r="G33" s="19" t="n"/>
       <c r="H33" s="19" t="n"/>
       <c r="I33" s="19" t="n"/>
-      <c r="J33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J33" s="19" t="n"/>
       <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
-      <c r="M33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M33" s="19" t="n"/>
       <c r="N33" s="19" t="n"/>
       <c r="O33" s="19" t="n"/>
-      <c r="P33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="P33" s="19" t="n"/>
       <c r="Q33" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$P$7,C33:P33,"Y"),"")</f>
         <v/>
@@ -5513,12 +5567,16 @@
       </c>
       <c r="B34" s="32" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="C34" s="33" t="n"/>
       <c r="D34" s="33" t="n"/>
-      <c r="E34" s="33" t="n"/>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5533,26 +5591,14 @@
         </is>
       </c>
       <c r="K34" s="33" t="n"/>
-      <c r="L34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L34" s="33" t="n"/>
       <c r="M34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="N34" s="33" t="n"/>
+      <c r="O34" s="33" t="n"/>
       <c r="P34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5577,23 +5623,51 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
       <c r="D35" s="19" t="n"/>
       <c r="E35" s="19" t="n"/>
-      <c r="F35" s="19" t="n"/>
+      <c r="F35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G35" s="19" t="n"/>
       <c r="H35" s="19" t="n"/>
       <c r="I35" s="19" t="n"/>
-      <c r="J35" s="19" t="n"/>
+      <c r="J35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K35" s="19" t="n"/>
-      <c r="L35" s="19" t="n"/>
-      <c r="M35" s="19" t="n"/>
-      <c r="N35" s="19" t="n"/>
-      <c r="O35" s="19" t="n"/>
-      <c r="P35" s="19" t="n"/>
+      <c r="L35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="Q35" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$P$7,C35:P35,"Y"),"")</f>
         <v/>
@@ -5613,7 +5687,7 @@
       </c>
       <c r="B36" s="32" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C36" s="33" t="n"/>
@@ -5649,31 +5723,19 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="C37" s="19" t="n"/>
-      <c r="D37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D37" s="19" t="n"/>
       <c r="E37" s="19" t="n"/>
       <c r="F37" s="19" t="n"/>
       <c r="G37" s="19" t="n"/>
-      <c r="H37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="H37" s="19" t="n"/>
       <c r="I37" s="19" t="n"/>
       <c r="J37" s="19" t="n"/>
       <c r="K37" s="19" t="n"/>
-      <c r="L37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L37" s="19" t="n"/>
       <c r="M37" s="19" t="n"/>
       <c r="N37" s="19" t="n"/>
       <c r="O37" s="19" t="n"/>
@@ -5697,19 +5759,31 @@
       </c>
       <c r="B38" s="32" t="inlineStr">
         <is>
-          <t>Zach</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="C38" s="33" t="n"/>
-      <c r="D38" s="33" t="n"/>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E38" s="33" t="n"/>
       <c r="F38" s="33" t="n"/>
       <c r="G38" s="33" t="n"/>
-      <c r="H38" s="33" t="n"/>
+      <c r="H38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I38" s="33" t="n"/>
       <c r="J38" s="33" t="n"/>
       <c r="K38" s="33" t="n"/>
-      <c r="L38" s="33" t="n"/>
+      <c r="L38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M38" s="33" t="n"/>
       <c r="N38" s="33" t="n"/>
       <c r="O38" s="33" t="n"/>
@@ -5727,81 +5801,117 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr"/>
-      <c r="B39" s="36" t="inlineStr">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="19" t="n"/>
+      <c r="P39" s="19" t="n"/>
+      <c r="Q39" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$P$7,C39:P39,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R39" s="28">
+        <f>COUNTIF(C39:P39,"Y")</f>
+        <v/>
+      </c>
+      <c r="S39" s="29">
+        <f>SUMPRODUCT((C$7:$P$7=1)*(C39:P39="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>Total on shift</t>
         </is>
       </c>
-      <c r="C39" s="6">
-        <f>COUNTIF(C14:C38,"Y")</f>
-        <v/>
-      </c>
-      <c r="D39" s="6">
-        <f>COUNTIF(D14:D38,"Y")</f>
-        <v/>
-      </c>
-      <c r="E39" s="6">
-        <f>COUNTIF(E14:E38,"Y")</f>
-        <v/>
-      </c>
-      <c r="F39" s="6">
-        <f>COUNTIF(F14:F38,"Y")</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>COUNTIF(G14:G38,"Y")</f>
-        <v/>
-      </c>
-      <c r="H39" s="6">
-        <f>COUNTIF(H14:H38,"Y")</f>
-        <v/>
-      </c>
-      <c r="I39" s="6">
-        <f>COUNTIF(I14:I38,"Y")</f>
-        <v/>
-      </c>
-      <c r="J39" s="6">
-        <f>COUNTIF(J14:J38,"Y")</f>
-        <v/>
-      </c>
-      <c r="K39" s="6">
-        <f>COUNTIF(K14:K38,"Y")</f>
-        <v/>
-      </c>
-      <c r="L39" s="6">
-        <f>COUNTIF(L14:L38,"Y")</f>
-        <v/>
-      </c>
-      <c r="M39" s="6">
-        <f>COUNTIF(M14:M38,"Y")</f>
-        <v/>
-      </c>
-      <c r="N39" s="6">
-        <f>COUNTIF(N14:N38,"Y")</f>
-        <v/>
-      </c>
-      <c r="O39" s="6">
-        <f>COUNTIF(O14:O38,"Y")</f>
-        <v/>
-      </c>
-      <c r="P39" s="6">
-        <f>COUNTIF(P14:P38,"Y")</f>
-        <v/>
-      </c>
-      <c r="Q39" s="3" t="inlineStr"/>
-      <c r="R39" s="6">
-        <f>SUM(R14:R38)</f>
-        <v/>
-      </c>
-      <c r="S39" s="37">
-        <f>SUM(S14:S38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="12" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
+      <c r="C40" s="6">
+        <f>COUNTIF(C14:C39,"Y")</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>COUNTIF(D14:D39,"Y")</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>COUNTIF(E14:E39,"Y")</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>COUNTIF(F14:F39,"Y")</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>COUNTIF(G14:G39,"Y")</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>COUNTIF(H14:H39,"Y")</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>COUNTIF(I14:I39,"Y")</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>COUNTIF(J14:J39,"Y")</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>COUNTIF(K14:K39,"Y")</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>COUNTIF(L14:L39,"Y")</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>COUNTIF(M14:M39,"Y")</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>COUNTIF(N14:N39,"Y")</f>
+        <v/>
+      </c>
+      <c r="O40" s="6">
+        <f>COUNTIF(O14:O39,"Y")</f>
+        <v/>
+      </c>
+      <c r="P40" s="6">
+        <f>COUNTIF(P14:P39,"Y")</f>
+        <v/>
+      </c>
+      <c r="Q40" s="3" t="inlineStr"/>
+      <c r="R40" s="6">
+        <f>SUM(R14:R39)</f>
+        <v/>
+      </c>
+      <c r="S40" s="37">
+        <f>SUM(S14:S39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>Y = on shift during shop's meal window. Personal Avg = average score of shops worked. Bonus = $50 per 100% shop worked.</t>
         </is>
@@ -5809,10 +5919,10 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A41:S41"/>
     <mergeCell ref="A19:S19"/>
     <mergeCell ref="A13:S13"/>
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="A40:S40"/>
     <mergeCell ref="A18:S18"/>
     <mergeCell ref="A12:S12"/>
     <mergeCell ref="A2:S2"/>
@@ -5829,7 +5939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6960,7 +7070,7 @@
       </c>
       <c r="B30" s="32" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="C30" s="33" t="n"/>
@@ -6995,7 +7105,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
@@ -7030,7 +7140,7 @@
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="C32" s="33" t="n"/>
@@ -7065,46 +7175,22 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Lidy</t>
-        </is>
-      </c>
-      <c r="C33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Kenzie</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="n"/>
       <c r="D33" s="19" t="n"/>
       <c r="E33" s="19" t="n"/>
-      <c r="F33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F33" s="19" t="n"/>
       <c r="G33" s="19" t="n"/>
       <c r="H33" s="19" t="n"/>
-      <c r="I33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="I33" s="19" t="n"/>
       <c r="J33" s="19" t="n"/>
-      <c r="K33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
-      <c r="M33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M33" s="19" t="n"/>
       <c r="N33" s="19" t="n"/>
-      <c r="O33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="O33" s="19" t="n"/>
       <c r="P33" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$O$7,C33:O33,"Y"),"")</f>
         <v/>
@@ -7124,10 +7210,14 @@
       </c>
       <c r="B34" s="32" t="inlineStr">
         <is>
-          <t>Maylin</t>
-        </is>
-      </c>
-      <c r="C34" s="33" t="n"/>
+          <t>Lidy</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D34" s="33" t="n"/>
       <c r="E34" s="33" t="n"/>
       <c r="F34" s="26" t="inlineStr">
@@ -7142,20 +7232,24 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K34" s="33" t="n"/>
+      <c r="J34" s="33" t="n"/>
+      <c r="K34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L34" s="33" t="n"/>
-      <c r="M34" s="33" t="n"/>
-      <c r="N34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O34" s="33" t="n"/>
+      <c r="M34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N34" s="33" t="n"/>
+      <c r="O34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P34" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$O$7,C34:O34,"Y"),"")</f>
         <v/>
@@ -7175,21 +7269,37 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
       <c r="D35" s="19" t="n"/>
       <c r="E35" s="19" t="n"/>
-      <c r="F35" s="19" t="n"/>
+      <c r="F35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G35" s="19" t="n"/>
       <c r="H35" s="19" t="n"/>
-      <c r="I35" s="19" t="n"/>
-      <c r="J35" s="19" t="n"/>
+      <c r="I35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K35" s="19" t="n"/>
       <c r="L35" s="19" t="n"/>
       <c r="M35" s="19" t="n"/>
-      <c r="N35" s="19" t="n"/>
+      <c r="N35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="O35" s="19" t="n"/>
       <c r="P35" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$O$7,C35:O35,"Y"),"")</f>
@@ -7210,7 +7320,7 @@
       </c>
       <c r="B36" s="32" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C36" s="33" t="n"/>
@@ -7220,27 +7330,11 @@
       <c r="G36" s="33" t="n"/>
       <c r="H36" s="33" t="n"/>
       <c r="I36" s="33" t="n"/>
-      <c r="J36" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J36" s="33" t="n"/>
       <c r="K36" s="33" t="n"/>
-      <c r="L36" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M36" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N36" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L36" s="33" t="n"/>
+      <c r="M36" s="33" t="n"/>
+      <c r="N36" s="33" t="n"/>
       <c r="O36" s="33" t="n"/>
       <c r="P36" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$O$7,C36:O36,"Y"),"")</f>
@@ -7261,27 +7355,15 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="C37" s="19" t="n"/>
       <c r="D37" s="19" t="n"/>
-      <c r="E37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E37" s="19" t="n"/>
       <c r="F37" s="19" t="n"/>
-      <c r="G37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G37" s="19" t="n"/>
+      <c r="H37" s="19" t="n"/>
       <c r="I37" s="19" t="n"/>
       <c r="J37" s="26" t="inlineStr">
         <is>
@@ -7289,9 +7371,21 @@
         </is>
       </c>
       <c r="K37" s="19" t="n"/>
-      <c r="L37" s="19" t="n"/>
-      <c r="M37" s="19" t="n"/>
-      <c r="N37" s="19" t="n"/>
+      <c r="L37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="O37" s="19" t="n"/>
       <c r="P37" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$O$7,C37:O37,"Y"),"")</f>
@@ -7312,17 +7406,33 @@
       </c>
       <c r="B38" s="32" t="inlineStr">
         <is>
-          <t>Zach</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="C38" s="33" t="n"/>
       <c r="D38" s="33" t="n"/>
-      <c r="E38" s="33" t="n"/>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F38" s="33" t="n"/>
-      <c r="G38" s="33" t="n"/>
-      <c r="H38" s="33" t="n"/>
+      <c r="G38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I38" s="33" t="n"/>
-      <c r="J38" s="33" t="n"/>
+      <c r="J38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K38" s="33" t="n"/>
       <c r="L38" s="33" t="n"/>
       <c r="M38" s="33" t="n"/>
@@ -7341,77 +7451,112 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr"/>
-      <c r="B39" s="36" t="inlineStr">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="19" t="n"/>
+      <c r="P39" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$O$7,C39:O39,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="Q39" s="28">
+        <f>COUNTIF(C39:O39,"Y")</f>
+        <v/>
+      </c>
+      <c r="R39" s="29">
+        <f>SUMPRODUCT((C$7:$O$7=1)*(C39:O39="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>Total on shift</t>
         </is>
       </c>
-      <c r="C39" s="6">
-        <f>COUNTIF(C14:C38,"Y")</f>
-        <v/>
-      </c>
-      <c r="D39" s="6">
-        <f>COUNTIF(D14:D38,"Y")</f>
-        <v/>
-      </c>
-      <c r="E39" s="6">
-        <f>COUNTIF(E14:E38,"Y")</f>
-        <v/>
-      </c>
-      <c r="F39" s="6">
-        <f>COUNTIF(F14:F38,"Y")</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>COUNTIF(G14:G38,"Y")</f>
-        <v/>
-      </c>
-      <c r="H39" s="6">
-        <f>COUNTIF(H14:H38,"Y")</f>
-        <v/>
-      </c>
-      <c r="I39" s="6">
-        <f>COUNTIF(I14:I38,"Y")</f>
-        <v/>
-      </c>
-      <c r="J39" s="6">
-        <f>COUNTIF(J14:J38,"Y")</f>
-        <v/>
-      </c>
-      <c r="K39" s="6">
-        <f>COUNTIF(K14:K38,"Y")</f>
-        <v/>
-      </c>
-      <c r="L39" s="6">
-        <f>COUNTIF(L14:L38,"Y")</f>
-        <v/>
-      </c>
-      <c r="M39" s="6">
-        <f>COUNTIF(M14:M38,"Y")</f>
-        <v/>
-      </c>
-      <c r="N39" s="6">
-        <f>COUNTIF(N14:N38,"Y")</f>
-        <v/>
-      </c>
-      <c r="O39" s="6">
-        <f>COUNTIF(O14:O38,"Y")</f>
-        <v/>
-      </c>
-      <c r="P39" s="3" t="inlineStr"/>
-      <c r="Q39" s="6">
-        <f>SUM(Q14:Q38)</f>
-        <v/>
-      </c>
-      <c r="R39" s="37">
-        <f>SUM(R14:R38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="12" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
+      <c r="C40" s="6">
+        <f>COUNTIF(C14:C39,"Y")</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>COUNTIF(D14:D39,"Y")</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>COUNTIF(E14:E39,"Y")</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>COUNTIF(F14:F39,"Y")</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>COUNTIF(G14:G39,"Y")</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>COUNTIF(H14:H39,"Y")</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>COUNTIF(I14:I39,"Y")</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>COUNTIF(J14:J39,"Y")</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>COUNTIF(K14:K39,"Y")</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>COUNTIF(L14:L39,"Y")</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>COUNTIF(M14:M39,"Y")</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>COUNTIF(N14:N39,"Y")</f>
+        <v/>
+      </c>
+      <c r="O40" s="6">
+        <f>COUNTIF(O14:O39,"Y")</f>
+        <v/>
+      </c>
+      <c r="P40" s="3" t="inlineStr"/>
+      <c r="Q40" s="6">
+        <f>SUM(Q14:Q39)</f>
+        <v/>
+      </c>
+      <c r="R40" s="37">
+        <f>SUM(R14:R39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>Y = on shift during shop's meal window. Personal Avg = average score of shops worked. Bonus = $50 per 100% shop worked.</t>
         </is>
@@ -7420,11 +7565,11 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A18:R18"/>
+    <mergeCell ref="A41:R41"/>
     <mergeCell ref="A2:R2"/>
     <mergeCell ref="A19:R19"/>
     <mergeCell ref="A13:R13"/>
     <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A40:R40"/>
     <mergeCell ref="A12:R12"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -7439,7 +7584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8587,7 +8732,7 @@
       </c>
       <c r="B30" s="32" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="C30" s="33" t="n"/>
@@ -8623,7 +8768,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
@@ -8659,7 +8804,7 @@
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="C32" s="33" t="n"/>
@@ -8695,42 +8840,22 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="C33" s="19" t="n"/>
-      <c r="D33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D33" s="19" t="n"/>
       <c r="E33" s="19" t="n"/>
       <c r="F33" s="19" t="n"/>
       <c r="G33" s="19" t="n"/>
       <c r="H33" s="19" t="n"/>
       <c r="I33" s="19" t="n"/>
-      <c r="J33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J33" s="19" t="n"/>
+      <c r="K33" s="19" t="n"/>
       <c r="L33" s="19" t="n"/>
-      <c r="M33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M33" s="19" t="n"/>
       <c r="N33" s="19" t="n"/>
-      <c r="O33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="O33" s="19" t="n"/>
       <c r="P33" s="19" t="n"/>
       <c r="Q33" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$P$7,C33:P33,"Y"),"")</f>
@@ -8751,7 +8876,7 @@
       </c>
       <c r="B34" s="32" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="C34" s="33" t="n"/>
@@ -8765,25 +8890,29 @@
       <c r="G34" s="33" t="n"/>
       <c r="H34" s="33" t="n"/>
       <c r="I34" s="33" t="n"/>
-      <c r="J34" s="33" t="n"/>
-      <c r="K34" s="33" t="n"/>
-      <c r="L34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M34" s="33" t="n"/>
+      <c r="J34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L34" s="33" t="n"/>
+      <c r="M34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="N34" s="33" t="n"/>
       <c r="O34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="P34" s="33" t="n"/>
       <c r="Q34" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$P$7,C34:P34,"Y"),"")</f>
         <v/>
@@ -8803,11 +8932,15 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E35" s="19" t="n"/>
       <c r="F35" s="19" t="n"/>
       <c r="G35" s="19" t="n"/>
@@ -8815,11 +8948,23 @@
       <c r="I35" s="19" t="n"/>
       <c r="J35" s="19" t="n"/>
       <c r="K35" s="19" t="n"/>
-      <c r="L35" s="19" t="n"/>
+      <c r="L35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M35" s="19" t="n"/>
       <c r="N35" s="19" t="n"/>
-      <c r="O35" s="19" t="n"/>
-      <c r="P35" s="19" t="n"/>
+      <c r="O35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="Q35" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$P$7,C35:P35,"Y"),"")</f>
         <v/>
@@ -8839,7 +8984,7 @@
       </c>
       <c r="B36" s="32" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C36" s="33" t="n"/>
@@ -8852,11 +8997,7 @@
       <c r="J36" s="33" t="n"/>
       <c r="K36" s="33" t="n"/>
       <c r="L36" s="33" t="n"/>
-      <c r="M36" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M36" s="33" t="n"/>
       <c r="N36" s="33" t="n"/>
       <c r="O36" s="33" t="n"/>
       <c r="P36" s="33" t="n"/>
@@ -8879,32 +9020,24 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Samuel</t>
-        </is>
-      </c>
-      <c r="C37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="n"/>
       <c r="D37" s="19" t="n"/>
-      <c r="E37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E37" s="19" t="n"/>
       <c r="F37" s="19" t="n"/>
       <c r="G37" s="19" t="n"/>
       <c r="H37" s="19" t="n"/>
-      <c r="I37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="I37" s="19" t="n"/>
       <c r="J37" s="19" t="n"/>
       <c r="K37" s="19" t="n"/>
       <c r="L37" s="19" t="n"/>
-      <c r="M37" s="19" t="n"/>
+      <c r="M37" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="N37" s="19" t="n"/>
       <c r="O37" s="19" t="n"/>
       <c r="P37" s="19" t="n"/>
@@ -8927,16 +9060,28 @@
       </c>
       <c r="B38" s="32" t="inlineStr">
         <is>
-          <t>Zach</t>
-        </is>
-      </c>
-      <c r="C38" s="33" t="n"/>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D38" s="33" t="n"/>
-      <c r="E38" s="33" t="n"/>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F38" s="33" t="n"/>
       <c r="G38" s="33" t="n"/>
       <c r="H38" s="33" t="n"/>
-      <c r="I38" s="33" t="n"/>
+      <c r="I38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J38" s="33" t="n"/>
       <c r="K38" s="33" t="n"/>
       <c r="L38" s="33" t="n"/>
@@ -8957,81 +9102,117 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr"/>
-      <c r="B39" s="36" t="inlineStr">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="19" t="n"/>
+      <c r="P39" s="19" t="n"/>
+      <c r="Q39" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$P$7,C39:P39,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R39" s="28">
+        <f>COUNTIF(C39:P39,"Y")</f>
+        <v/>
+      </c>
+      <c r="S39" s="29">
+        <f>SUMPRODUCT((C$7:$P$7=1)*(C39:P39="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>Total on shift</t>
         </is>
       </c>
-      <c r="C39" s="6">
-        <f>COUNTIF(C14:C38,"Y")</f>
-        <v/>
-      </c>
-      <c r="D39" s="6">
-        <f>COUNTIF(D14:D38,"Y")</f>
-        <v/>
-      </c>
-      <c r="E39" s="6">
-        <f>COUNTIF(E14:E38,"Y")</f>
-        <v/>
-      </c>
-      <c r="F39" s="6">
-        <f>COUNTIF(F14:F38,"Y")</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>COUNTIF(G14:G38,"Y")</f>
-        <v/>
-      </c>
-      <c r="H39" s="6">
-        <f>COUNTIF(H14:H38,"Y")</f>
-        <v/>
-      </c>
-      <c r="I39" s="6">
-        <f>COUNTIF(I14:I38,"Y")</f>
-        <v/>
-      </c>
-      <c r="J39" s="6">
-        <f>COUNTIF(J14:J38,"Y")</f>
-        <v/>
-      </c>
-      <c r="K39" s="6">
-        <f>COUNTIF(K14:K38,"Y")</f>
-        <v/>
-      </c>
-      <c r="L39" s="6">
-        <f>COUNTIF(L14:L38,"Y")</f>
-        <v/>
-      </c>
-      <c r="M39" s="6">
-        <f>COUNTIF(M14:M38,"Y")</f>
-        <v/>
-      </c>
-      <c r="N39" s="6">
-        <f>COUNTIF(N14:N38,"Y")</f>
-        <v/>
-      </c>
-      <c r="O39" s="6">
-        <f>COUNTIF(O14:O38,"Y")</f>
-        <v/>
-      </c>
-      <c r="P39" s="6">
-        <f>COUNTIF(P14:P38,"Y")</f>
-        <v/>
-      </c>
-      <c r="Q39" s="3" t="inlineStr"/>
-      <c r="R39" s="6">
-        <f>SUM(R14:R38)</f>
-        <v/>
-      </c>
-      <c r="S39" s="37">
-        <f>SUM(S14:S38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="12" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
+      <c r="C40" s="6">
+        <f>COUNTIF(C14:C39,"Y")</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>COUNTIF(D14:D39,"Y")</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>COUNTIF(E14:E39,"Y")</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>COUNTIF(F14:F39,"Y")</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>COUNTIF(G14:G39,"Y")</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>COUNTIF(H14:H39,"Y")</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>COUNTIF(I14:I39,"Y")</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>COUNTIF(J14:J39,"Y")</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>COUNTIF(K14:K39,"Y")</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>COUNTIF(L14:L39,"Y")</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>COUNTIF(M14:M39,"Y")</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>COUNTIF(N14:N39,"Y")</f>
+        <v/>
+      </c>
+      <c r="O40" s="6">
+        <f>COUNTIF(O14:O39,"Y")</f>
+        <v/>
+      </c>
+      <c r="P40" s="6">
+        <f>COUNTIF(P14:P39,"Y")</f>
+        <v/>
+      </c>
+      <c r="Q40" s="3" t="inlineStr"/>
+      <c r="R40" s="6">
+        <f>SUM(R14:R39)</f>
+        <v/>
+      </c>
+      <c r="S40" s="37">
+        <f>SUM(S14:S39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>Y = on shift during shop's meal window. Personal Avg = average score of shops worked. Bonus = $50 per 100% shop worked.</t>
         </is>
@@ -9039,10 +9220,10 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A41:S41"/>
     <mergeCell ref="A19:S19"/>
     <mergeCell ref="A13:S13"/>
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="A40:S40"/>
     <mergeCell ref="A18:S18"/>
     <mergeCell ref="A12:S12"/>
     <mergeCell ref="A2:S2"/>
@@ -9059,7 +9240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P40"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9550,7 +9731,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M15" s="27" t="n"/>
+      <c r="M15" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="N15" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C15:M15,"Y"),"")</f>
         <v/>
@@ -9583,11 +9768,7 @@
       <c r="J16" s="27" t="n"/>
       <c r="K16" s="27" t="n"/>
       <c r="L16" s="27" t="n"/>
-      <c r="M16" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M16" s="27" t="n"/>
       <c r="N16" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C16:M16,"Y"),"")</f>
         <v/>
@@ -9620,11 +9801,7 @@
       <c r="J17" s="27" t="n"/>
       <c r="K17" s="27" t="n"/>
       <c r="L17" s="27" t="n"/>
-      <c r="M17" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M17" s="27" t="n"/>
       <c r="N17" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C17:M17,"Y"),"")</f>
         <v/>
@@ -9770,7 +9947,11 @@
       <c r="J23" s="19" t="n"/>
       <c r="K23" s="19" t="n"/>
       <c r="L23" s="19" t="n"/>
-      <c r="M23" s="19" t="n"/>
+      <c r="M23" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="N23" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C23:M23,"Y"),"")</f>
         <v/>
@@ -9947,11 +10128,7 @@
       <c r="J28" s="33" t="n"/>
       <c r="K28" s="33" t="n"/>
       <c r="L28" s="33" t="n"/>
-      <c r="M28" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M28" s="33" t="n"/>
       <c r="N28" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C28:M28,"Y"),"")</f>
         <v/>
@@ -10016,7 +10193,7 @@
       </c>
       <c r="B30" s="32" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="C30" s="33" t="n"/>
@@ -10029,7 +10206,11 @@
       <c r="J30" s="33" t="n"/>
       <c r="K30" s="33" t="n"/>
       <c r="L30" s="33" t="n"/>
-      <c r="M30" s="33" t="n"/>
+      <c r="M30" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="N30" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C30:M30,"Y"),"")</f>
         <v/>
@@ -10049,7 +10230,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
@@ -10082,7 +10263,7 @@
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="C32" s="33" t="n"/>
@@ -10115,44 +10296,20 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="C33" s="19" t="n"/>
-      <c r="D33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D33" s="19" t="n"/>
       <c r="E33" s="19" t="n"/>
-      <c r="F33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F33" s="19" t="n"/>
       <c r="G33" s="19" t="n"/>
-      <c r="H33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="H33" s="19" t="n"/>
       <c r="I33" s="19" t="n"/>
-      <c r="J33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="J33" s="19" t="n"/>
       <c r="K33" s="19" t="n"/>
-      <c r="L33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M33" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L33" s="19" t="n"/>
+      <c r="M33" s="19" t="n"/>
       <c r="N33" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C33:M33,"Y"),"")</f>
         <v/>
@@ -10172,32 +10329,44 @@
       </c>
       <c r="B34" s="32" t="inlineStr">
         <is>
-          <t>Maylin</t>
-        </is>
-      </c>
-      <c r="C34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Lidy</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="n"/>
       <c r="D34" s="26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="E34" s="33" t="n"/>
-      <c r="F34" s="33" t="n"/>
+      <c r="F34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G34" s="33" t="n"/>
-      <c r="H34" s="33" t="n"/>
+      <c r="H34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I34" s="33" t="n"/>
-      <c r="J34" s="33" t="n"/>
-      <c r="K34" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L34" s="33" t="n"/>
-      <c r="M34" s="33" t="n"/>
+      <c r="J34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K34" s="33" t="n"/>
+      <c r="L34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M34" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="N34" s="18">
         <f>IFERROR(AVERAGEIFS($C$7:$M$7,C34:M34,"Y"),"")</f>
         <v/>
@@ -10217,18 +10386,30 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>Mike</t>
-        </is>
-      </c>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
+          <t>Maylin</t>
+        </is>
+      </c>
+      <c r="C35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E35" s="19" t="n"/>
       <c r="F35" s="19" t="n"/>
       <c r="G35" s="19" t="n"/>
       <c r="H35" s="19" t="n"/>
       <c r="I35" s="19" t="n"/>
       <c r="J35" s="19" t="n"/>
-      <c r="K35" s="19" t="n"/>
+      <c r="K35" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L35" s="19" t="n"/>
       <c r="M35" s="19" t="n"/>
       <c r="N35" s="18">
@@ -10250,7 +10431,7 @@
       </c>
       <c r="B36" s="32" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C36" s="33" t="n"/>
@@ -10283,34 +10464,18 @@
       </c>
       <c r="B37" s="35" t="inlineStr">
         <is>
-          <t>Samuel</t>
-        </is>
-      </c>
-      <c r="C37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="n"/>
       <c r="D37" s="19" t="n"/>
       <c r="E37" s="19" t="n"/>
       <c r="F37" s="19" t="n"/>
-      <c r="G37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G37" s="19" t="n"/>
       <c r="H37" s="19" t="n"/>
-      <c r="I37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="I37" s="19" t="n"/>
       <c r="J37" s="19" t="n"/>
-      <c r="K37" s="26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="K37" s="19" t="n"/>
       <c r="L37" s="19" t="n"/>
       <c r="M37" s="19" t="n"/>
       <c r="N37" s="18">
@@ -10332,18 +10497,34 @@
       </c>
       <c r="B38" s="32" t="inlineStr">
         <is>
-          <t>Zach</t>
-        </is>
-      </c>
-      <c r="C38" s="33" t="n"/>
+          <t>Samuel</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D38" s="33" t="n"/>
       <c r="E38" s="33" t="n"/>
       <c r="F38" s="33" t="n"/>
-      <c r="G38" s="33" t="n"/>
+      <c r="G38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H38" s="33" t="n"/>
-      <c r="I38" s="33" t="n"/>
+      <c r="I38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J38" s="33" t="n"/>
-      <c r="K38" s="33" t="n"/>
+      <c r="K38" s="26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L38" s="33" t="n"/>
       <c r="M38" s="33" t="n"/>
       <c r="N38" s="18">
@@ -10359,69 +10540,102 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr"/>
-      <c r="B39" s="36" t="inlineStr">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="18">
+        <f>IFERROR(AVERAGEIFS($C$7:$M$7,C39:M39,"Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O39" s="28">
+        <f>COUNTIF(C39:M39,"Y")</f>
+        <v/>
+      </c>
+      <c r="P39" s="29">
+        <f>SUMPRODUCT((C$7:$M$7=1)*(C39:M39="Y"))*50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>Total on shift</t>
         </is>
       </c>
-      <c r="C39" s="6">
-        <f>COUNTIF(C14:C38,"Y")</f>
-        <v/>
-      </c>
-      <c r="D39" s="6">
-        <f>COUNTIF(D14:D38,"Y")</f>
-        <v/>
-      </c>
-      <c r="E39" s="6">
-        <f>COUNTIF(E14:E38,"Y")</f>
-        <v/>
-      </c>
-      <c r="F39" s="6">
-        <f>COUNTIF(F14:F38,"Y")</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>COUNTIF(G14:G38,"Y")</f>
-        <v/>
-      </c>
-      <c r="H39" s="6">
-        <f>COUNTIF(H14:H38,"Y")</f>
-        <v/>
-      </c>
-      <c r="I39" s="6">
-        <f>COUNTIF(I14:I38,"Y")</f>
-        <v/>
-      </c>
-      <c r="J39" s="6">
-        <f>COUNTIF(J14:J38,"Y")</f>
-        <v/>
-      </c>
-      <c r="K39" s="6">
-        <f>COUNTIF(K14:K38,"Y")</f>
-        <v/>
-      </c>
-      <c r="L39" s="6">
-        <f>COUNTIF(L14:L38,"Y")</f>
-        <v/>
-      </c>
-      <c r="M39" s="6">
-        <f>COUNTIF(M14:M38,"Y")</f>
-        <v/>
-      </c>
-      <c r="N39" s="3" t="inlineStr"/>
-      <c r="O39" s="6">
-        <f>SUM(O14:O38)</f>
-        <v/>
-      </c>
-      <c r="P39" s="37">
-        <f>SUM(P14:P38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="12" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
+      <c r="C40" s="6">
+        <f>COUNTIF(C14:C39,"Y")</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>COUNTIF(D14:D39,"Y")</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>COUNTIF(E14:E39,"Y")</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>COUNTIF(F14:F39,"Y")</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>COUNTIF(G14:G39,"Y")</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>COUNTIF(H14:H39,"Y")</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>COUNTIF(I14:I39,"Y")</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>COUNTIF(J14:J39,"Y")</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>COUNTIF(K14:K39,"Y")</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>COUNTIF(L14:L39,"Y")</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>COUNTIF(M14:M39,"Y")</f>
+        <v/>
+      </c>
+      <c r="N40" s="3" t="inlineStr"/>
+      <c r="O40" s="6">
+        <f>SUM(O14:O39)</f>
+        <v/>
+      </c>
+      <c r="P40" s="37">
+        <f>SUM(P14:P39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>Y = on shift during shop's meal window. Personal Avg = average score of shops worked. Bonus = $50 per 100% shop worked.</t>
         </is>
@@ -10431,10 +10645,10 @@
   <mergeCells count="7">
     <mergeCell ref="A13:P13"/>
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A40:P40"/>
     <mergeCell ref="A18:P18"/>
     <mergeCell ref="A12:P12"/>
     <mergeCell ref="A19:P19"/>
+    <mergeCell ref="A41:P41"/>
     <mergeCell ref="A2:P2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
directory + tracker: restore Kaisha Brewer (E2065272938) as Active
Kaisha was incorrectly removed. Re-added to EMPLOYEES list (alphabetical,
phone PENDING) and CREW list. Shop tracker regenerated — June 4 100% shop
payout shows $46.00 (n=5: Bri, Kaisha, Lidy, Vicki, Zack).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>Kayla Valenzuela</t>
+          <t>Kaisha Brewer</t>
         </is>
       </c>
       <c r="C28" s="28" t="n"/>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla Valenzuela</t>
         </is>
       </c>
       <c r="C29" s="28" t="n"/>
@@ -1549,30 +1549,22 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>Lidy Henry</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="28" t="n"/>
-      <c r="E30" s="30" t="n">
-        <v>80</v>
-      </c>
+      <c r="E30" s="28" t="n"/>
       <c r="F30" s="28" t="n"/>
-      <c r="G30" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="G30" s="28" t="n"/>
       <c r="H30" s="28" t="n"/>
       <c r="I30" s="28" t="n"/>
-      <c r="J30" s="30" t="n">
-        <v>85</v>
-      </c>
+      <c r="J30" s="28" t="n"/>
       <c r="K30" s="23">
         <f>IFERROR(AVERAGE(C30:J30),"")</f>
         <v/>
       </c>
-      <c r="L30" s="24" t="n">
-        <v>38.33</v>
-      </c>
+      <c r="L30" s="28" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -1582,25 +1574,23 @@
       </c>
       <c r="B31" s="27" t="inlineStr">
         <is>
-          <t>Maylin Hernandez Rodriguez</t>
+          <t>Lidy Henry</t>
         </is>
       </c>
       <c r="C31" s="28" t="n"/>
-      <c r="D31" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="28" t="n"/>
-      <c r="F31" s="25" t="n">
-        <v>72</v>
-      </c>
+      <c r="D31" s="28" t="n"/>
+      <c r="E31" s="30" t="n">
+        <v>80</v>
+      </c>
+      <c r="F31" s="28" t="n"/>
       <c r="G31" s="22" t="n">
         <v>100</v>
       </c>
       <c r="H31" s="28" t="n"/>
-      <c r="I31" s="30" t="n">
-        <v>80</v>
-      </c>
-      <c r="J31" s="28" t="n"/>
+      <c r="I31" s="28" t="n"/>
+      <c r="J31" s="30" t="n">
+        <v>85</v>
+      </c>
       <c r="K31" s="23">
         <f>IFERROR(AVERAGE(C31:J31),"")</f>
         <v/>
@@ -1617,32 +1607,32 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Mike</t>
-        </is>
-      </c>
-      <c r="C32" s="29" t="n">
-        <v>92</v>
-      </c>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="30" t="n">
-        <v>80</v>
-      </c>
+          <t>Maylin Hernandez Rodriguez</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="n"/>
+      <c r="D32" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="28" t="n"/>
       <c r="F32" s="25" t="n">
         <v>72</v>
       </c>
-      <c r="G32" s="28" t="n"/>
+      <c r="G32" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="H32" s="28" t="n"/>
       <c r="I32" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="J32" s="30" t="n">
-        <v>85</v>
-      </c>
+      <c r="J32" s="28" t="n"/>
       <c r="K32" s="23">
         <f>IFERROR(AVERAGE(C32:J32),"")</f>
         <v/>
       </c>
-      <c r="L32" s="28" t="n"/>
+      <c r="L32" s="24" t="n">
+        <v>38.33</v>
+      </c>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
@@ -1652,17 +1642,27 @@
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>Nyatiek Keah</t>
-        </is>
-      </c>
-      <c r="C33" s="28" t="n"/>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="n">
+        <v>92</v>
+      </c>
       <c r="D33" s="28" t="n"/>
-      <c r="E33" s="28" t="n"/>
-      <c r="F33" s="28" t="n"/>
+      <c r="E33" s="30" t="n">
+        <v>80</v>
+      </c>
+      <c r="F33" s="25" t="n">
+        <v>72</v>
+      </c>
       <c r="G33" s="28" t="n"/>
       <c r="H33" s="28" t="n"/>
-      <c r="I33" s="28" t="n"/>
-      <c r="J33" s="28" t="n"/>
+      <c r="I33" s="30" t="n">
+        <v>80</v>
+      </c>
+      <c r="J33" s="30" t="n">
+        <v>85</v>
+      </c>
       <c r="K33" s="23">
         <f>IFERROR(AVERAGE(C33:J33),"")</f>
         <v/>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek Keah</t>
         </is>
       </c>
       <c r="C34" s="28" t="n"/>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B35" s="27" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="C35" s="28" t="n"/>
@@ -1727,32 +1727,22 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>Samuel Galban Rocha</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="C36" s="28" t="n"/>
-      <c r="D36" s="25" t="n">
-        <v>0</v>
-      </c>
+      <c r="D36" s="28" t="n"/>
       <c r="E36" s="28" t="n"/>
-      <c r="F36" s="25" t="n">
-        <v>72</v>
-      </c>
+      <c r="F36" s="28" t="n"/>
       <c r="G36" s="28" t="n"/>
-      <c r="H36" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="I36" s="30" t="n">
-        <v>80</v>
-      </c>
+      <c r="H36" s="28" t="n"/>
+      <c r="I36" s="28" t="n"/>
       <c r="J36" s="28" t="n"/>
       <c r="K36" s="23">
         <f>IFERROR(AVERAGE(C36:J36),"")</f>
         <v/>
       </c>
-      <c r="L36" s="24" t="n">
-        <v>46</v>
-      </c>
+      <c r="L36" s="28" t="n"/>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
@@ -1762,25 +1752,60 @@
       </c>
       <c r="B37" s="27" t="inlineStr">
         <is>
-          <t>Zack Whitten</t>
+          <t>Samuel Galban Rocha</t>
         </is>
       </c>
       <c r="C37" s="28" t="n"/>
-      <c r="D37" s="28" t="n"/>
+      <c r="D37" s="25" t="n">
+        <v>0</v>
+      </c>
       <c r="E37" s="28" t="n"/>
-      <c r="F37" s="28" t="n"/>
+      <c r="F37" s="25" t="n">
+        <v>72</v>
+      </c>
       <c r="G37" s="28" t="n"/>
-      <c r="H37" s="28" t="n"/>
-      <c r="I37" s="28" t="n"/>
+      <c r="H37" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I37" s="30" t="n">
+        <v>80</v>
+      </c>
       <c r="J37" s="28" t="n"/>
       <c r="K37" s="23">
         <f>IFERROR(AVERAGE(C37:J37),"")</f>
         <v/>
       </c>
-      <c r="L37" s="28" t="n"/>
-    </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="31" t="inlineStr">
+      <c r="L37" s="24" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Zack Whitten</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+      <c r="H38" s="28" t="n"/>
+      <c r="I38" s="28" t="n"/>
+      <c r="J38" s="28" t="n"/>
+      <c r="K38" s="23">
+        <f>IFERROR(AVERAGE(C38:J38),"")</f>
+        <v/>
+      </c>
+      <c r="L38" s="28" t="n"/>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Score = shop score if on shift during meal window; blank if not. MTD SCORE = average of scores worked. MTD DOLLARS = $230 ÷ on-shift count per 100% shop.</t>
         </is>
@@ -1788,7 +1813,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A38:L38"/>
+    <mergeCell ref="A39:L39"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -1804,7 +1829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2495,7 +2520,7 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>Kayla Valenzuela</t>
+          <t>Kaisha Brewer</t>
         </is>
       </c>
       <c r="C28" s="28" t="n"/>
@@ -2518,7 +2543,7 @@
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla Valenzuela</t>
         </is>
       </c>
       <c r="C29" s="28" t="n"/>
@@ -2541,28 +2566,20 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>Lidy Henry</t>
-        </is>
-      </c>
-      <c r="C30" s="22" t="n">
-        <v>100</v>
-      </c>
+          <t>Kenzie</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="n"/>
       <c r="D30" s="28" t="n"/>
-      <c r="E30" s="25" t="n">
-        <v>69</v>
-      </c>
+      <c r="E30" s="28" t="n"/>
       <c r="F30" s="28" t="n"/>
-      <c r="G30" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="G30" s="28" t="n"/>
       <c r="H30" s="28" t="n"/>
       <c r="I30" s="23">
         <f>IFERROR(AVERAGE(C30:H30),"")</f>
         <v/>
       </c>
-      <c r="J30" s="24" t="n">
-        <v>84.33</v>
-      </c>
+      <c r="J30" s="28" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -2572,19 +2589,17 @@
       </c>
       <c r="B31" s="27" t="inlineStr">
         <is>
-          <t>Maylin Hernandez Rodriguez</t>
-        </is>
-      </c>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="22" t="n">
+          <t>Lidy Henry</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n">
         <v>100</v>
       </c>
+      <c r="D31" s="28" t="n"/>
       <c r="E31" s="25" t="n">
         <v>69</v>
       </c>
-      <c r="F31" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="F31" s="28" t="n"/>
       <c r="G31" s="22" t="n">
         <v>100</v>
       </c>
@@ -2594,7 +2609,7 @@
         <v/>
       </c>
       <c r="J31" s="24" t="n">
-        <v>153.33</v>
+        <v>84.33</v>
       </c>
     </row>
     <row r="32" ht="17" customHeight="1">
@@ -2605,29 +2620,29 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Mike</t>
-        </is>
-      </c>
-      <c r="C32" s="22" t="n">
+          <t>Maylin Hernandez Rodriguez</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="n"/>
+      <c r="D32" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="D32" s="28" t="n"/>
       <c r="E32" s="25" t="n">
         <v>69</v>
       </c>
-      <c r="F32" s="28" t="n"/>
+      <c r="F32" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="G32" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="H32" s="29" t="n">
-        <v>95</v>
-      </c>
+      <c r="H32" s="28" t="n"/>
       <c r="I32" s="23">
         <f>IFERROR(AVERAGE(C32:H32),"")</f>
         <v/>
       </c>
       <c r="J32" s="24" t="n">
-        <v>84.33</v>
+        <v>153.33</v>
       </c>
     </row>
     <row r="33" ht="17" customHeight="1">
@@ -2638,20 +2653,30 @@
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>Nyatiek Keah</t>
-        </is>
-      </c>
-      <c r="C33" s="28" t="n"/>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="D33" s="28" t="n"/>
-      <c r="E33" s="28" t="n"/>
+      <c r="E33" s="25" t="n">
+        <v>69</v>
+      </c>
       <c r="F33" s="28" t="n"/>
-      <c r="G33" s="28" t="n"/>
-      <c r="H33" s="28" t="n"/>
+      <c r="G33" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H33" s="29" t="n">
+        <v>95</v>
+      </c>
       <c r="I33" s="23">
         <f>IFERROR(AVERAGE(C33:H33),"")</f>
         <v/>
       </c>
-      <c r="J33" s="28" t="n"/>
+      <c r="J33" s="24" t="n">
+        <v>84.33</v>
+      </c>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
@@ -2661,7 +2686,7 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek Keah</t>
         </is>
       </c>
       <c r="C34" s="28" t="n"/>
@@ -2684,7 +2709,7 @@
       </c>
       <c r="B35" s="27" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="C35" s="28" t="n"/>
@@ -2707,26 +2732,20 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>Samuel Galban Rocha</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="C36" s="28" t="n"/>
-      <c r="D36" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="D36" s="28" t="n"/>
       <c r="E36" s="28" t="n"/>
-      <c r="F36" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="F36" s="28" t="n"/>
       <c r="G36" s="28" t="n"/>
       <c r="H36" s="28" t="n"/>
       <c r="I36" s="23">
         <f>IFERROR(AVERAGE(C36:H36),"")</f>
         <v/>
       </c>
-      <c r="J36" s="24" t="n">
-        <v>115</v>
-      </c>
+      <c r="J36" s="28" t="n"/>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
@@ -2736,23 +2755,52 @@
       </c>
       <c r="B37" s="27" t="inlineStr">
         <is>
-          <t>Zack Whitten</t>
+          <t>Samuel Galban Rocha</t>
         </is>
       </c>
       <c r="C37" s="28" t="n"/>
-      <c r="D37" s="28" t="n"/>
+      <c r="D37" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="E37" s="28" t="n"/>
-      <c r="F37" s="28" t="n"/>
+      <c r="F37" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="G37" s="28" t="n"/>
       <c r="H37" s="28" t="n"/>
       <c r="I37" s="23">
         <f>IFERROR(AVERAGE(C37:H37),"")</f>
         <v/>
       </c>
-      <c r="J37" s="28" t="n"/>
-    </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="31" t="inlineStr">
+      <c r="J37" s="24" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Zack Whitten</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+      <c r="H38" s="28" t="n"/>
+      <c r="I38" s="23">
+        <f>IFERROR(AVERAGE(C38:H38),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="28" t="n"/>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Score = shop score if on shift during meal window; blank if not. MTD SCORE = average of scores worked. MTD DOLLARS = $230 ÷ on-shift count per 100% shop.</t>
         </is>
@@ -2760,9 +2808,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A39:J39"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A38:J38"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2776,7 +2824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3424,7 +3472,7 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>Kayla Valenzuela</t>
+          <t>Kaisha Brewer</t>
         </is>
       </c>
       <c r="C28" s="28" t="n"/>
@@ -3446,7 +3494,7 @@
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla Valenzuela</t>
         </is>
       </c>
       <c r="C29" s="28" t="n"/>
@@ -3468,25 +3516,19 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>Lidy Henry</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="C30" s="28" t="n"/>
-      <c r="D30" s="30" t="n">
-        <v>80</v>
-      </c>
+      <c r="D30" s="28" t="n"/>
       <c r="E30" s="28" t="n"/>
       <c r="F30" s="28" t="n"/>
-      <c r="G30" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="G30" s="28" t="n"/>
       <c r="H30" s="23">
         <f>IFERROR(AVERAGE(C30:G30),"")</f>
         <v/>
       </c>
-      <c r="I30" s="24" t="n">
-        <v>38.33</v>
-      </c>
+      <c r="I30" s="28" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -3496,21 +3538,15 @@
       </c>
       <c r="B31" s="27" t="inlineStr">
         <is>
-          <t>Maylin Hernandez Rodriguez</t>
-        </is>
-      </c>
-      <c r="C31" s="25" t="n">
-        <v>72</v>
-      </c>
+          <t>Lidy Henry</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="n"/>
       <c r="D31" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="E31" s="25" t="n">
-        <v>72</v>
-      </c>
-      <c r="F31" s="25" t="n">
-        <v>49</v>
-      </c>
+      <c r="E31" s="28" t="n"/>
+      <c r="F31" s="28" t="n"/>
       <c r="G31" s="22" t="n">
         <v>100</v>
       </c>
@@ -3530,19 +3566,31 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Mike</t>
-        </is>
-      </c>
-      <c r="C32" s="28" t="n"/>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="28" t="n"/>
-      <c r="F32" s="28" t="n"/>
-      <c r="G32" s="28" t="n"/>
+          <t>Maylin Hernandez Rodriguez</t>
+        </is>
+      </c>
+      <c r="C32" s="25" t="n">
+        <v>72</v>
+      </c>
+      <c r="D32" s="30" t="n">
+        <v>80</v>
+      </c>
+      <c r="E32" s="25" t="n">
+        <v>72</v>
+      </c>
+      <c r="F32" s="25" t="n">
+        <v>49</v>
+      </c>
+      <c r="G32" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="H32" s="23">
         <f>IFERROR(AVERAGE(C32:G32),"")</f>
         <v/>
       </c>
-      <c r="I32" s="28" t="n"/>
+      <c r="I32" s="24" t="n">
+        <v>38.33</v>
+      </c>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
@@ -3552,7 +3600,7 @@
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>Nyatiek Keah</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C33" s="28" t="n"/>
@@ -3574,7 +3622,7 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek Keah</t>
         </is>
       </c>
       <c r="C34" s="28" t="n"/>
@@ -3596,7 +3644,7 @@
       </c>
       <c r="B35" s="27" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="C35" s="28" t="n"/>
@@ -3618,12 +3666,10 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>Samuel Galban Rocha</t>
-        </is>
-      </c>
-      <c r="C36" s="25" t="n">
-        <v>72</v>
-      </c>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="n"/>
       <c r="D36" s="28" t="n"/>
       <c r="E36" s="28" t="n"/>
       <c r="F36" s="28" t="n"/>
@@ -3642,10 +3688,12 @@
       </c>
       <c r="B37" s="27" t="inlineStr">
         <is>
-          <t>Zack Whitten</t>
-        </is>
-      </c>
-      <c r="C37" s="28" t="n"/>
+          <t>Samuel Galban Rocha</t>
+        </is>
+      </c>
+      <c r="C37" s="25" t="n">
+        <v>72</v>
+      </c>
       <c r="D37" s="28" t="n"/>
       <c r="E37" s="28" t="n"/>
       <c r="F37" s="28" t="n"/>
@@ -3656,8 +3704,30 @@
       </c>
       <c r="I37" s="28" t="n"/>
     </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="31" t="inlineStr">
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Zack Whitten</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+      <c r="H38" s="23">
+        <f>IFERROR(AVERAGE(C38:G38),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="28" t="n"/>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Score = shop score if on shift during meal window; blank if not. MTD SCORE = average of scores worked. MTD DOLLARS = $230 ÷ on-shift count per 100% shop.</t>
         </is>
@@ -3667,7 +3737,7 @@
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="A39:I39"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3681,7 +3751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4376,7 +4446,7 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>Kayla Valenzuela</t>
+          <t>Kaisha Brewer</t>
         </is>
       </c>
       <c r="C28" s="28" t="n"/>
@@ -4399,7 +4469,7 @@
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla Valenzuela</t>
         </is>
       </c>
       <c r="C29" s="28" t="n"/>
@@ -4422,21 +4492,15 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>Lidy Henry</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="C30" s="28" t="n"/>
-      <c r="D30" s="30" t="n">
-        <v>87</v>
-      </c>
+      <c r="D30" s="28" t="n"/>
       <c r="E30" s="28" t="n"/>
-      <c r="F30" s="25" t="n">
-        <v>47</v>
-      </c>
+      <c r="F30" s="28" t="n"/>
       <c r="G30" s="28" t="n"/>
-      <c r="H30" s="30" t="n">
-        <v>87</v>
-      </c>
+      <c r="H30" s="28" t="n"/>
       <c r="I30" s="23">
         <f>IFERROR(AVERAGE(C30:H30),"")</f>
         <v/>
@@ -4451,26 +4515,26 @@
       </c>
       <c r="B31" s="27" t="inlineStr">
         <is>
-          <t>Maylin Hernandez Rodriguez</t>
-        </is>
-      </c>
-      <c r="C31" s="29" t="n">
-        <v>97</v>
-      </c>
-      <c r="D31" s="28" t="n"/>
+          <t>Lidy Henry</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="n"/>
+      <c r="D31" s="30" t="n">
+        <v>87</v>
+      </c>
       <c r="E31" s="28" t="n"/>
-      <c r="F31" s="28" t="n"/>
-      <c r="G31" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H31" s="28" t="n"/>
+      <c r="F31" s="25" t="n">
+        <v>47</v>
+      </c>
+      <c r="G31" s="28" t="n"/>
+      <c r="H31" s="30" t="n">
+        <v>87</v>
+      </c>
       <c r="I31" s="23">
         <f>IFERROR(AVERAGE(C31:H31),"")</f>
         <v/>
       </c>
-      <c r="J31" s="24" t="n">
-        <v>38.33</v>
-      </c>
+      <c r="J31" s="28" t="n"/>
     </row>
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
@@ -4480,20 +4544,26 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Mike</t>
-        </is>
-      </c>
-      <c r="C32" s="28" t="n"/>
+          <t>Maylin Hernandez Rodriguez</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="n">
+        <v>97</v>
+      </c>
       <c r="D32" s="28" t="n"/>
       <c r="E32" s="28" t="n"/>
       <c r="F32" s="28" t="n"/>
-      <c r="G32" s="28" t="n"/>
+      <c r="G32" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="H32" s="28" t="n"/>
       <c r="I32" s="23">
         <f>IFERROR(AVERAGE(C32:H32),"")</f>
         <v/>
       </c>
-      <c r="J32" s="28" t="n"/>
+      <c r="J32" s="24" t="n">
+        <v>38.33</v>
+      </c>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
@@ -4503,7 +4573,7 @@
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>Nyatiek Keah</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C33" s="28" t="n"/>
@@ -4526,30 +4596,20 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
-        </is>
-      </c>
-      <c r="C34" s="29" t="n">
-        <v>97</v>
-      </c>
+          <t>Nyatiek Keah</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="n"/>
       <c r="D34" s="28" t="n"/>
-      <c r="E34" s="29" t="n">
-        <v>95</v>
-      </c>
-      <c r="F34" s="25" t="n">
-        <v>47</v>
-      </c>
-      <c r="G34" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="E34" s="28" t="n"/>
+      <c r="F34" s="28" t="n"/>
+      <c r="G34" s="28" t="n"/>
       <c r="H34" s="28" t="n"/>
       <c r="I34" s="23">
         <f>IFERROR(AVERAGE(C34:H34),"")</f>
         <v/>
       </c>
-      <c r="J34" s="24" t="n">
-        <v>38.33</v>
-      </c>
+      <c r="J34" s="28" t="n"/>
     </row>
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
@@ -4559,20 +4619,30 @@
       </c>
       <c r="B35" s="27" t="inlineStr">
         <is>
-          <t>Ryan</t>
-        </is>
-      </c>
-      <c r="C35" s="28" t="n"/>
+          <t>Richard Gibbs</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="n">
+        <v>97</v>
+      </c>
       <c r="D35" s="28" t="n"/>
-      <c r="E35" s="28" t="n"/>
-      <c r="F35" s="28" t="n"/>
-      <c r="G35" s="28" t="n"/>
+      <c r="E35" s="29" t="n">
+        <v>95</v>
+      </c>
+      <c r="F35" s="25" t="n">
+        <v>47</v>
+      </c>
+      <c r="G35" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="H35" s="28" t="n"/>
       <c r="I35" s="23">
         <f>IFERROR(AVERAGE(C35:H35),"")</f>
         <v/>
       </c>
-      <c r="J35" s="28" t="n"/>
+      <c r="J35" s="24" t="n">
+        <v>38.33</v>
+      </c>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
@@ -4582,12 +4652,10 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>Samuel Galban Rocha</t>
-        </is>
-      </c>
-      <c r="C36" s="29" t="n">
-        <v>97</v>
-      </c>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="n"/>
       <c r="D36" s="28" t="n"/>
       <c r="E36" s="28" t="n"/>
       <c r="F36" s="28" t="n"/>
@@ -4607,10 +4675,12 @@
       </c>
       <c r="B37" s="27" t="inlineStr">
         <is>
-          <t>Zack Whitten</t>
-        </is>
-      </c>
-      <c r="C37" s="28" t="n"/>
+          <t>Samuel Galban Rocha</t>
+        </is>
+      </c>
+      <c r="C37" s="29" t="n">
+        <v>97</v>
+      </c>
       <c r="D37" s="28" t="n"/>
       <c r="E37" s="28" t="n"/>
       <c r="F37" s="28" t="n"/>
@@ -4622,8 +4692,31 @@
       </c>
       <c r="J37" s="28" t="n"/>
     </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="31" t="inlineStr">
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Zack Whitten</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+      <c r="H38" s="28" t="n"/>
+      <c r="I38" s="23">
+        <f>IFERROR(AVERAGE(C38:H38),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="28" t="n"/>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Score = shop score if on shift during meal window; blank if not. MTD SCORE = average of scores worked. MTD DOLLARS = $230 ÷ on-shift count per 100% shop.</t>
         </is>
@@ -4631,9 +4724,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A39:J39"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A38:J38"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4647,7 +4740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5344,7 +5437,7 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>Kayla Valenzuela</t>
+          <t>Kaisha Brewer</t>
         </is>
       </c>
       <c r="C28" s="28" t="n"/>
@@ -5367,7 +5460,7 @@
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla Valenzuela</t>
         </is>
       </c>
       <c r="C29" s="28" t="n"/>
@@ -5390,28 +5483,20 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>Lidy Henry</t>
-        </is>
-      </c>
-      <c r="C30" s="22" t="n">
-        <v>100</v>
-      </c>
+          <t>Kenzie</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="n"/>
       <c r="D30" s="28" t="n"/>
-      <c r="E30" s="29" t="n">
-        <v>95</v>
-      </c>
+      <c r="E30" s="28" t="n"/>
       <c r="F30" s="28" t="n"/>
-      <c r="G30" s="25" t="n">
-        <v>60</v>
-      </c>
+      <c r="G30" s="28" t="n"/>
       <c r="H30" s="28" t="n"/>
       <c r="I30" s="23">
         <f>IFERROR(AVERAGE(C30:H30),"")</f>
         <v/>
       </c>
-      <c r="J30" s="24" t="n">
-        <v>46</v>
-      </c>
+      <c r="J30" s="28" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -5421,27 +5506,27 @@
       </c>
       <c r="B31" s="27" t="inlineStr">
         <is>
-          <t>Maylin Hernandez Rodriguez</t>
-        </is>
-      </c>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="22" t="n">
+          <t>Lidy Henry</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="E31" s="28" t="n"/>
+      <c r="D31" s="28" t="n"/>
+      <c r="E31" s="29" t="n">
+        <v>95</v>
+      </c>
       <c r="F31" s="28" t="n"/>
       <c r="G31" s="25" t="n">
         <v>60</v>
       </c>
-      <c r="H31" s="29" t="n">
-        <v>92</v>
-      </c>
+      <c r="H31" s="28" t="n"/>
       <c r="I31" s="23">
         <f>IFERROR(AVERAGE(C31:H31),"")</f>
         <v/>
       </c>
       <c r="J31" s="24" t="n">
-        <v>38.33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32" ht="17" customHeight="1">
@@ -5452,20 +5537,28 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin Hernandez Rodriguez</t>
         </is>
       </c>
       <c r="C32" s="28" t="n"/>
-      <c r="D32" s="28" t="n"/>
+      <c r="D32" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="E32" s="28" t="n"/>
       <c r="F32" s="28" t="n"/>
-      <c r="G32" s="28" t="n"/>
-      <c r="H32" s="28" t="n"/>
+      <c r="G32" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="H32" s="29" t="n">
+        <v>92</v>
+      </c>
       <c r="I32" s="23">
         <f>IFERROR(AVERAGE(C32:H32),"")</f>
         <v/>
       </c>
-      <c r="J32" s="28" t="n"/>
+      <c r="J32" s="24" t="n">
+        <v>38.33</v>
+      </c>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
@@ -5475,7 +5568,7 @@
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>Nyatiek Keah</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C33" s="28" t="n"/>
@@ -5498,14 +5591,12 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek Keah</t>
         </is>
       </c>
       <c r="C34" s="28" t="n"/>
       <c r="D34" s="28" t="n"/>
-      <c r="E34" s="29" t="n">
-        <v>95</v>
-      </c>
+      <c r="E34" s="28" t="n"/>
       <c r="F34" s="28" t="n"/>
       <c r="G34" s="28" t="n"/>
       <c r="H34" s="28" t="n"/>
@@ -5523,12 +5614,14 @@
       </c>
       <c r="B35" s="27" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="C35" s="28" t="n"/>
       <c r="D35" s="28" t="n"/>
-      <c r="E35" s="28" t="n"/>
+      <c r="E35" s="29" t="n">
+        <v>95</v>
+      </c>
       <c r="F35" s="28" t="n"/>
       <c r="G35" s="28" t="n"/>
       <c r="H35" s="28" t="n"/>
@@ -5546,7 +5639,7 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>Samuel Galban Rocha</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="C36" s="28" t="n"/>
@@ -5569,7 +5662,7 @@
       </c>
       <c r="B37" s="27" t="inlineStr">
         <is>
-          <t>Zack Whitten</t>
+          <t>Samuel Galban Rocha</t>
         </is>
       </c>
       <c r="C37" s="28" t="n"/>
@@ -5584,8 +5677,31 @@
       </c>
       <c r="J37" s="28" t="n"/>
     </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="31" t="inlineStr">
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Zack Whitten</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+      <c r="H38" s="28" t="n"/>
+      <c r="I38" s="23">
+        <f>IFERROR(AVERAGE(C38:H38),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="28" t="n"/>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Score = shop score if on shift during meal window; blank if not. MTD SCORE = average of scores worked. MTD DOLLARS = $230 ÷ on-shift count per 100% shop.</t>
         </is>
@@ -5593,9 +5709,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A39:J39"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A38:J38"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5609,7 +5725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6110,16 +6226,20 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>Kayla Valenzuela</t>
+          <t>Kaisha Brewer</t>
         </is>
       </c>
       <c r="C28" s="28" t="n"/>
-      <c r="D28" s="28" t="n"/>
+      <c r="D28" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="E28" s="23">
         <f>IFERROR(AVERAGE(C28:D28),"")</f>
         <v/>
       </c>
-      <c r="F28" s="28" t="n"/>
+      <c r="F28" s="24" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="29" ht="17" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
@@ -6129,7 +6249,7 @@
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla Valenzuela</t>
         </is>
       </c>
       <c r="C29" s="28" t="n"/>
@@ -6148,22 +6268,16 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>Lidy Henry</t>
-        </is>
-      </c>
-      <c r="C30" s="29" t="n">
-        <v>95</v>
-      </c>
-      <c r="D30" s="22" t="n">
-        <v>100</v>
-      </c>
+          <t>Kenzie</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="n"/>
+      <c r="D30" s="28" t="n"/>
       <c r="E30" s="23">
         <f>IFERROR(AVERAGE(C30:D30),"")</f>
         <v/>
       </c>
-      <c r="F30" s="24" t="n">
-        <v>46</v>
-      </c>
+      <c r="F30" s="28" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -6173,16 +6287,22 @@
       </c>
       <c r="B31" s="27" t="inlineStr">
         <is>
-          <t>Maylin Hernandez Rodriguez</t>
-        </is>
-      </c>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="28" t="n"/>
+          <t>Lidy Henry</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="n">
+        <v>95</v>
+      </c>
+      <c r="D31" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="E31" s="23">
         <f>IFERROR(AVERAGE(C31:D31),"")</f>
         <v/>
       </c>
-      <c r="F31" s="28" t="n"/>
+      <c r="F31" s="24" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
@@ -6192,7 +6312,7 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Maylin Hernandez Rodriguez</t>
         </is>
       </c>
       <c r="C32" s="28" t="n"/>
@@ -6211,7 +6331,7 @@
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>Nyatiek Keah</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="C33" s="28" t="n"/>
@@ -6230,7 +6350,7 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek Keah</t>
         </is>
       </c>
       <c r="C34" s="28" t="n"/>
@@ -6249,7 +6369,7 @@
       </c>
       <c r="B35" s="27" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="C35" s="28" t="n"/>
@@ -6268,7 +6388,7 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>Samuel Galban Rocha</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="C36" s="28" t="n"/>
@@ -6287,23 +6407,42 @@
       </c>
       <c r="B37" s="27" t="inlineStr">
         <is>
-          <t>Zack Whitten</t>
+          <t>Samuel Galban Rocha</t>
         </is>
       </c>
       <c r="C37" s="28" t="n"/>
-      <c r="D37" s="22" t="n">
-        <v>100</v>
-      </c>
+      <c r="D37" s="28" t="n"/>
       <c r="E37" s="23">
         <f>IFERROR(AVERAGE(C37:D37),"")</f>
         <v/>
       </c>
-      <c r="F37" s="24" t="n">
+      <c r="F37" s="28" t="n"/>
+    </row>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Zack Whitten</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="E38" s="23">
+        <f>IFERROR(AVERAGE(C38:D38),"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="24" t="n">
         <v>46</v>
       </c>
     </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="31" t="inlineStr">
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Score = shop score if on shift during meal window; blank if not. MTD SCORE = average of scores worked. MTD DOLLARS = $230 ÷ on-shift count per 100% shop.</t>
         </is>
@@ -6311,8 +6450,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A39:F39"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Daily brief 2026-06-18 — shop refresh (6/14 80%), new hires Serina+Ryan, team notes + dashboard wire
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5725,15 +5725,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -5758,10 +5759,15 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>WEEK 3</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
           <t>MTD SCORE</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>MTD DOLLARS</t>
         </is>
@@ -5784,8 +5790,13 @@
           <t>06/04</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>06/14</t>
+        </is>
+      </c>
       <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="4" t="inlineStr"/>
@@ -5804,8 +5815,13 @@
           <t>Lunch</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="9" t="inlineStr"/>
@@ -5820,8 +5836,11 @@
       <c r="D5" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="E5" s="9" t="inlineStr"/>
+      <c r="E5" s="13" t="n">
+        <v>80</v>
+      </c>
       <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="9" t="inlineStr"/>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="15" t="inlineStr"/>
@@ -5834,6 +5853,7 @@
       <c r="D6" s="17" t="n"/>
       <c r="E6" s="17" t="n"/>
       <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
     </row>
     <row r="7" ht="14" customHeight="1">
       <c r="A7" s="15" t="inlineStr"/>
@@ -5846,6 +5866,7 @@
       <c r="D7" s="17" t="n"/>
       <c r="E7" s="17" t="n"/>
       <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="8" ht="14" customHeight="1">
       <c r="A8" s="15" t="inlineStr"/>
@@ -5858,6 +5879,7 @@
       <c r="D8" s="17" t="n"/>
       <c r="E8" s="17" t="n"/>
       <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9" ht="14" customHeight="1">
       <c r="A9" s="15" t="inlineStr"/>
@@ -5870,6 +5892,7 @@
       <c r="D9" s="17" t="n"/>
       <c r="E9" s="17" t="n"/>
       <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="15" t="inlineStr"/>
@@ -5882,6 +5905,7 @@
       <c r="D10" s="17" t="n"/>
       <c r="E10" s="17" t="n"/>
       <c r="F10" s="17" t="n"/>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
@@ -5891,12 +5915,13 @@
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>MTD SCORE</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>MTD DOLLARS</t>
         </is>
@@ -5919,11 +5944,12 @@
       <c r="D12" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="E12" s="23">
-        <f>IFERROR(AVERAGE(C12:D12),"")</f>
-        <v/>
-      </c>
-      <c r="F12" s="24" t="n">
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="23">
+        <f>IFERROR(AVERAGE(C12:E12),"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -5940,11 +5966,12 @@
       </c>
       <c r="C13" s="21" t="n"/>
       <c r="D13" s="21" t="n"/>
-      <c r="E13" s="23">
-        <f>IFERROR(AVERAGE(C13:D13),"")</f>
-        <v/>
-      </c>
-      <c r="F13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="23">
+        <f>IFERROR(AVERAGE(C13:E13),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="21" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -5959,11 +5986,12 @@
       </c>
       <c r="C14" s="21" t="n"/>
       <c r="D14" s="21" t="n"/>
-      <c r="E14" s="23">
-        <f>IFERROR(AVERAGE(C14:D14),"")</f>
-        <v/>
-      </c>
-      <c r="F14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="23">
+        <f>IFERROR(AVERAGE(C14:E14),"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="21" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
@@ -5978,11 +6006,12 @@
       </c>
       <c r="C15" s="28" t="n"/>
       <c r="D15" s="28" t="n"/>
-      <c r="E15" s="23">
-        <f>IFERROR(AVERAGE(C15:D15),"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="28" t="n"/>
+      <c r="E15" s="28" t="n"/>
+      <c r="F15" s="23">
+        <f>IFERROR(AVERAGE(C15:E15),"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="28" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
@@ -5997,11 +6026,12 @@
       </c>
       <c r="C16" s="28" t="n"/>
       <c r="D16" s="28" t="n"/>
-      <c r="E16" s="23">
-        <f>IFERROR(AVERAGE(C16:D16),"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="28" t="n"/>
+      <c r="E16" s="28" t="n"/>
+      <c r="F16" s="23">
+        <f>IFERROR(AVERAGE(C16:E16),"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="28" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
@@ -6016,11 +6046,12 @@
       </c>
       <c r="C17" s="28" t="n"/>
       <c r="D17" s="28" t="n"/>
-      <c r="E17" s="23">
-        <f>IFERROR(AVERAGE(C17:D17),"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="28" t="n"/>
+      <c r="E17" s="28" t="n"/>
+      <c r="F17" s="23">
+        <f>IFERROR(AVERAGE(C17:E17),"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="28" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
@@ -6035,11 +6066,12 @@
       </c>
       <c r="C18" s="28" t="n"/>
       <c r="D18" s="28" t="n"/>
-      <c r="E18" s="23">
-        <f>IFERROR(AVERAGE(C18:D18),"")</f>
-        <v/>
-      </c>
-      <c r="F18" s="28" t="n"/>
+      <c r="E18" s="28" t="n"/>
+      <c r="F18" s="23">
+        <f>IFERROR(AVERAGE(C18:E18),"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="28" t="n"/>
     </row>
     <row r="19" ht="17" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
@@ -6056,11 +6088,12 @@
       <c r="D19" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="E19" s="23">
-        <f>IFERROR(AVERAGE(C19:D19),"")</f>
-        <v/>
-      </c>
-      <c r="F19" s="24" t="n">
+      <c r="E19" s="28" t="n"/>
+      <c r="F19" s="23">
+        <f>IFERROR(AVERAGE(C19:E19),"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6077,11 +6110,12 @@
       </c>
       <c r="C20" s="28" t="n"/>
       <c r="D20" s="28" t="n"/>
-      <c r="E20" s="23">
-        <f>IFERROR(AVERAGE(C20:D20),"")</f>
-        <v/>
-      </c>
-      <c r="F20" s="28" t="n"/>
+      <c r="E20" s="28" t="n"/>
+      <c r="F20" s="23">
+        <f>IFERROR(AVERAGE(C20:E20),"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="28" t="n"/>
     </row>
     <row r="21" ht="17" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
@@ -6096,11 +6130,12 @@
       </c>
       <c r="C21" s="28" t="n"/>
       <c r="D21" s="28" t="n"/>
-      <c r="E21" s="23">
-        <f>IFERROR(AVERAGE(C21:D21),"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="28" t="n"/>
+      <c r="E21" s="28" t="n"/>
+      <c r="F21" s="23">
+        <f>IFERROR(AVERAGE(C21:E21),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="28" t="n"/>
     </row>
     <row r="22" ht="17" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
@@ -6115,11 +6150,12 @@
       </c>
       <c r="C22" s="28" t="n"/>
       <c r="D22" s="28" t="n"/>
-      <c r="E22" s="23">
-        <f>IFERROR(AVERAGE(C22:D22),"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="28" t="n"/>
+      <c r="E22" s="28" t="n"/>
+      <c r="F22" s="23">
+        <f>IFERROR(AVERAGE(C22:E22),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="28" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -6136,11 +6172,12 @@
         <v>95</v>
       </c>
       <c r="D23" s="28" t="n"/>
-      <c r="E23" s="23">
-        <f>IFERROR(AVERAGE(C23:D23),"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="28" t="n"/>
+      <c r="E23" s="28" t="n"/>
+      <c r="F23" s="23">
+        <f>IFERROR(AVERAGE(C23:E23),"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="28" t="n"/>
     </row>
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
@@ -6155,11 +6192,12 @@
       </c>
       <c r="C24" s="28" t="n"/>
       <c r="D24" s="28" t="n"/>
-      <c r="E24" s="23">
-        <f>IFERROR(AVERAGE(C24:D24),"")</f>
-        <v/>
-      </c>
-      <c r="F24" s="28" t="n"/>
+      <c r="E24" s="28" t="n"/>
+      <c r="F24" s="23">
+        <f>IFERROR(AVERAGE(C24:E24),"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="28" t="n"/>
     </row>
     <row r="25" ht="17" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
@@ -6174,11 +6212,12 @@
       </c>
       <c r="C25" s="28" t="n"/>
       <c r="D25" s="28" t="n"/>
-      <c r="E25" s="23">
-        <f>IFERROR(AVERAGE(C25:D25),"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="28" t="n"/>
+      <c r="E25" s="28" t="n"/>
+      <c r="F25" s="23">
+        <f>IFERROR(AVERAGE(C25:E25),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="28" t="n"/>
     </row>
     <row r="26" ht="17" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
@@ -6193,11 +6232,12 @@
       </c>
       <c r="C26" s="28" t="n"/>
       <c r="D26" s="28" t="n"/>
-      <c r="E26" s="23">
-        <f>IFERROR(AVERAGE(C26:D26),"")</f>
-        <v/>
-      </c>
-      <c r="F26" s="28" t="n"/>
+      <c r="E26" s="28" t="n"/>
+      <c r="F26" s="23">
+        <f>IFERROR(AVERAGE(C26:E26),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="28" t="n"/>
     </row>
     <row r="27" ht="17" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
@@ -6212,11 +6252,12 @@
       </c>
       <c r="C27" s="28" t="n"/>
       <c r="D27" s="28" t="n"/>
-      <c r="E27" s="23">
-        <f>IFERROR(AVERAGE(C27:D27),"")</f>
-        <v/>
-      </c>
-      <c r="F27" s="28" t="n"/>
+      <c r="E27" s="28" t="n"/>
+      <c r="F27" s="23">
+        <f>IFERROR(AVERAGE(C27:E27),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="28" t="n"/>
     </row>
     <row r="28" ht="17" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
@@ -6233,11 +6274,12 @@
       <c r="D28" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="E28" s="23">
-        <f>IFERROR(AVERAGE(C28:D28),"")</f>
-        <v/>
-      </c>
-      <c r="F28" s="24" t="n">
+      <c r="E28" s="28" t="n"/>
+      <c r="F28" s="23">
+        <f>IFERROR(AVERAGE(C28:E28),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6254,11 +6296,12 @@
       </c>
       <c r="C29" s="28" t="n"/>
       <c r="D29" s="28" t="n"/>
-      <c r="E29" s="23">
-        <f>IFERROR(AVERAGE(C29:D29),"")</f>
-        <v/>
-      </c>
-      <c r="F29" s="28" t="n"/>
+      <c r="E29" s="28" t="n"/>
+      <c r="F29" s="23">
+        <f>IFERROR(AVERAGE(C29:E29),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="28" t="n"/>
     </row>
     <row r="30" ht="17" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
@@ -6273,11 +6316,12 @@
       </c>
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="28" t="n"/>
-      <c r="E30" s="23">
-        <f>IFERROR(AVERAGE(C30:D30),"")</f>
-        <v/>
-      </c>
-      <c r="F30" s="28" t="n"/>
+      <c r="E30" s="28" t="n"/>
+      <c r="F30" s="23">
+        <f>IFERROR(AVERAGE(C30:E30),"")</f>
+        <v/>
+      </c>
+      <c r="G30" s="28" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -6296,11 +6340,12 @@
       <c r="D31" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="E31" s="23">
-        <f>IFERROR(AVERAGE(C31:D31),"")</f>
-        <v/>
-      </c>
-      <c r="F31" s="24" t="n">
+      <c r="E31" s="28" t="n"/>
+      <c r="F31" s="23">
+        <f>IFERROR(AVERAGE(C31:E31),"")</f>
+        <v/>
+      </c>
+      <c r="G31" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6317,11 +6362,12 @@
       </c>
       <c r="C32" s="28" t="n"/>
       <c r="D32" s="28" t="n"/>
-      <c r="E32" s="23">
-        <f>IFERROR(AVERAGE(C32:D32),"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="28" t="n"/>
+      <c r="E32" s="28" t="n"/>
+      <c r="F32" s="23">
+        <f>IFERROR(AVERAGE(C32:E32),"")</f>
+        <v/>
+      </c>
+      <c r="G32" s="28" t="n"/>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
@@ -6336,11 +6382,12 @@
       </c>
       <c r="C33" s="28" t="n"/>
       <c r="D33" s="28" t="n"/>
-      <c r="E33" s="23">
-        <f>IFERROR(AVERAGE(C33:D33),"")</f>
-        <v/>
-      </c>
-      <c r="F33" s="28" t="n"/>
+      <c r="E33" s="28" t="n"/>
+      <c r="F33" s="23">
+        <f>IFERROR(AVERAGE(C33:E33),"")</f>
+        <v/>
+      </c>
+      <c r="G33" s="28" t="n"/>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
@@ -6355,11 +6402,12 @@
       </c>
       <c r="C34" s="28" t="n"/>
       <c r="D34" s="28" t="n"/>
-      <c r="E34" s="23">
-        <f>IFERROR(AVERAGE(C34:D34),"")</f>
-        <v/>
-      </c>
-      <c r="F34" s="28" t="n"/>
+      <c r="E34" s="28" t="n"/>
+      <c r="F34" s="23">
+        <f>IFERROR(AVERAGE(C34:E34),"")</f>
+        <v/>
+      </c>
+      <c r="G34" s="28" t="n"/>
     </row>
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
@@ -6374,11 +6422,12 @@
       </c>
       <c r="C35" s="28" t="n"/>
       <c r="D35" s="28" t="n"/>
-      <c r="E35" s="23">
-        <f>IFERROR(AVERAGE(C35:D35),"")</f>
-        <v/>
-      </c>
-      <c r="F35" s="28" t="n"/>
+      <c r="E35" s="28" t="n"/>
+      <c r="F35" s="23">
+        <f>IFERROR(AVERAGE(C35:E35),"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="28" t="n"/>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
@@ -6393,11 +6442,12 @@
       </c>
       <c r="C36" s="28" t="n"/>
       <c r="D36" s="28" t="n"/>
-      <c r="E36" s="23">
-        <f>IFERROR(AVERAGE(C36:D36),"")</f>
-        <v/>
-      </c>
-      <c r="F36" s="28" t="n"/>
+      <c r="E36" s="28" t="n"/>
+      <c r="F36" s="23">
+        <f>IFERROR(AVERAGE(C36:E36),"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="28" t="n"/>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
@@ -6412,11 +6462,12 @@
       </c>
       <c r="C37" s="28" t="n"/>
       <c r="D37" s="28" t="n"/>
-      <c r="E37" s="23">
-        <f>IFERROR(AVERAGE(C37:D37),"")</f>
-        <v/>
-      </c>
-      <c r="F37" s="28" t="n"/>
+      <c r="E37" s="28" t="n"/>
+      <c r="F37" s="23">
+        <f>IFERROR(AVERAGE(C37:E37),"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="28" t="n"/>
     </row>
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
@@ -6433,11 +6484,12 @@
       <c r="D38" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="E38" s="23">
-        <f>IFERROR(AVERAGE(C38:D38),"")</f>
-        <v/>
-      </c>
-      <c r="F38" s="24" t="n">
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="23">
+        <f>IFERROR(AVERAGE(C38:E38),"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6451,8 +6503,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A39:G39"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily brief 2026-06-19 — team notes + shop refresh (80% 6/14) + dashboard wire + 6/18 parbrink parse
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Auto-refresh: shop tracker triggered by Marketforce email 2026-06-25 (6/21 + 6/24 both 100%)
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5725,7 +5725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5733,8 +5733,10 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -5764,10 +5766,20 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
+          <t>WEEK 4</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>WEEK 5</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>MTD SCORE</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>MTD DOLLARS</t>
         </is>
@@ -5795,8 +5807,18 @@
           <t>06/14</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>06/21</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>06/24</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="4" t="inlineStr"/>
@@ -5820,8 +5842,18 @@
           <t>Dinner</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="9" t="inlineStr"/>
@@ -5839,8 +5871,14 @@
       <c r="E5" s="13" t="n">
         <v>80</v>
       </c>
-      <c r="F5" s="9" t="inlineStr"/>
-      <c r="G5" s="9" t="inlineStr"/>
+      <c r="F5" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="9" t="inlineStr"/>
+      <c r="I5" s="9" t="inlineStr"/>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="15" t="inlineStr"/>
@@ -5854,6 +5892,8 @@
       <c r="E6" s="17" t="n"/>
       <c r="F6" s="17" t="n"/>
       <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
     </row>
     <row r="7" ht="14" customHeight="1">
       <c r="A7" s="15" t="inlineStr"/>
@@ -5867,6 +5907,8 @@
       <c r="E7" s="17" t="n"/>
       <c r="F7" s="17" t="n"/>
       <c r="G7" s="17" t="n"/>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
     </row>
     <row r="8" ht="14" customHeight="1">
       <c r="A8" s="15" t="inlineStr"/>
@@ -5880,6 +5922,8 @@
       <c r="E8" s="17" t="n"/>
       <c r="F8" s="17" t="n"/>
       <c r="G8" s="17" t="n"/>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
     </row>
     <row r="9" ht="14" customHeight="1">
       <c r="A9" s="15" t="inlineStr"/>
@@ -5893,6 +5937,8 @@
       <c r="E9" s="17" t="n"/>
       <c r="F9" s="17" t="n"/>
       <c r="G9" s="17" t="n"/>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
     </row>
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="15" t="inlineStr"/>
@@ -5906,6 +5952,8 @@
       <c r="E10" s="17" t="n"/>
       <c r="F10" s="17" t="n"/>
       <c r="G10" s="17" t="n"/>
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="17" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
@@ -5916,12 +5964,14 @@
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>MTD SCORE</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>MTD DOLLARS</t>
         </is>
@@ -5945,11 +5995,13 @@
         <v>100</v>
       </c>
       <c r="E12" s="21" t="n"/>
-      <c r="F12" s="23">
-        <f>IFERROR(AVERAGE(C12:E12),"")</f>
-        <v/>
-      </c>
-      <c r="G12" s="24" t="n">
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="23">
+        <f>IFERROR(AVERAGE(C12:G12),"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -5967,11 +6019,13 @@
       <c r="C13" s="21" t="n"/>
       <c r="D13" s="21" t="n"/>
       <c r="E13" s="21" t="n"/>
-      <c r="F13" s="23">
-        <f>IFERROR(AVERAGE(C13:E13),"")</f>
-        <v/>
-      </c>
+      <c r="F13" s="21" t="n"/>
       <c r="G13" s="21" t="n"/>
+      <c r="H13" s="23">
+        <f>IFERROR(AVERAGE(C13:G13),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="21" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -5987,11 +6041,13 @@
       <c r="C14" s="21" t="n"/>
       <c r="D14" s="21" t="n"/>
       <c r="E14" s="21" t="n"/>
-      <c r="F14" s="23">
-        <f>IFERROR(AVERAGE(C14:E14),"")</f>
-        <v/>
-      </c>
+      <c r="F14" s="21" t="n"/>
       <c r="G14" s="21" t="n"/>
+      <c r="H14" s="23">
+        <f>IFERROR(AVERAGE(C14:G14),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="21" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
@@ -6007,11 +6063,13 @@
       <c r="C15" s="28" t="n"/>
       <c r="D15" s="28" t="n"/>
       <c r="E15" s="28" t="n"/>
-      <c r="F15" s="23">
-        <f>IFERROR(AVERAGE(C15:E15),"")</f>
-        <v/>
-      </c>
+      <c r="F15" s="28" t="n"/>
       <c r="G15" s="28" t="n"/>
+      <c r="H15" s="23">
+        <f>IFERROR(AVERAGE(C15:G15),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="28" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
@@ -6027,11 +6085,13 @@
       <c r="C16" s="28" t="n"/>
       <c r="D16" s="28" t="n"/>
       <c r="E16" s="28" t="n"/>
-      <c r="F16" s="23">
-        <f>IFERROR(AVERAGE(C16:E16),"")</f>
-        <v/>
-      </c>
+      <c r="F16" s="28" t="n"/>
       <c r="G16" s="28" t="n"/>
+      <c r="H16" s="23">
+        <f>IFERROR(AVERAGE(C16:G16),"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="28" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
@@ -6047,11 +6107,13 @@
       <c r="C17" s="28" t="n"/>
       <c r="D17" s="28" t="n"/>
       <c r="E17" s="28" t="n"/>
-      <c r="F17" s="23">
-        <f>IFERROR(AVERAGE(C17:E17),"")</f>
-        <v/>
-      </c>
+      <c r="F17" s="28" t="n"/>
       <c r="G17" s="28" t="n"/>
+      <c r="H17" s="23">
+        <f>IFERROR(AVERAGE(C17:G17),"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="28" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
@@ -6067,11 +6129,13 @@
       <c r="C18" s="28" t="n"/>
       <c r="D18" s="28" t="n"/>
       <c r="E18" s="28" t="n"/>
-      <c r="F18" s="23">
-        <f>IFERROR(AVERAGE(C18:E18),"")</f>
-        <v/>
-      </c>
+      <c r="F18" s="28" t="n"/>
       <c r="G18" s="28" t="n"/>
+      <c r="H18" s="23">
+        <f>IFERROR(AVERAGE(C18:G18),"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="28" t="n"/>
     </row>
     <row r="19" ht="17" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
@@ -6089,11 +6153,13 @@
         <v>100</v>
       </c>
       <c r="E19" s="28" t="n"/>
-      <c r="F19" s="23">
-        <f>IFERROR(AVERAGE(C19:E19),"")</f>
-        <v/>
-      </c>
-      <c r="G19" s="24" t="n">
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28" t="n"/>
+      <c r="H19" s="23">
+        <f>IFERROR(AVERAGE(C19:G19),"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6111,11 +6177,13 @@
       <c r="C20" s="28" t="n"/>
       <c r="D20" s="28" t="n"/>
       <c r="E20" s="28" t="n"/>
-      <c r="F20" s="23">
-        <f>IFERROR(AVERAGE(C20:E20),"")</f>
-        <v/>
-      </c>
+      <c r="F20" s="28" t="n"/>
       <c r="G20" s="28" t="n"/>
+      <c r="H20" s="23">
+        <f>IFERROR(AVERAGE(C20:G20),"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="28" t="n"/>
     </row>
     <row r="21" ht="17" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
@@ -6131,11 +6199,13 @@
       <c r="C21" s="28" t="n"/>
       <c r="D21" s="28" t="n"/>
       <c r="E21" s="28" t="n"/>
-      <c r="F21" s="23">
-        <f>IFERROR(AVERAGE(C21:E21),"")</f>
-        <v/>
-      </c>
+      <c r="F21" s="28" t="n"/>
       <c r="G21" s="28" t="n"/>
+      <c r="H21" s="23">
+        <f>IFERROR(AVERAGE(C21:G21),"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="28" t="n"/>
     </row>
     <row r="22" ht="17" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
@@ -6151,11 +6221,13 @@
       <c r="C22" s="28" t="n"/>
       <c r="D22" s="28" t="n"/>
       <c r="E22" s="28" t="n"/>
-      <c r="F22" s="23">
-        <f>IFERROR(AVERAGE(C22:E22),"")</f>
-        <v/>
-      </c>
+      <c r="F22" s="28" t="n"/>
       <c r="G22" s="28" t="n"/>
+      <c r="H22" s="23">
+        <f>IFERROR(AVERAGE(C22:G22),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="28" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -6175,11 +6247,13 @@
       <c r="E23" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="F23" s="23">
-        <f>IFERROR(AVERAGE(C23:E23),"")</f>
-        <v/>
-      </c>
+      <c r="F23" s="28" t="n"/>
       <c r="G23" s="28" t="n"/>
+      <c r="H23" s="23">
+        <f>IFERROR(AVERAGE(C23:G23),"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="28" t="n"/>
     </row>
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="26" t="inlineStr">
@@ -6195,11 +6269,13 @@
       <c r="C24" s="28" t="n"/>
       <c r="D24" s="28" t="n"/>
       <c r="E24" s="28" t="n"/>
-      <c r="F24" s="23">
-        <f>IFERROR(AVERAGE(C24:E24),"")</f>
-        <v/>
-      </c>
+      <c r="F24" s="28" t="n"/>
       <c r="G24" s="28" t="n"/>
+      <c r="H24" s="23">
+        <f>IFERROR(AVERAGE(C24:G24),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="28" t="n"/>
     </row>
     <row r="25" ht="17" customHeight="1">
       <c r="A25" s="26" t="inlineStr">
@@ -6215,11 +6291,13 @@
       <c r="C25" s="28" t="n"/>
       <c r="D25" s="28" t="n"/>
       <c r="E25" s="28" t="n"/>
-      <c r="F25" s="23">
-        <f>IFERROR(AVERAGE(C25:E25),"")</f>
-        <v/>
-      </c>
+      <c r="F25" s="28" t="n"/>
       <c r="G25" s="28" t="n"/>
+      <c r="H25" s="23">
+        <f>IFERROR(AVERAGE(C25:G25),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="28" t="n"/>
     </row>
     <row r="26" ht="17" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
@@ -6237,11 +6315,13 @@
       <c r="E26" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="F26" s="23">
-        <f>IFERROR(AVERAGE(C26:E26),"")</f>
-        <v/>
-      </c>
+      <c r="F26" s="28" t="n"/>
       <c r="G26" s="28" t="n"/>
+      <c r="H26" s="23">
+        <f>IFERROR(AVERAGE(C26:G26),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="28" t="n"/>
     </row>
     <row r="27" ht="17" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
@@ -6257,11 +6337,13 @@
       <c r="C27" s="28" t="n"/>
       <c r="D27" s="28" t="n"/>
       <c r="E27" s="28" t="n"/>
-      <c r="F27" s="23">
-        <f>IFERROR(AVERAGE(C27:E27),"")</f>
-        <v/>
-      </c>
+      <c r="F27" s="28" t="n"/>
       <c r="G27" s="28" t="n"/>
+      <c r="H27" s="23">
+        <f>IFERROR(AVERAGE(C27:G27),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="28" t="n"/>
     </row>
     <row r="28" ht="17" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
@@ -6279,11 +6361,13 @@
         <v>100</v>
       </c>
       <c r="E28" s="28" t="n"/>
-      <c r="F28" s="23">
-        <f>IFERROR(AVERAGE(C28:E28),"")</f>
-        <v/>
-      </c>
-      <c r="G28" s="24" t="n">
+      <c r="F28" s="28" t="n"/>
+      <c r="G28" s="28" t="n"/>
+      <c r="H28" s="23">
+        <f>IFERROR(AVERAGE(C28:G28),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6301,11 +6385,13 @@
       <c r="C29" s="28" t="n"/>
       <c r="D29" s="28" t="n"/>
       <c r="E29" s="28" t="n"/>
-      <c r="F29" s="23">
-        <f>IFERROR(AVERAGE(C29:E29),"")</f>
-        <v/>
-      </c>
+      <c r="F29" s="28" t="n"/>
       <c r="G29" s="28" t="n"/>
+      <c r="H29" s="23">
+        <f>IFERROR(AVERAGE(C29:G29),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="28" t="n"/>
     </row>
     <row r="30" ht="17" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
@@ -6321,11 +6407,13 @@
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="28" t="n"/>
       <c r="E30" s="28" t="n"/>
-      <c r="F30" s="23">
-        <f>IFERROR(AVERAGE(C30:E30),"")</f>
-        <v/>
-      </c>
+      <c r="F30" s="28" t="n"/>
       <c r="G30" s="28" t="n"/>
+      <c r="H30" s="23">
+        <f>IFERROR(AVERAGE(C30:G30),"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="28" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -6345,11 +6433,13 @@
         <v>100</v>
       </c>
       <c r="E31" s="28" t="n"/>
-      <c r="F31" s="23">
-        <f>IFERROR(AVERAGE(C31:E31),"")</f>
-        <v/>
-      </c>
-      <c r="G31" s="24" t="n">
+      <c r="F31" s="28" t="n"/>
+      <c r="G31" s="28" t="n"/>
+      <c r="H31" s="23">
+        <f>IFERROR(AVERAGE(C31:G31),"")</f>
+        <v/>
+      </c>
+      <c r="I31" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6369,11 +6459,13 @@
       <c r="E32" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="F32" s="23">
-        <f>IFERROR(AVERAGE(C32:E32),"")</f>
-        <v/>
-      </c>
+      <c r="F32" s="28" t="n"/>
       <c r="G32" s="28" t="n"/>
+      <c r="H32" s="23">
+        <f>IFERROR(AVERAGE(C32:G32),"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="28" t="n"/>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
@@ -6389,11 +6481,13 @@
       <c r="C33" s="28" t="n"/>
       <c r="D33" s="28" t="n"/>
       <c r="E33" s="28" t="n"/>
-      <c r="F33" s="23">
-        <f>IFERROR(AVERAGE(C33:E33),"")</f>
-        <v/>
-      </c>
+      <c r="F33" s="28" t="n"/>
       <c r="G33" s="28" t="n"/>
+      <c r="H33" s="23">
+        <f>IFERROR(AVERAGE(C33:G33),"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="28" t="n"/>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="26" t="inlineStr">
@@ -6409,11 +6503,13 @@
       <c r="C34" s="28" t="n"/>
       <c r="D34" s="28" t="n"/>
       <c r="E34" s="28" t="n"/>
-      <c r="F34" s="23">
-        <f>IFERROR(AVERAGE(C34:E34),"")</f>
-        <v/>
-      </c>
+      <c r="F34" s="28" t="n"/>
       <c r="G34" s="28" t="n"/>
+      <c r="H34" s="23">
+        <f>IFERROR(AVERAGE(C34:G34),"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="28" t="n"/>
     </row>
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
@@ -6431,11 +6527,13 @@
       <c r="E35" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="F35" s="23">
-        <f>IFERROR(AVERAGE(C35:E35),"")</f>
-        <v/>
-      </c>
+      <c r="F35" s="28" t="n"/>
       <c r="G35" s="28" t="n"/>
+      <c r="H35" s="23">
+        <f>IFERROR(AVERAGE(C35:G35),"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="28" t="n"/>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
@@ -6451,11 +6549,13 @@
       <c r="C36" s="28" t="n"/>
       <c r="D36" s="28" t="n"/>
       <c r="E36" s="28" t="n"/>
-      <c r="F36" s="23">
-        <f>IFERROR(AVERAGE(C36:E36),"")</f>
-        <v/>
-      </c>
+      <c r="F36" s="28" t="n"/>
       <c r="G36" s="28" t="n"/>
+      <c r="H36" s="23">
+        <f>IFERROR(AVERAGE(C36:G36),"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="28" t="n"/>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
@@ -6471,11 +6571,13 @@
       <c r="C37" s="28" t="n"/>
       <c r="D37" s="28" t="n"/>
       <c r="E37" s="28" t="n"/>
-      <c r="F37" s="23">
-        <f>IFERROR(AVERAGE(C37:E37),"")</f>
-        <v/>
-      </c>
+      <c r="F37" s="28" t="n"/>
       <c r="G37" s="28" t="n"/>
+      <c r="H37" s="23">
+        <f>IFERROR(AVERAGE(C37:G37),"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="28" t="n"/>
     </row>
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
@@ -6493,11 +6595,13 @@
         <v>100</v>
       </c>
       <c r="E38" s="28" t="n"/>
-      <c r="F38" s="23">
-        <f>IFERROR(AVERAGE(C38:E38),"")</f>
-        <v/>
-      </c>
-      <c r="G38" s="24" t="n">
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+      <c r="H38" s="23">
+        <f>IFERROR(AVERAGE(C38:G38),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -6510,9 +6614,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A39:I39"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
shop tracker: add June 21 (100%) and June 24 (100%) shops — June now 5 shops, 3x100%
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Daily brief 2026-07-02 (watchdog rescue) — team notes + dashboard wire, shop refresh (6/25 100%), directory +Megan Kurschner
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
watchdog: CT labor + COGS + food cost refresh, final rewire
- CT labor: date 2026-07-05, labor_percent 24.91% (Monday boundary — last posted day Sat 7/4)
- CT COGS: cogs_variance.json created, FP% 23.0% (week ending 7/5)
- Food cost plan: updated from stale 2026-05-03 to 2026-07-05 (FP% 23.0)
- Shops: KF scraper confirmed no new shops since 6/25 (126 total, Q-avg 89%)
- Dashboard rewire: labor source=ct_labor, food cost week=23.0%, 52/54 sections wired

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Auto-refresh: shop tracker triggered by Marketforce email 2026-07-09
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="July" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6696,4 +6697,667 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SECRET SHOPPER SCORES — JULY 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>WEEK 1</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>MTD SCORE</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>MTD DOLLARS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>07/03</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Meal Period</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="9" t="inlineStr"/>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>85</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="15" t="inlineStr"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Overall Experience</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="17" t="n"/>
+    </row>
+    <row r="7" ht="14" customHeight="1">
+      <c r="A7" s="15" t="inlineStr"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Enthusiasm</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+    </row>
+    <row r="8" ht="14" customHeight="1">
+      <c r="A8" s="15" t="inlineStr"/>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Likely to Return</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+    </row>
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="15" t="inlineStr"/>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Likely to Recommend</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="A10" s="15" t="inlineStr"/>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Exceptional Act?</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>INDIVIDUAL PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>MTD SCORE</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>MTD DOLLARS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Vicki Lucey</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="23">
+        <f>IFERROR(AVERAGE(C12:C12),"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="21" t="n"/>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>Kasey Wilson</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="23">
+        <f>IFERROR(AVERAGE(C13:C13),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="21" t="n"/>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Nathan Roberts</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="23">
+        <f>IFERROR(AVERAGE(C14:C14),"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="21" t="n"/>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Ailen Gonzalez Cardero</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="n"/>
+      <c r="D15" s="23">
+        <f>IFERROR(AVERAGE(C15:C15),"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="28" t="n"/>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>Anthony Pirtle</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="n"/>
+      <c r="D16" s="23">
+        <f>IFERROR(AVERAGE(C16:C16),"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="28" t="n"/>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>Ash</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="n"/>
+      <c r="D17" s="23">
+        <f>IFERROR(AVERAGE(C17:C17),"")</f>
+        <v/>
+      </c>
+      <c r="E17" s="28" t="n"/>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>Autumn Hearn</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="n"/>
+      <c r="D18" s="23">
+        <f>IFERROR(AVERAGE(C18:C18),"")</f>
+        <v/>
+      </c>
+      <c r="E18" s="28" t="n"/>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>Brianna Gatewood</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="n"/>
+      <c r="D19" s="23">
+        <f>IFERROR(AVERAGE(C19:C19),"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="28" t="n"/>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>DaKayla Dorsey</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="n"/>
+      <c r="D20" s="23">
+        <f>IFERROR(AVERAGE(C20:C20),"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="28" t="n"/>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>Damon</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="n"/>
+      <c r="D21" s="23">
+        <f>IFERROR(AVERAGE(C21:C21),"")</f>
+        <v/>
+      </c>
+      <c r="E21" s="28" t="n"/>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>Divan</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="n"/>
+      <c r="D22" s="23">
+        <f>IFERROR(AVERAGE(C22:C22),"")</f>
+        <v/>
+      </c>
+      <c r="E22" s="28" t="n"/>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>Francisco Llorente Mejias</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="n"/>
+      <c r="D23" s="23">
+        <f>IFERROR(AVERAGE(C23:C23),"")</f>
+        <v/>
+      </c>
+      <c r="E23" s="28" t="n"/>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>Grace</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="n"/>
+      <c r="D24" s="23">
+        <f>IFERROR(AVERAGE(C24:C24),"")</f>
+        <v/>
+      </c>
+      <c r="E24" s="28" t="n"/>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>Jada Cox</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="n"/>
+      <c r="D25" s="23">
+        <f>IFERROR(AVERAGE(C25:C25),"")</f>
+        <v/>
+      </c>
+      <c r="E25" s="28" t="n"/>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>Jeremiah Matthews</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="n"/>
+      <c r="D26" s="23">
+        <f>IFERROR(AVERAGE(C26:C26),"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="28" t="n"/>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Kable</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="n"/>
+      <c r="D27" s="23">
+        <f>IFERROR(AVERAGE(C27:C27),"")</f>
+        <v/>
+      </c>
+      <c r="E27" s="28" t="n"/>
+    </row>
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>Kaisha Brewer</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="n"/>
+      <c r="D28" s="23">
+        <f>IFERROR(AVERAGE(C28:C28),"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="28" t="n"/>
+    </row>
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>Kayla Valenzuela</t>
+        </is>
+      </c>
+      <c r="C29" s="28" t="n"/>
+      <c r="D29" s="23">
+        <f>IFERROR(AVERAGE(C29:C29),"")</f>
+        <v/>
+      </c>
+      <c r="E29" s="28" t="n"/>
+    </row>
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>Kenzie</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="n"/>
+      <c r="D30" s="23">
+        <f>IFERROR(AVERAGE(C30:C30),"")</f>
+        <v/>
+      </c>
+      <c r="E30" s="28" t="n"/>
+    </row>
+    <row r="31" ht="17" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>Lidy Henry</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="n"/>
+      <c r="D31" s="23">
+        <f>IFERROR(AVERAGE(C31:C31),"")</f>
+        <v/>
+      </c>
+      <c r="E31" s="28" t="n"/>
+    </row>
+    <row r="32" ht="17" customHeight="1">
+      <c r="A32" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>Maylin Hernandez Rodriguez</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="n"/>
+      <c r="D32" s="23">
+        <f>IFERROR(AVERAGE(C32:C32),"")</f>
+        <v/>
+      </c>
+      <c r="E32" s="28" t="n"/>
+    </row>
+    <row r="33" ht="17" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="n"/>
+      <c r="D33" s="23">
+        <f>IFERROR(AVERAGE(C33:C33),"")</f>
+        <v/>
+      </c>
+      <c r="E33" s="28" t="n"/>
+    </row>
+    <row r="34" ht="17" customHeight="1">
+      <c r="A34" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>Nyatiek Keah</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="n"/>
+      <c r="D34" s="23">
+        <f>IFERROR(AVERAGE(C34:C34),"")</f>
+        <v/>
+      </c>
+      <c r="E34" s="28" t="n"/>
+    </row>
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>Richard Gibbs</t>
+        </is>
+      </c>
+      <c r="C35" s="28" t="n"/>
+      <c r="D35" s="23">
+        <f>IFERROR(AVERAGE(C35:C35),"")</f>
+        <v/>
+      </c>
+      <c r="E35" s="28" t="n"/>
+    </row>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="n"/>
+      <c r="D36" s="23">
+        <f>IFERROR(AVERAGE(C36:C36),"")</f>
+        <v/>
+      </c>
+      <c r="E36" s="28" t="n"/>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>Samuel Galban Rocha</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="n"/>
+      <c r="D37" s="23">
+        <f>IFERROR(AVERAGE(C37:C37),"")</f>
+        <v/>
+      </c>
+      <c r="E37" s="28" t="n"/>
+    </row>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>CREW</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Zack Whitten</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="23">
+        <f>IFERROR(AVERAGE(C38:C38),"")</f>
+        <v/>
+      </c>
+      <c r="E38" s="28" t="n"/>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t>Score = shop score if on shift during meal window; blank if not. MTD SCORE = average of scores worked. MTD DOLLARS = $230 ÷ on-shift count per 100% shop.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A11:B11"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Daily brief 2026-07-30 — new 100% shop (7/23), team notes + missing temps + dashboard wire
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="July" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="July" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Daily refresh 2026-08-07: ComplianceMate sweep + morning pipeline outputs
- ComplianceMate: today's live pull (list_completions + all_list_completions
  roster), rollups recomputed, dashboard CM section rewired
- Bundled in already-uncommitted output from this morning's other automated
  runs (outlook brief missing-temps block, shop-payout draft check, shop
  tracker/performance refresh) that were sitting dirty in the working tree
  at sweep start — pushing now to close the chain rather than leave local
  work stranded
</commit_message>
<xml_diff>
--- a/Shop_Tracker_2065_2026.xlsx
+++ b/Shop_Tracker_2065_2026.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="January" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="February" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="March" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="April" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="June" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="July" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="August" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="January" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="February" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="March" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="July" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="August" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>